<commit_message>
Confirmation audit fixes: two stored sources described everywhere, stamped-paper text check, Excel wording, rules 0.3.1.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Answer: one row per indicator, sorted by the ease of adoption score. The score is a rule of thumb used only as a sort order, not a recommendation; every factor has its own column, so you can sort by any of them. Sensors x products: for each indicator, which of the 129 products in the Stygar 2021 list name it in their own description and which a published study tested. Schemes: what each certification scheme requires. Product list and Sources: where everything comes from.</t>
+          <t>Answer: one row per indicator, sorted by the ease of adoption score. The score is a rule of thumb used only as a sort order, not a recommendation; every factor has its own column, so you can sort by any of them. Sensors x products: for each indicator, which of the 129 products in the Stygar 2021 list contain one of the indicator's search words in their own description, and which a published study tested. Schemes: what each certification scheme requires. Product list and Sources: where everything comes from.</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work in progress. Rows marked 'Not yet checked' have no sensor or scheme research yet; their score is not meaningful and the ranking is provisional until every row is complete.</t>
+          <t>Work in progress. Rows marked 'Not yet checked' have no sensor evidence grade and no scheme rows yet (their Maroto Molina rating is coded in 2_research/indicators.csv); their score is not meaningful and the ranking is provisional until every row is complete.</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       <c r="A30" s="3" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no welfare scientist has reviewed the table yet.</t>
+          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no review by a welfare scientist is recorded in the repository.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), one device per farm and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro). All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
+          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), one device per farm, and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>EFSA Table 27 page 43 rates bulk milk SCC high feasibility because records are readily available, with low sensitivity; The class comes from the routine_data list in rules.md rule 4.4 (somatic cell count from records), not from the records rule, because EFSA names records only in the feasibility line; that line, records readily available, is the evidence that the value already exists. So the class is routine_data although no PLF product measures the bulk tank.</t>
+          <t>EFSA Table 27 page 43 rates bulk milk SCC high feasibility because records are readily available, with low sensitivity; the class comes from the routine_data list in rules.md rule 4.4 (somatic cell count from records), not from the records rule, because EFSA names records only in the feasibility line; that line, records readily available, is the evidence that the value already exists. The class list applies here and not to I006 because it names somatic cell count from records and EFSA calls the bulk milk SCC records readily available; mastitis incidence (I006) is not in the class list, and EFSA calls its records dependent on availability and accuracy of vet/farm records. So the class is routine_data although no PLF product measures the bulk tank.</t>
         </is>
       </c>
     </row>
@@ -6937,7 +6937,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="T3" s="7" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -7721,7 +7721,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="P25" s="8" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
         </is>
       </c>
       <c r="AS29" s="7" t="inlineStr">
@@ -18309,7 +18309,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>CC BY-ND 4.0, except six third party figures</t>
+          <t>CC BY-ND 4.0 for EFSA's own content; Figures 2, 3, 4, 5, 7 and 8 are third party and not covered</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Second confirmation audit fixes: saved web pages checked by phrase, robust stamped check, schemes status counts partial reads.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work in progress. Rows marked 'Not yet checked' have no sensor evidence grade and no scheme rows yet (their Maroto Molina rating is coded in 2_research/indicators.csv); their score is not meaningful and the ranking is provisional until every row is complete.</t>
+          <t>Work in progress. Rows marked 'Not yet checked' have no row in 2_research/sensor_coverage.csv yet, so no sensor evidence grade (their Maroto Molina rating is coded in 2_research/indicators.csv); their score is not meaningful and the ranking is provisional until every row is complete.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes, abbreviations and terms used in the cells. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
+          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), one device per farm, and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
+          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), one installation per parlour (rules.md rule 4.4, milk analysers), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 0 aims name bulk milk or bulk tank. The SCC products in the appendix measure single animals or quarters: Lely MQC-C (validated, ref 43) somatic cell count of each cow, LIC Protrack SCC individual somatic cell count, GEA M6850 SCC on each udder quarter; DeLaval OCC and DCC aims say udder health monitoring. That is the Welfare Quality measure I057, not bulk tank SCC. Maroto Molina do not discuss bulk tank SCC.</t>
+          <t>Keyword scan: 0 aims name bulk milk or bulk tank. The SCC products in the appendix measure single animals or quarters: Lely MQC-C (validated, ref 43) somatic cell count of each cow, LIC Protrack SCC individual somatic cell count, GEA M6850 SCC on each udder quarter; DeLaval OCC and DCC aims say udder health monitoring. That is individual cow SCC, the Welfare Quality measure I057 and the EFSA measure I058, not bulk tank SCC. Maroto Molina do not discuss bulk tank SCC.</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Kevin's files kept public by the author's decision; list 1 and scheme counts correct under partial reads; rules 0.3.2.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work in progress. Rows marked 'Not yet checked' have no row in 2_research/sensor_coverage.csv yet, so no sensor evidence grade (their Maroto Molina rating is coded in 2_research/indicators.csv); their score is not meaningful and the ranking is provisional until every row is complete.</t>
+          <t>Work in progress. Rows whose Row status is 'Not yet checked' have no row in 2_research/sensor_coverage.csv yet, so no sensor evidence grade (their Maroto Molina rating is coded in 2_research/indicators.csv); their score is not meaningful and the ranking is provisional until every row is complete.</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Checked for 0 of 58 indicators so far.</t>
+          <t>All four schemes checked for 0 of 58 indicators so far, at least one for 0.</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>0 confirmed; the schemes are checked for 0 of 58 indicators so far. Column (a) shows the sensor evidence beside each one.</t>
+          <t>0 confirmed; all four schemes checked for 0 of 58 indicators so far, at least one for 0. Column (a) shows the sensor evidence beside each one.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
+          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names and sensor types, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), one installation per parlour (rules.md rule 4.4, milk analysers), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
+          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), farm_fixed under rule 4.4 (an analyser at the milking point is one installation per parlour), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Independent check of the four schemes: one quote corrected (Certified Humane I050), four reasoning fixes.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -11369,7 +11369,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No numbered requirement names digital dermatitis. Searched: dermatitis, digital, claw, hoof, foot, infection, lesion. The only mention is an information box after H 3.8 (PDF 49, printed 47) listing digital dermatitis among diseases for which monitoring the incidence of lameness is useful; boxes are not standards (Guide, PDF 6, printed 4), and the box names lameness incidence, not a digital dermatitis score. Nearest requirement: H 3.1 b) (PDF 48, printed 46), feet of all cattle inspected at least annually by a competent foot trimmer for signs of abnormal wear, infection or excessive growth; infection is a general class, not a synonym of digital dermatitis, so it is not counted here (the same clause is the unsure candidate for I003). related_resource: H 3.7 footbathing facility with an antibacterial agent (PDF 49, printed 47); H 1.5 h) main disease problems listed in the VHWP (PDF 45, printed 43). The justification document (PDF 7, printed 5) names digital dermatitis only as a foot condition linked to cows standing with two feet out of the cubicle. Rule 2: box text does not count.</t>
+          <t>No numbered requirement names digital dermatitis. Searched: dermatitis, digital, claw, hoof, foot, infection, lesion. The only mention is an information box after H 3.8 (PDF 49, printed 47) listing digital dermatitis among diseases for which monitoring the incidence of lameness is useful; boxes are not standards (Guide, PDF 6, printed 4), and the box names lameness incidence, not a digital dermatitis score. Nearest requirement: H 3.1 b) (PDF 48, printed 46), feet of all cattle inspected at least annually by a competent foot trimmer for signs of abnormal wear, infection or excessive growth; infection is a general class, not a synonym of digital dermatitis, so it is not counted here (the same clause is recorded as related practice for I003). related_resource: H 3.7 footbathing facility with an antibacterial agent (PDF 49, printed 47); H 1.5 h) main disease problems listed in the VHWP (PDF 45, printed 43). The justification document (PDF 7, printed 5) names digital dermatitis only as a foot condition linked to cows standing with two feet out of the cubicle. Rule 2: box text does not count.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -14095,7 +14095,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "Mortality of Heifers from 3-weeks pre-calving and cows must not exceed 4% per 12-month period." (3.H.6 (Mortality and Culling), PDF 26 (printed 16)). Names cow mortality with a number. Marked at Steps 1, 2 and 3. At Steps 4 to 5+, 3.H.7 on the same page sets 2%. Other mortality limits: 3.H.5, all Steps, weaned Heifers 2% (PDF 26); 3.H.3, Steps 1 to 3, pre weaning 6%, and 3.H.4, Steps 4 to 5+, 4% (PDF 25, printed 15). GAP's Mortality "excludes stillborn Calves" and, per info note 3.H.6a, "This percentage excludes Culls", which include euthanized animals, whereas the Welfare Quality measure counts animals dead, euthanized and emergency slaughtered (protocol PDF 35), so the GAP figure is narrower. It is coded required because the requirement names mortality itself in adult cows, the same measure name, and is not broader wording (rule 6); the difference is recorded here. How checked: section note (PDF 25) "Mortality will be assessed by a review of records", repeated in Appendix I (PDF 59, printed 49); info note 3.H.6c "Auditors will evaluate this standard by calculating an annual percentage"; 3.H.1, all Steps, "Records of Mortality and Culling by animal group ... must be kept". Monthly Mortality rate is also reported under 5.H.4 d (PDF 38, printed 28). Coded unsure when the four schemes were merged on 8 October 2026: the wording is narrower than the Welfare Quality mortality measure, and rule 6 covers broader wording but not narrower wording, so the rules do not settle it (open_questions.md).</t>
+          <t>Candidate: "Mortality of Heifers from 3-weeks pre-calving and cows must not exceed 4% per 12-month period." (3.H.6 (Mortality and Culling), PDF 26 (printed 16)). Names cow mortality with a number. Marked at Steps 1, 2 and 3. At Steps 4 to 5+, 3.H.7 on the same page sets 2%. Other mortality limits: 3.H.5, all Steps, weaned Heifers 2% (PDF 26); 3.H.3, Steps 1 to 3, pre weaning 6%, and 3.H.4, Steps 4 to 5+, 4% (PDF 25, printed 15). GAP's Mortality "excludes stillborn Calves" and, per info note 3.H.6a, "This percentage excludes Culls", which include euthanized animals, whereas the Welfare Quality measure counts animals dead, euthanized and emergency slaughtered (protocol PDF 35), so the GAP figure is narrower. The reading for required: the requirement names mortality itself in adult cows, the same measure name, and is not broader wording (rule 6). How checked: section note (PDF 25) "Mortality will be assessed by a review of records", repeated in Appendix I (PDF 59, printed 49); info note 3.H.6c "Auditors will evaluate this standard by calculating an annual percentage"; 3.H.1, all Steps, "Records of Mortality and Culling by animal group ... must be kept". Monthly Mortality rate is also reported under 5.H.4 d (PDF 38, printed 28). Coded unsure when the four schemes were merged on 8 October 2026: the wording is narrower than the Welfare Quality mortality measure, and rule 6 covers broader wording but not narrower wording, so the rules do not settle it (open_questions.md).</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -14234,7 +14234,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>"11. Non-ambulatory animals Tolerance limits on herd performance or behavioral parameters for the above conditions must be delineated in the Animal Health Plan." (H 1 a 11, PDF 35 (printed 26))</t>
+          <t>"The herd must be continually monitored for performance, including production diseases, infectious diseases, and injury as a result of housing/husbandry/handling, such as: ... 11. Non-ambulatory animals" (H 1 a 11, PDF 34 to 35 (printed 25 to 26))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Data audit: RSPCA I037 recoded to required (hind quarters is Welfare Quality's own term); counts and examples updated.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -2887,178 +2887,178 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>I037</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Cleanliness of flank/upper legs</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Welfare Quality only</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Observed or recorded on the animal</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>FARM has only a related housing, equipment or practice rule</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>RSPCA Assured (UK): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals; unclear whether Certified Humane (US) requires it</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US)</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>1 + 2 + 0 + 1 + 2</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>Welfare Quality PDF page 27 (printed 26): an animal based measure scored on the hind quarters, upper hind leg, flank and rear view including tail, excluding udder; 0 for no dirt or minor splashing, 2 for separate or continuous plaques of dirt. Maroto Molina page 3: regarding cow dirtiness, no automatic monitoring systems were found in the literature, but image analysis systems could be used for that; technologies developed to monitor faeces in carcasses (Windham et al. 2003; Seo et al. 2019) could be adapted to evaluate cow dirtiness. Keyword scan: 0 aims name dirt, hygiene or cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: to the best knowledge of the authors there are currently no available technologies able to assess the cleanliness of animals, though rapid development in vision based monitoring for individual identification could prompt algorithms for it.</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>I051</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Disbudding/Dehorning</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Welfare Quality only</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>About farm management</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>Not yet checked</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr"/>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr"/>
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Not yet checked</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Not yet checked</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>Named in FARM, with a number to meet</t>
         </is>
       </c>
-      <c r="P20" s="5" t="n">
+      <c r="P21" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="Q20" s="5" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
-      <c r="R20" s="5" t="inlineStr">
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="S20" s="5" t="inlineStr">
+      <c r="S21" s="5" t="inlineStr">
         <is>
           <t>Yes: FARM v5 (US industry), Global Animal Partnership (US)</t>
         </is>
       </c>
-      <c r="T20" s="5" t="n">
+      <c r="T21" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="U20" s="5" t="inlineStr">
+      <c r="U21" s="5" t="inlineStr">
         <is>
           <t>0 + 0 + 0 + 3 + 3</t>
         </is>
       </c>
-      <c r="V20" s="5" t="inlineStr">
+      <c r="V21" s="5" t="inlineStr">
         <is>
           <t>Not yet checked</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr"/>
-      <c r="X20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>I032</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Water flow</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Welfare Quality only</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>About the housing or equipment</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="2" t="inlineStr">
-        <is>
-          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked</t>
-        </is>
-      </c>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="U21" s="2" t="inlineStr">
-        <is>
-          <t>1 + 2 + 0 + 1 + 1</t>
-        </is>
-      </c>
-      <c r="V21" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="W21" s="2" t="inlineStr">
-        <is>
-          <t>Welfare Quality PDF page 25 (printed 24): a resource based measure; the flow per water point is checked by collecting the overflow for one minute, sufficient at 10 L/min for a bowl and 20 L/min for a trough. Maroto Molina page 2: from a PLF perspective, monitoring the number and status of water points has no relevance, as it is possible to actually measure water consumption of every cow; a combination of RFID and flowmeters could provide these data (Cardot et al. 2008). That is a substitute measure, water intake per cow, so the grade is research_only under factor 1. Stygar Table 2 page 7 lists Water intake, Insentec (45), research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation in the supplementary study table; the appendix row is Hokofarm Group RIC, load cells and RFID, aim measures individual feed and water intake, flag yes. Stygar page 10: regarding the thirst criterion only resource based indicators are evaluated, so PLF technologies can provide additional single animal level information. Keyword scan: 0 aims name water flow or a flowmeter.</t>
-        </is>
-      </c>
-      <c r="X21" s="2" t="inlineStr">
-        <is>
-          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class.</t>
-        </is>
-      </c>
+      <c r="W21" s="5" t="inlineStr"/>
+      <c r="X21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>I033</t>
+          <t>I032</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Functioning of water points</t>
+          <t>Water flow</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="W22" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality PDF page 25 (printed 24): a resource based measure; the assessor checks that drinkers work correctly, that levers are movable and water flows when moved; scored 0 working correctly, 2 malfunctioning. Maroto Molina page 2: from a PLF perspective, monitoring the number and status of water points has no relevance, as it is possible to actually measure water consumption of every cow; a combination of RFID and flowmeters could provide these data (Cardot et al. 2008). That is a substitute measure, water intake per cow, so the grade is research_only under factor 1. Stygar Table 2 page 7 lists Water intake, Insentec (45), research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation in the supplementary study table; the appendix row is Hokofarm Group RIC, load cells and RFID, aim measures individual feed and water intake, flag yes. Stygar page 10: regarding the thirst criterion only resource based indicators are evaluated, so PLF technologies can provide additional single animal level information. Keyword scan: 0 aims name a drinker or a water point.</t>
+          <t>Welfare Quality PDF page 25 (printed 24): a resource based measure; the flow per water point is checked by collecting the overflow for one minute, sufficient at 10 L/min for a bowl and 20 L/min for a trough. Maroto Molina page 2: from a PLF perspective, monitoring the number and status of water points has no relevance, as it is possible to actually measure water consumption of every cow; a combination of RFID and flowmeters could provide these data (Cardot et al. 2008). That is a substitute measure, water intake per cow, so the grade is research_only under factor 1. Stygar Table 2 page 7 lists Water intake, Insentec (45), research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation in the supplementary study table; the appendix row is Hokofarm Group RIC, load cells and RFID, aim measures individual feed and water intake, flag yes. Stygar page 10: regarding the thirst criterion only resource based indicators are evaluated, so PLF technologies can provide additional single animal level information. Keyword scan: 0 aims name water flow or a flowmeter.</t>
         </is>
       </c>
       <c r="X22" s="2" t="inlineStr">
@@ -3156,12 +3156,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>I037</t>
+          <t>I033</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Cleanliness of flank/upper legs</t>
+          <t>Functioning of water points</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -3172,7 +3172,7 @@
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
+          <t>About the housing or equipment</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Global Animal Partnership (US): inspector looks at the animals; unclear whether RSPCA Assured (UK), Certified Humane (US) requires it</t>
+          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>Yes: Global Animal Partnership (US)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T23" s="2" t="n">
@@ -3231,12 +3231,12 @@
       </c>
       <c r="W23" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality PDF page 27 (printed 26): an animal based measure scored on the hind quarters, upper hind leg, flank and rear view including tail, excluding udder; 0 for no dirt or minor splashing, 2 for separate or continuous plaques of dirt. Maroto Molina page 3: regarding cow dirtiness, no automatic monitoring systems were found in the literature, but image analysis systems could be used for that; technologies developed to monitor faeces in carcasses (Windham et al. 2003; Seo et al. 2019) could be adapted to evaluate cow dirtiness. Keyword scan: 0 aims name dirt, hygiene or cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: to the best knowledge of the authors there are currently no available technologies able to assess the cleanliness of animals, though rapid development in vision based monitoring for individual identification could prompt algorithms for it.</t>
+          <t>Welfare Quality PDF page 25 (printed 24): a resource based measure; the assessor checks that drinkers work correctly, that levers are movable and water flows when moved; scored 0 working correctly, 2 malfunctioning. Maroto Molina page 2: from a PLF perspective, monitoring the number and status of water points has no relevance, as it is possible to actually measure water consumption of every cow; a combination of RFID and flowmeters could provide these data (Cardot et al. 2008). That is a substitute measure, water intake per cow, so the grade is research_only under factor 1. Stygar Table 2 page 7 lists Water intake, Insentec (45), research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation in the supplementary study table; the appendix row is Hokofarm Group RIC, load cells and RFID, aim measures individual feed and water intake, flag yes. Stygar page 10: regarding the thirst criterion only resource based indicators are evaluated, so PLF technologies can provide additional single animal level information. Keyword scan: 0 aims name a drinker or a water point.</t>
         </is>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says.</t>
+          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class.</t>
         </is>
       </c>
     </row>
@@ -11696,7 +11696,7 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Searched for somatic, SCC, cell count, bulk tank and milk quality. SCC appears only in the acronym list (PDF 9) and in the Milking Procedure science box, which says certain milking practices are associated with lower herd somatic cell count (PDF 70). No standard names bulk milk SCC. The Antibiotic Stewardship standard tests sold milk for antibiotics, not cell count (Chapter 2, PDF 16). Related requirements: "The Herd Health Plan (HHP) has a written protocol for milking procedures." (Chapter 4, Milking Procedure, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56). Not required: the only herd level SCC wording is in a science box (PDF 70), which is not a standard (rule 2); under rule 6 a herd level count would name this row.</t>
+          <t>Searched for somatic, SCC, cell count, bulk tank and milk quality. SCC appears only in the acronym list (PDF 9) and in the Milking Procedure science box, which says certain milking practices are associated with lower herd somatic cell count (PDF 70). No standard names bulk milk SCC. The Antibiotic Stewardship standard tests sold milk for antibiotics, not cell count (Chapter 2, PDF 16). Related requirements: "The Herd Health Plan (HHP) has a written protocol for milking procedures." (Chapter 4, Milking Procedure, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56). Not required: the only herd level SCC wording is in a science box (PDF 70), which is not a standard (rule 2); under rule 6 a herd level count would name this row. The same box's reference list also has a title with herd somatic cell count (PDF 71), which is a reference, not a standard.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -13424,7 +13424,7 @@
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the udder. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108).</t>
+          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the udder. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108). The figure carries labels stored as glyph codes (for example rear udder attachment, flank, hock and knee); they mark landmarks, and the scored areas A and B are defined only by the drawing.</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "Visually assess the one randomly selected side of the animal and behind, only including the hind quarters to coronary band and udder: Scoring: 0 = Clean No dirt or only minor splashing present 2 = Very Dirty An area of dirtiness (i.e. layer or plaques of dirt) amounting to at least forearm length (40cm) in any dimension." (WA 1.1 a); Appendix 4 item 3 (Cleanliness), PDF 98 (printed 96)). Candidate: Appendix 4 item 3, binding through WA 1.1 a) (PDF 57, printed 55) under rule 3: one visual cleanliness score for one randomly selected side and behind, covering the hind quarters to coronary band and udder, very dirty at 40cm or more. The text lists the hind quarters, the coronary band and the udder; the score sheet (PDF 102, printed 100) lists no region for cleanliness. Reading 1, required: the listed span from the hind quarters down to the coronary band takes in the upper hind legs, so cleanliness of the upper legs is scored. Reading 2, not required: the flank and upper legs are not listed, and hind quarters is not a direct synonym of flank and upper legs (rule 6). Rule 9 does not say whether a listed span names the parts inside it. how_checked is visual_inspection either way: the protocol says Visually assess, and scheme personnel carry it out (WA 1.1 d) ii). related_resource: E 8.5, pasture managed so that the cattle are kept clean (PDF 25, printed 23); E 5.4, a clean, dry cubicle bed (PDF 19, printed 17).</t>
+          <t>"Visually assess the one randomly selected side of the animal and behind, only including the hind quarters to coronary band and udder: Scoring: 0 = Clean No dirt or only minor splashing present 2 = Very Dirty An area of dirtiness (i.e. layer or plaques of dirt) amounting to at least forearm length (40cm) in any dimension." (WA 1.1 a); Appendix 4 item 3 (Cleanliness), PDF 98 (printed 96))</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -13488,7 +13488,7 @@
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the flank or upper legs. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108).</t>
+          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the flank or upper legs. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108). The figure carries labels stored as glyph codes (for example rear udder attachment, flank, hock and knee); they mark landmarks, and the scored areas A and B are defined only by the drawing.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -13552,7 +13552,7 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the lower legs. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108).</t>
+          <t>Not required under rule 9. The nearest requirement is "Lactating Cows: 90% or more of lactating cows observed score 2 or less on the FARM Hygiene Scorecard." (Chapter 9, Hygiene, PDF 160). The scorecard (PDF 161) gives one score for mud or manure "in areas A or B"; its text lists no body region, and the areas are shown only in a figure, so the score does not name the lower legs. Welfare Quality scores udder, flank/upper legs and lower legs separately. The same 90% benchmark is set for pre-weaned calves, weaned heifers and dry cows (PDF 160). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), whose evaluation uses hygiene scores "as an animal-based measure of environment cleanliness"; the calving area must also be clean (Chapter 5, PDF 108). The figure carries labels stored as glyph codes (for example rear udder attachment, flank, hock and knee); they mark landmarks, and the scored areas A and B are defined only by the drawing.</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Repository stands alone: no links to the old repository, plain Start here section, one command to download and prove the sources.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -18031,7 +18031,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Column 3, not yet started: what RSPCA Assured requires and how it is checked; already quoted in the worked example in rules.md.</t>
+          <t>Column 3: what RSPCA Assured requires and how it is checked; already quoted in the worked example in rules.md.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -18073,7 +18073,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Column 3, not yet started: the RSPCA's stated reasons for its requirements, for the notes in crosswalk.csv.</t>
+          <t>Column 3: the RSPCA's stated reasons for its requirements, for the notes in crosswalk.csv.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -18115,7 +18115,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Column 3, not yet started: what FARM requires, and the industry naming factor, since FARM is the dairy industry's own programme; already quoted in rules.md.</t>
+          <t>Column 3: what FARM requires, and the industry naming factor, since FARM is the dairy industry's own programme; already quoted in rules.md.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -18157,7 +18157,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Column 3, not yet started: what Global Animal Partnership requires and how it is checked.</t>
+          <t>Column 3: what Global Animal Partnership requires and how it is checked.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -18199,7 +18199,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Column 3, not yet started: what Certified Humane requires and how it is checked.</t>
+          <t>Column 3: what Certified Humane requires and how it is checked.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit corrections: body condition required by all four labels; plain claims made exact; I059 device needed unsure; download fixes.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -687,7 +687,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>The cheapest kind of equipment that measures it. Classes, in the order the score ranks them: nothing extra (3 points), one device per farm (2), one device per animal (1), a sample or a scoring by a person (0), or no technology named in the sources (0). 'Nothing extra' can appear where no sensor exists, because the value is already taken from milk or farm records (2_research/rules.md, rule 4.4).</t>
+          <t>The cheapest kind of equipment that measures it. Classes, in the order the score ranks them: nothing extra (3 points), one device per farm (2), one device per animal (1), a sample or a scoring by a person (0), or no technology named in the sources (0), or unclear when the rules do not settle it (0). 'Nothing extra' can appear where no sensor exists, because the value is already taken from milk or farm records (2_research/rules.md, rule 4.4).</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="X38" s="2" t="inlineStr">
         <is>
-          <t>As on I040, the substitute measure has commercial products, which the grade does not credit, because the Welfare Quality measure is whether the farm gives access to an outdoor loafing area or pasture, not where the cow is. Device needed: among the technologies proposed, the only one with appendix products whose aims state the substitute measurement is GPS positioning, and all seven are worn (collars and an ear tag), so animal_mounted; satellite imagery is not a device on the farm and has no appendix row. The records rule of rule 4.4 does not apply, because the definition takes the value from the manager's answers and names no records. IceTag's aim names "pastur activity" with the number of steps, a step count at pasture, not access to it; the search word pasture does not match that spelling, and a reader who searched pastur would count 1. Stygar Table 2 page 7 validates grazing time (MooMonitor+ 29, RumiWatch 29 and 38, research farm, high performance column), a feeding behaviour, not the provision of access, so under rule 4.2 it is not the same measure. I053, the Welfare Quality access to pasture measure under appropriate behaviour, is a separate row.</t>
+          <t>As on I040, the substitute measure has commercial products, which the grade does not credit, because the Welfare Quality measure is whether the farm gives access to an outdoor loafing area or pasture, not where the cow is. Device needed: among the technologies proposed, the only one with appendix products whose aims state the substitute measurement is GPS positioning, and all seven are worn (collars and an ear tag), so animal_mounted; satellite imagery is not a device on the farm and has no appendix row. Four more aims name location or tracking: CowView (appendix row 64), CowManager (row 26) and Smartbow (row 117, indoor location), all worn, and Taggle (row 123), an RFID radiolocation system whose aim, Tracking system, does not state location; none of them changes the class. The records rule of rule 4.4 does not apply, because the definition takes the value from the manager's answers and names no records. IceTag's aim names "pastur activity" with the number of steps, a step count at pasture, not access to it; the search word pasture does not match that spelling, and a reader who searched pastur would count 1. Stygar Table 2 page 7 validates grazing time (MooMonitor+ 29, RumiWatch 29 and 38, research farm, high performance column), a feeding behaviour, not the provision of access, so under rule 4.2 it is not the same measure. I053, the Welfare Quality access to pasture measure under appropriate behaviour, is a separate row.</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>No appendix aim names nasal discharge, and Maroto Molina propose a technology, so research_only. The maroto_molina_technology column of indicators.csv attaches the integration of body temperature sensors with feed and water intake monitoring to this row, and the image analysis tested in pigs to I045 only. HerdInsight's health disorder validation (30) is not the same measure as nasal discharge, the reading already applied on I006, so it is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030 classes a bolus combination animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
+          <t>No appendix aim names nasal discharge, and Maroto Molina propose a technology, so research_only. The maroto_molina_technology column of indicators.csv attaches the integration of body temperature sensors with feed and water intake monitoring to this row, and the image analysis tested in pigs to I045 only. HerdInsight's health disorder validation (30) is not the same measure as nasal discharge, the reading already applied on I006, so it is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6085,7 @@
       </c>
       <c r="X53" s="2" t="inlineStr">
         <is>
-          <t>Same passage and same reading as I043 (the maroto_molina_technology column of indicators.csv): no appendix aim names ocular discharge, and Maroto Molina propose the integration of body temperature sensors with intake monitoring, so research_only; HerdInsight's health disorder validation (30) is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030 classes a bolus combination animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
+          <t>Same passage and same reading as I043 (the maroto_molina_technology column of indicators.csv): no appendix aim names ocular discharge, and Maroto Molina propose the integration of body temperature sensors with intake monitoring, so research_only; HerdInsight's health disorder validation (30) is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>A substitute measure, so research_only under rules.md rule 4.2, whatever the products for the substitute; the grade does not credit them, as on I030 and I040. Device needed: the cheapest class with a commercial product for the substitute measurement. Herd Navigator (P012), an inline milk analyser of progesterone, LDH and BHB whose aim states heat measurement, is farm_fixed under the milk analyser line of rule 4.4; the other 30 aims naming heat detection or monitoring are collars, leg tags and ear tags, animal_mounted. The electronic nose analyses a sample and is not automatic, and the human biosensors are worn and under development; neither has an appendix row. So device needed is unsure, with two candidates. farm_fixed, if the appendix word heat is read as oestrus: Maroto Molina use heat duration and oestrus monitoring in the same passage (page 3), and Stygar calls these tools estrus detection (pages 3 and 9); Herd Navigator is then the cheapest. Or no commercial product for the substitute, because no aim states oestrus, which leaves the class among technologies with no named type. The missing rule is whether an aim word that is a common synonym of the measurement states it. Listed in open_questions.md. The 31 heat aims are not counted in vendors naming it, because heat is the substitute, not the measure, the same treatment as water intake on I030.</t>
+          <t>A substitute measure, so research_only under rules.md rule 4.2, whatever the products for the substitute; the grade does not credit them, as on I030 and I040. Device needed: the cheapest class with a commercial product for the substitute measurement. Herd Navigator (P012), an inline milk analyser of progesterone, LDH and BHB whose aim states heat measurement, is farm_fixed under the milk analyser line of rule 4.4; the other 30 aims naming heat detection or monitoring are collars, leg tags and ear tags, animal_mounted. The electronic nose analyses a sample and is not automatic, and the human biosensors are worn and under development; neither has an appendix row. So device needed is unsure, with two candidates. farm_fixed, if the appendix word heat is read as oestrus: Maroto Molina use heat duration and oestrus monitoring in the same passage (page 3), and Stygar calls these tools estrus detection (pages 3 and 9); Herd Navigator is then the cheapest. Or, because no aim states oestrus, no commercial product for the substitute, so rule 4.4 takes the cheapest class among the technologies proposed: animal_mounted, for the worn biosensors, although Maroto Molina's oestrus monitoring itself names no technology. The missing rule is whether an aim word that is a common synonym of the measurement states it. Listed in open_questions.md. The 31 heat aims are not counted in vendors naming it, because heat is the substitute, not the measure, the same treatment as water intake on I030.</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>A sample or a scoring by a person</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>No product and not discussed, so none. Device needed sample_or_procedure because the method named in the indicator is a milk sample sent for laboratory culture, read as a sample of the kind the rule 4.4 class list names (a blood or rumen sample). The other reading, none, also scores 0. Mastiline Luci names a mastitis sensor only in its sensor type, and only the aim column is read, so it is not cited.</t>
+          <t>No product and not discussed, so none. Device needed is unsure, with two candidates: sample_or_procedure, if a milk sample sent for laboratory culture, the method named in the indicator, is read as a sample of the kind the rule 4.4 class list names; or none, because that list names only a blood or rumen sample and no sensor source names a technology for the row. The missing rule is whether a milk sample for laboratory analysis is such a sample. Both score 0. Listed in open_questions.md. Mastiline Luci names a mastitis sensor only in its sensor type, and only the aim column is read, so it is not cited.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Product links checked again (product_links.csv, rule 4.10) and found_along_the_way.md, a record of where the sources disagree.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -754,36 +754,40 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
+          <t>Product list: links</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Link (2021) is the link the Stygar team printed in their spreadsheet. On the date in Checked, each was opened again. Works or Moved: it still opens a page that names the product. Wrong page: it opens a page that does not, such as a dealer's page, a parked domain or an unrelated site. Broken: an error or no answer. Link today is the maker's current page for the product where one was found, otherwise the nearest live maker page, as the next column says. 2_research/product_links.csv holds the same, with the rule in 2_research/rules.md, rule 4.10. The links change no grade, count or score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Ease of adoption score</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>0 to 15, five factors of 0 to 3 added together (2_research/rules.md, section 5). Ties are sorted by indicator id. A sort order, not a welfare judgement. Score parts are shown in the order: sensor + device + vendors + FARM + schemes.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>WHAT THIS DOES NOT SHOW</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>The sensor evidence is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products, studies and links are as those papers found them; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>'Tested' means a published study tested the product for the measure, as Stygar 2021 coded it; many of those tests fell below Stygar's high performance bar, which the column 'What was tested, and how well' shows.</t>
         </is>
       </c>
     </row>
@@ -791,7 +795,7 @@
       <c r="A31" s="3" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>The certification schemes have been read for every indicator.</t>
+          <t>'Tested' means a published study tested the product for the measure, as Stygar 2021 coded it; many of those tests fell below Stygar's high performance bar, which the column 'What was tested, and how well' shows.</t>
         </is>
       </c>
     </row>
@@ -799,45 +803,53 @@
       <c r="A32" s="3" t="inlineStr"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no review by a welfare scientist is recorded in the repository.</t>
+          <t>The certification schemes have been read for every indicator.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no review by a welfare scientist is recorded in the repository.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO CHECK ANY CELL</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names and sensor types, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
-        </is>
-      </c>
+      <c r="A34" s="3" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Who checked it</t>
+          <t>HOW TO CHECK ANY CELL</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Before each push, an AI auditing agent checks the changes against the source pages; 2_research/audit_log.md lists the versions that passed. The author plans to spot check ten rows after each push; each spot check is logged in 2_research/decision_log.md with its date and the rows read.</t>
+          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names and sensor types, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>Who checked it</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Before each push, an AI auditing agent checks the changes against the source pages; 2_research/audit_log.md lists the versions that passed. The author plans to spot check ten rows after each push; each spot check is logged in 2_research/decision_log.md with its date and the rows read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
           <t>Built from</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>The tables in 2_research/ by 3_code/build_output.py. Do not edit this file by hand; change the tables and run the script.</t>
         </is>
@@ -1110,7 +1122,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7 lists Stepmetrix (54) under Locomotion score, commercial farm, in the lower performance column; page 7 text: all tools for physical condition and health were classified under lower performance, and locomotion score assessment was poor for 54. Table 1 page 6 places ref 54 in the independent validation column (Bicalho et al. 2007). Appendix aim for StepMatrix: analyzes gait pressure to detect limp, for lameness diagnosis. Maroto Molina page 3: accelerometers, pressure mats, image analysis, multi sensor systems.</t>
+          <t>Stygar Table 2 page 7 lists Stepmetrix (54) under Locomotion score, commercial farm, in the lower performance column; page 7 text: all tools for physical condition and health were classified under lower performance, and locomotion score assessment was poor for 54. Table 1 page 6 places ref 54 in the independent validation column (Bicalho et al. 2007). Appendix aim for StepMatrix, as printed: Analyzes gat pressure to detect limp, for lameness diagnosis (gat for gait). Maroto Molina page 3: accelerometers, pressure mats, image analysis, multi sensor systems.</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
@@ -12600,7 +12612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:O130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12612,6 +12624,12 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12660,6 +12678,36 @@
           <t>Link (2021)</t>
         </is>
       </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>The 2021 link today</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Link today</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>What the link today shows</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>What that page says</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Note on the link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -12697,6 +12745,32 @@
           <t>https://www.i4pd.co.uk/work/well-cow-bolus-ph-and-temperature-monitor/</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.i4pd.co.uk/</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Product not found on i4 Product Design site (design consultancy); Well Cow company listed as out of business; searched 'WellCow bolus pH temperature' and 'i4 product design Well Cow bolus'.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -12742,6 +12816,32 @@
           <t>https://www.afimilk.com/cow-monitoring</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afimilk.com/how-we-help/cow-monitoring/</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to Afimilk cow monitoring page, which lists AfiAct III only; page does not say AfiAct III replaces AfiAct II.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -12783,6 +12883,32 @@
           <t>https://www.afimilk.com/cow-monitoring</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afimilk.com/how-we-help/cow-monitoring/</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>AfiCollar is a smart sensor that collects data on each cow's eating</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -12824,6 +12950,32 @@
           <t>https://www.afimilk.com/parlor-automation</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afimilk.com/how-we-help/dairy-automation/</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>AfiLab is an inline milk analyzer</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -12861,6 +13013,32 @@
           <t>https://www.afimilk.com/parlor-automation</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afimilk.com/how-we-help/dairy-automation/</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Afimilk MPC &amp; Milk Meter</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -12898,6 +13076,36 @@
           <t>https://www.agersens.com/</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gallagher.eu/en_export/advice-inspiration/electric-fencing/eshepherd-virtual-fencing</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>eShepherd virtual fencing puts you in control of your cattle</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>agersens.com redirects through cu-bx.com and fronteer.us to an unrelated restaurant site; Gallagher (acquired Agersens 2021) sells eShepherd on its own site, though the page does not mention Agersens.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -12935,6 +13143,32 @@
           <t>https://www.agricam.se/sensorer?lang=en</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>https://agricam.se/</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Product not found on Agricam site, which now lists Bacticam, KlövKoll and other tools; searched 'Agricam CaDDi mastitis thermal camera' and 'Agricam CaDDi site:agricam.se'.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -12972,6 +13206,28 @@
           <t>https://www.agrismart.co.uk/farming-solutions/bolus/</t>
         </is>
       </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Domain does not resolve; searched 'Agrismart cattle bolus rumen temperature' and 'Agrismart UK bolus farming solutions', no maker site found.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -13013,6 +13269,36 @@
           <t>https://www.allflex.global/product/sensehub-dairy/</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msd-animal-health.co.uk/hub/sensehub/dairy/</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>SenseHub Dairy is a single, accessible source of insight</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Page states Allflex was acquired by MSD Animal Health in 2019.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -13054,6 +13340,32 @@
           <t>https://www.scrdairy.com/cow-intelligence/heatime-hr-system.html</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.msd-animal-health.co.uk/hub/sensehub/dairy/</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Old link redirects via allflex.global/product/heatimepro/ to msd.sensehub.com, which does not name Heatime; MSD page only says Heatime later evolved into SenseTime and then SenseHub, without naming Heatime HR or Hi-Tag.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -13091,6 +13403,36 @@
           <t>http://www.scrdairy.com/herd-intelligence/scr-heatime-hr-system.html</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.allflex.global/sea/product/heatime-pro/</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Heatime® Pro+ is a powerful, yet easy to use, PC-based system</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Old link redirects to msd.sensehub.com which does not name Heatime; product page found on Allflex Southeast Asia site.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -13128,6 +13470,36 @@
           <t>https://www.atlagri.com/about-us-2018/</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.atlagri.com/feeding</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Out of Parlour Feeding System</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Stygar's name is generic; the match to ATL's out of parlour feeding system is an inference.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -13165,6 +13537,28 @@
           <t>https://play.google.com/store/apps/details?id=com.bayer.bcscowdition&amp;hl=en</t>
         </is>
       </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>App delisted from Google Play; Bayer Animal Health went to Elanco in 2020 and no current Cowdition page found; bayer.com blocks fetching (403).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -13202,6 +13596,32 @@
           <t>http://www.biocontrol.no/products/controlling-and-recording-feed-intake/</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>https://biocontrol.no/products-2/controlling-and-recording-feed-intake/</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Controlling and Recording Feed Intake</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -13239,6 +13659,32 @@
           <t>https://biotic.com/calves/</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>https://biotic.com/calves/</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>The Biotic ID-TEK system is an easy-to-use calf feeding system</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -13276,6 +13722,36 @@
           <t>https://boumatic.com/us_es/productos/heatseeker-cow-monitoring-systems-us</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/products/realtime</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>RealTime Rumination &amp; Localisation</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>The page names RealTime Rumination &amp; Localisation; reading RL as that is an inference.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -13321,6 +13797,32 @@
           <t>https://kruegersboumatic.com/automation/stepmetrix/</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Old link is a live dealer page (Krueger's Bou-Matic, which sells and services BouMatic) naming StepMetrix; product not found on boumatic.com; searched 'BouMatic StepMetrix' and 'StepMetrix site:boumatic.com'.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -13358,6 +13860,32 @@
           <t>http://www.electromechagri.com/parlour-feeding-solutions/boumatic-calf-feeding-system/</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Old link was a dealer page; no BouMatic calf feeder found on boumatic.com; searched 'BouMatic calf feeder automatic calf feeding system'.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -13395,6 +13923,36 @@
           <t>https://boumatic.com/us_en/products/gemini-miking-robot-1-2</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/products/gemini-up/</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>The Gemini UP has had modifications from the previous Gemini model</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>The page names Gemini UP and says it has modifications from the previous Gemini model; it does not say it replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -13432,6 +13990,36 @@
           <t>https://boumatic.com/us_en/products/gemini-the-boumatic-milking-robot-1-1-1</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/products/gemini-up/</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>GEMINI UP DOUBLE BOX</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>The page names Gemini UP and says it has modifications from the previous Gemini model; it does not say it replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -13473,6 +14061,32 @@
           <t>https://www.cainthus.com/alus</t>
         </is>
       </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://ever.ag/</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>cainthus.com redirects to an Ever.Ag page now titled Maternity Warden that names neither Cainthus nor Alus; product not found on ever.ag.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -13510,6 +14124,28 @@
           <t>http://www.cattle-watch.com/</t>
         </is>
       </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Domain is a parked page that redirects to /lander; company later renamed Herd-itt and reported as ceased operating; no maker site found.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -13547,6 +14183,36 @@
           <t>https://www.cerestag.com/benefits/</t>
         </is>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://cerestag.com/</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>CERES TAG is a smart ear tag for animals</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Benefits page gone; the live home page names the product.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -13588,6 +14254,36 @@
           <t>https://ida.io/ida-for-farmers/</t>
         </is>
       </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://ida.io/</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Datamars Livestock and ida</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>ida.io now shows a redirect notice to Datamars Livestock, which bought Ida for Farmers in 2023; no Ida product page found on the Datamars Livestock site.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -13633,6 +14329,32 @@
           <t>https://www.cowmanager.com/en-us/</t>
         </is>
       </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cowmanager.com/</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>CowManager Ear Sensor</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -13670,6 +14392,36 @@
           <t>https://www.crv4all-international.com/service/ovalert/</t>
         </is>
       </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>https://crv4all.com/en/how-ovalert-works</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>How Ovalert works</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>The page names Ovalert but not the neck tag.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -13707,6 +14459,36 @@
           <t>https://www.crv4all-international.com/service/ovalert/</t>
         </is>
       </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>https://crv4all.com/en/how-ovalert-works</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>How Ovalert works</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>The page names Ovalert but not the leg tag.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -13748,6 +14530,32 @@
           <t>https://www.dairymaster.com/products/moomonitor/</t>
         </is>
       </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dairymaster.com/products/moomonitor/</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>The MooMonitor+ monitors cow neck movements 24×7</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -13785,6 +14593,36 @@
           <t>http://dairycare.co.za/product/activity-meter-system/</t>
         </is>
       </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-us/farm-solutions/farm-management/delaval-delpro/precision-analytics/delpro-activity-meters/</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>With DeLaval Activity Meters you are monitoring your cows</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Old link was a dealer page; DeLaval's own delaval-activity-meter-system URL redirects to this DelPro Activity meters page.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -13830,6 +14668,36 @@
           <t>http://www.delavalcorporate.com/our-products-and-services/farm-support/delaval-body-condition-scoring-bcs/</t>
         </is>
       </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-ca/knowledge-hub/educational-content/trending-topics/delaval-body-condition-scoring-bcs/</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval Body Condition Scoring (BCS)™</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>delavalcorporate.com refuses connections.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -13867,6 +14735,32 @@
           <t>https://www.delaval.com/en-ie/our-solutions/milking/udder-health--hygiene/milk-testing/delaval-cell-counter-dcc/#:~:text=Precise%20and%20fast%20somatic%20cell%20count%20measurement&amp;text=DeLaval%20cell%20counter%20DCC%20counts,act%20as%20fast%20as%20possible.</t>
         </is>
       </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-ie/milking-essentials/milking-accesories/occ-dcc/</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>The OCC &amp; DCC accurately measure your herd, cow or cow quarter somatic cell count.</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -13904,6 +14798,36 @@
           <t>https://www.delaval.com/en-nz/our-solutions/milking/udder-health--hygiene/milk-testing/delaval-online-cell-counter-occ/</t>
         </is>
       </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-nz/milking-essentials/milking-accesories/occ-dcc/</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>OCC &amp; DCC</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Old link redirects to the Cleaning &amp; Hygiene page; OCC now shares a page with DCC, and the page title reads OCC &amp; DCC, DeLaval.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -13941,6 +14865,32 @@
           <t>https://www.delaval.com/en-ie/our-solutions/feeding/feed-stations/delaval-feed-stations-fsc40-and-fsc400/</t>
         </is>
       </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Old link redirects to the general Feeding page; FSC40/FSC400 not found on delaval.com; searched 'DeLaval feed station FSC400 delaval.com' and '\FSC400\" DeLaval feed station concentrate'."</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -13978,6 +14928,36 @@
           <t>http://www3.delaval.com/ImageVaultFiles/id_198/cf_5/DeLaval_calf_feeders.PDF</t>
         </is>
       </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-in/farm-solutions/feeding/calf-feeders/</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval calf feeder CF150X</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>www3.delaval.com no longer resolves; product named in the page's rendered content (WebFetch sees only the title Calf Feeders)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -14015,6 +14995,36 @@
           <t>http://www3.delaval.com/ImageVaultFiles/id_198/cf_5/DeLaval_calf_feeders.PDF</t>
         </is>
       </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-gb/farm-solutions/feeding/calf-feeders/delaval-calf-feeder-cf500-cf1000/</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval calf feeder CF500+ &amp; CF1000+</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>www3.delaval.com no longer resolves</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -14052,6 +15062,36 @@
           <t>http://www3.delaval.com/ImageVaultFiles/id_198/cf_5/DeLaval_calf_feeders.PDF</t>
         </is>
       </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-gb/farm-solutions/feeding/calf-feeders/delaval-calf-feeder-cf500-cf1000/</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval calf feeder CF500+ &amp; CF1000+</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>www3.delaval.com no longer resolves</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -14089,6 +15129,36 @@
           <t>http://www.delavalcorporate.com/our-products-and-services/milking/automatic-milking/</t>
         </is>
       </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-nz/farm-solutions/milking/delaval-amr/delaval-automatic-milking-rotary-amr</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval Automatic Milking Rotary AMR™</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>delavalcorporate.com refuses connections</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -14126,6 +15196,36 @@
           <t>http://www.delavalcorporate.com/our-products-and-services/milking/automatic-milking/#/-/Product-Information1/Milking/Systems/Automatic/</t>
         </is>
       </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-gb/templates/delaval-vms-series</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval VMS™ - Robotic Milking System</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>delavalcorporate.com refuses connections; current page covers the VMS V300 series</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -14167,6 +15267,36 @@
           <t>https://www.delaval.com/en-ie/our-solutions/farm-management/delpro-precision-analytics/herd-navigator/</t>
         </is>
       </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.delaval.com/en-ie/farm-solutions/farm-management/delaval-delpro/precision-analytics/</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>DeLaval Herd Navigator™ enables progressive dairy farmers to</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to the Precision Analytics page; product named in rendered page content (WebFetch sees only the title)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -14204,6 +15334,36 @@
           <t>https://digitanimal.com/?lang=en</t>
         </is>
       </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>https://digitanimal.com/?lang=en</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Digitanimal EVO – GPS Tracker</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Stygar name is generic; page lists EVO; ECO and SAT GPS collars</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -14241,6 +15401,36 @@
           <t>https://www.doowa-rfid.com/ruminal-bolus/hdx-rfid-rumen-bolus-67-5g</t>
         </is>
       </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.doowa-rfid.com/</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>HDX RFID Rumen Bolus (67.5g)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Home page lists the product but its own product link (/products/hdx-rfid-rumen-bolus-67-5g) also returns 404</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -14286,6 +15476,28 @@
           <t>https://ecow.co.uk/</t>
         </is>
       </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Domain lapsed and now redirects to a UK domain backorder service; searched 'eCow eBolus' and 'eCow Ltd Toby Mottram' with no new maker site</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -14323,6 +15535,28 @@
           <t>https://eiodiagnostics.com/technology/</t>
         </is>
       </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>eiodiagnostics.com now redirects to an unrelated pizza site; press says the product became UdderHealth but no maker page confirms it</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -14360,6 +15594,32 @@
           <t>https://www.eli-innovation.com.au/smart-paddock-feeder.html</t>
         </is>
       </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eli-innovation.com.au/smart-paddock-feeder.html</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Eli Smart Paddock Feeder</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -14401,6 +15661,36 @@
           <t>http://www.engs-dairy.com/</t>
         </is>
       </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.engs-dairy.com/</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>We purchased Track a))) Cow system</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Named in customer reviews on the home page</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -14438,6 +15728,32 @@
           <t>https://www.farmtec.cz/en/milking-robot-galaxy-519.html</t>
         </is>
       </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.farmtec.cz/en/</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Farmtec home page live but no Galaxy robot; searched 'Farmtec Galaxy milking robot'</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -14479,6 +15795,32 @@
           <t>https://www.icerobotics.com/wp-content/uploads/2019/07/Lameness-Detection_June19.pdf</t>
         </is>
       </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.peacocktechnology.com/</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>icerobotics.com now redirects to Peacock Technology; PDF 404s; site names CowAlert and IDS i-QUBE but not IceTag</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -14524,6 +15866,36 @@
           <t>https://www.icerobotics.com/wp-content/uploads/2019/07/Lameness-Detection_June19.pdf</t>
         </is>
       </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.peacocktechnology.com/cowalert</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>CowAlert is a data processing and analysis tool</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>icerobotics.com/cowalert redirects here; page names CowAlert but not IceQube</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -14561,6 +15933,36 @@
           <t>http://www.felixcan.com/eng/Ruminal_Bolus.html</t>
         </is>
       </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>http://www.felixcan.com/eng/Ruminal_Bolus.html</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Technical File 74g Bolus</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>EI9024 appears only in the name of a linked technical file.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -14598,6 +16000,32 @@
           <t>https://www.flir.com/products/ax8-automation/</t>
         </is>
       </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flir.com/products/ax8-automation/</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>FLIR AX8 Thermal Imaging Camera For Condition and Safety Monitoring</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -14635,6 +16063,32 @@
           <t>https://www.flir.eu/</t>
         </is>
       </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.flir.com/en-eu/</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>flir.eu redirects to the Teledyne FLIR EU home page; none of the listed legacy cameras named; searched 'FLIR T300' and found only resellers</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -14672,6 +16126,36 @@
           <t>https://www.fluke.com/en/product/thermal-cameras/ti45ft</t>
         </is>
       </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fluke.com/en/product/thermal-cameras/ti45ft</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Fluke Ti45FT IR FlexCam® Thermal Imager</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>The page names the Ti45FT IR FlexCam; the word Pro is not on it.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -14709,6 +16193,32 @@
           <t>http://www.fofia.com/</t>
         </is>
       </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>http://www.fofia.com/</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Wuxi Fofia home page (Chinese) lists rumen tags but not ET912 or a pH bolus; https refuses connections so only http loads</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -14746,6 +16256,36 @@
           <t>https://www.followit.se/livestock/index.html</t>
         </is>
       </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.followit.se/livestock/index.html</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Pellego väger endast 175 gram</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>Page spells it Pellego; Stygar wrote Pellegro</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -14783,6 +16323,36 @@
           <t>https://www.followit.se/livestock/index.html</t>
         </is>
       </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.followit.se/</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>Tellus 2 (Tellus Ultra Light, Light, Small, Medium</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Livestock page does not name Tellus; home page names Tellus 2 only in its customer login list; no product page found</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -14820,6 +16390,36 @@
           <t>https://www.foerster-technik.com/</t>
         </is>
       </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foerster-technik.com/</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>COMPACT Smart</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Named in the home page menu under Automatic Calf Feeder</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -14857,6 +16457,36 @@
           <t>https://www.foerster-technik.com/</t>
         </is>
       </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foerster-technik.com/</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>VARIO Smart</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Named in the home page menu under Automatic Calf Feeder</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -14894,6 +16524,32 @@
           <t>https://www.foerster-technik.com/smart-calf-system-en/</t>
         </is>
       </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foerster-technik.com/</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to the Calf management page which does not name Smart Calf System; searched 'Förster-Technik Smart Calf System'</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -14931,6 +16587,32 @@
           <t>https://www.foerster-technik.com/smart-calf-system-en/</t>
         </is>
       </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foerster-technik.com/calf-management/</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>The Smart NeckBand identifies less active or conspicuous calves</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -14968,6 +16650,32 @@
           <t>https://fullwoodpacko.com/products/cow-monitoring-and-herd-management/crysta-lab-milk-analyser/</t>
         </is>
       </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>https://fullwood.com/en/</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>fullwoodpacko.com is now a parked reserved domain; Fullwood site names Crystal software and FULLSENSE but not Crysta Lab</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -15005,6 +16713,32 @@
           <t>https://fullwoodpacko.com/</t>
         </is>
       </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>https://fullwood.com/en/</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>fullwoodpacko.com is now a parked reserved domain; Vitality not found on fullwood.com</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -15042,6 +16776,36 @@
           <t>https://fullwoodpacko.com/products/robotic-milking/</t>
         </is>
       </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>https://fullwood.com/en/solutions/robotic-milking/merlin/</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>cows stand relaxed in the M²erlin milking robot</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>fullwoodpacko.com is parked; page headings use Merlin 2+ and the body says M²erlin</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -15079,6 +16843,32 @@
           <t>http://www.gea-cowview.com/</t>
         </is>
       </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>gea-cowview.com no longer resolves; no CowView page on gea.com; positioning now sold under CowScout but GEA does not say it replaces CowView</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -15116,6 +16906,32 @@
           <t>https://www.gea.com/en/products/milking-farming-barn/dairybarn-farm-equipment/barn-handling-routing/cow-treatment/animal-scale-taxatron-5000.jsp</t>
         </is>
       </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>Old URL redirects to a 404; searched 'GEA Taxatron animal scale' with no maker page</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -15161,6 +16977,36 @@
           <t>https://www.accelgen.com/upload/product/files/english/0412gea-cow-scout-brochure-lr.pdf</t>
         </is>
       </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/gea-herd-management/activity-detection-cowscout/</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>CowScout – Smart dairy herd monitoring</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>The page names CowScout but not the S variant; the 2021 link was a GEA brochure on a third party site.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -15198,6 +17044,36 @@
           <t>https://www.gea.com/en/products/calf-feeder-dairyfeed-j.jsp</t>
         </is>
       </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/dairyfeed-feeding-systems/calf-feeders/dairyfeed-f4110-f4120/</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>J C400 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -15235,6 +17111,36 @@
           <t>https://www.gea.com/en/products/calf-feeder-dairyfeed-j.jsp</t>
         </is>
       </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/dairyfeed-feeding-systems/calf-feeders/dairyfeed-f4110-f4120/</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>V600 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -15272,6 +17178,36 @@
           <t>https://www.gea.com/en/products/calf-feeder-dairyfeed-j.jsp</t>
         </is>
       </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/dairyfeed-feeding-systems/calf-feeders/dairyfeed-f4110-f4120/</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>V640 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -15309,6 +17245,32 @@
           <t>https://www.gea.com/en/products/automatic-feeding-dairyfeed-c-8000.jsp</t>
         </is>
       </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/dairyfeed-feeding-systems/calf-feeders/</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to the GEA calf feeders page, which does not name C 8000; searched 'GEA DairyFeed C 8000' with no GEA page found.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -15346,6 +17308,32 @@
           <t>https://www.gea.com/en/products/dairymilk-m6850-cell-count-sensor.jsp</t>
         </is>
       </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/milking-solutions/automatic-milking/dairymilk-m6850-cell-count-sensor/</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>GEA Dairy Milk M6850 Cell Count Class Sensor</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -15383,6 +17371,32 @@
           <t>https://www.gea.com/en/products/milking-farming-barn/dairyrobot-automated-milking/dairyrobot-r9500-robotic-milking-system.jsp</t>
         </is>
       </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/milking-solutions/automatic-milking/dairyrobot-r9500/</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>DairyRobot R9500</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -15420,6 +17434,32 @@
           <t>https://www.gea.com/en/products/milking-farming-barn/dairyrobot-automated-milking/rotary-parlor-dairyproq.jsp</t>
         </is>
       </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gea.com/en/products/milking-farming-barn/milking-solutions/automatic-milking/dairyproq/</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>GEA DairyProQ robotic milking carousel</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -15461,6 +17501,32 @@
           <t>https://growsafe.com/our-platform/</t>
         </is>
       </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>https://vytelle.com/our-platform</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>Link is 404 and growsafe.com now redirects to vytelle.com; Vytelle describes its own feed intake system but its visible text never names GrowSafe or a feed alley.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -15498,6 +17564,28 @@
           <t>https://www.animalhealthmonitoring.com/</t>
         </is>
       </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr"/>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>animalhealthmonitoring.com shows a Wix domain error and herdinsights.com refuses connections; searched 'HerdInsights cow collar' and found only third party pages.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -15539,6 +17627,28 @@
           <t>https://www.animalhealthmonitoring.com/</t>
         </is>
       </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>animalhealthmonitoring.com shows a Wix domain error and herdinsights.com refuses connections; searched 'HerdInsights smart collar' and found only third party pages.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -15576,6 +17686,32 @@
           <t>https://www.hetwin.at/en/hetwin-feed-concentrates-equipment.html</t>
         </is>
       </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hetwin.at/en/hetwin-feed-concentrates-equipment.html</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>HETWIN FEED CONCENTRATES EQUIPMENT</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -15617,6 +17753,36 @@
           <t>https://www.hokofarmgroup.com/ric/</t>
         </is>
       </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>https://hokofarmgroup.com/products/ric2discover/</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>our RIC system</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>Redirects to the RIC2DISCOVER page, which names the RIC system but does not say RIC2DISCOVER replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -15654,6 +17820,36 @@
           <t>https://www.holm-laue.de/index.php/hl100?ln=en-GB#ad-image-0</t>
         </is>
       </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.holm-laue.de/calfexpert/</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>im Vergleich zum Vorgänger H&amp;L 100</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>German CalfExpert page calls the H&amp;L 100 its predecessor (Vorgänger).</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -15691,6 +17887,36 @@
           <t>https://store.calfstar.com/products/automatic-calf-feeders?_pos=7&amp;_sid=10f9fd176&amp;_ss=r</t>
         </is>
       </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>https://store.calfstar.com/products/automatic-calf-feeders</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>The Calf Star Double Jug is connected to the CalfExpert</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>This is the store of Calf Star, a seller of Holm &amp; Laue CalfExpert feeders, not the maker's own site.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -15728,6 +17954,36 @@
           <t>https://www.holm-laue.de/index.php/calfguide</t>
         </is>
       </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.holm-laue.de/calfguide/</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>CalfExpert Tränkeautomaten</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>Link opens the CalfGuide page, which names CalfExpert; Holm &amp; Laue also has a dedicated page at holm-laue.de/calfexpert/.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -15765,6 +18021,36 @@
           <t>https://www.holm-laue.de/index.php/hygiene-station?ln=en-GB#ad-image-0</t>
         </is>
       </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.holm-laue.de/hygienestation/</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Hier setzt die HygieneStation von Holm &amp; Laue DEN neuen Standard</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>Old index.php address is 404; the HygieneStation page is on the current Holm &amp; Laue site (German).</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -15802,6 +18088,32 @@
           <t>https://www.holm-laue.de/index.php/calfguide</t>
         </is>
       </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.holm-laue.de/calfguide/</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Mit CalfGuide erhalten Sie eine Managementsoftware</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -15843,6 +18155,36 @@
           <t>https://www.rumiwatch.ch/</t>
         </is>
       </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rumiwatch.com/</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>RumiWatchSystem</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>rumiwatch.ch redirects to rumiwatch.com.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -15880,6 +18222,36 @@
           <t>http://jfcagri.com/cattle/evolution-calf-feeder/evo-s4/</t>
         </is>
       </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>https://jfcevolution.com/</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>The JFC Evolution Automatic Calf Feeder</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>Old page is 404; the JFC Agri site links its automatic calf feeder to jfcevolution.com, which lists the Evolution S4.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -15917,6 +18289,32 @@
           <t>https://www.lely.com/media/filer_public/77/81/7781ea55-1a10-4aa1-9a70-d80de1e28360/lely_dairy_equipment_en.pdf</t>
         </is>
       </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/barn/tags/</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>Brochure PDF is 404; the Lely tags page names no tag models; a Lely Australia page names a 'Qwes LD-HD' but does not say it is the HR-LD.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -15954,6 +18352,36 @@
           <t>https://www.lely.com/solutions/feeding/calm/</t>
         </is>
       </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/feeding/calm/</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>The Lely Calm helps dairy farmers achieve optimal growth.</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>The page names Lely Calm but not the Compact + model.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -15991,6 +18419,36 @@
           <t>https://www.lely.com/media/filer_public/fc/bf/fcbf8779-20ee-4eec-aeaa-7c8cf218587b/lely_calm_en.pdf</t>
         </is>
       </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/feeding/calm/</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>The Lely Calm helps dairy farmers achieve optimal growth.</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>The page names Lely Calm but not the Vario + model.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -16028,6 +18486,36 @@
           <t>https://www.lely.com/solutions/feeding/cosmix/</t>
         </is>
       </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/barn/</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>The Cosmix, in conjunction with the Astronaut and the Lely Tags</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>Cosmix page redirects to the Lely barn solutions page, which has a Cosmix section.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -16069,6 +18557,32 @@
           <t>https://www.lely.com/solutions/milking/astronaut-a4/</t>
         </is>
       </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/milking/astronaut/</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>Astronaut page now sells the Astronaut A5 Next; A4 appears only in a customer quote and the page does not say the A5 replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -16110,6 +18624,36 @@
           <t>https://www.lely.com/news/2015/03/20/caring-milk-quality-together/</t>
         </is>
       </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/farming-insights/lely-mqc-c-supports-dry-cow-therapy/</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>How the Lely MQC-C supports selective dry cow therapy</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>2015 news page is 404; this is a Lely article page about the MQC-C, no standalone product page found.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -16147,6 +18691,32 @@
           <t>https://www.licautomation.com/products/milk-monitoring/</t>
         </is>
       </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lic.co.nz/</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr"/>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>licautomation.com refuses connections; LIC sold LIC Automation to MSD Animal Health in 2021 and no maker page for Saber Milk was found.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -16184,6 +18754,32 @@
           <t>https://www.lic.co.nz/products-and-services/automation/protrack-body-condition-scoring/</t>
         </is>
       </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lic.co.nz/</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>LIC page is 404; LIC home shows only a ProTrack login link; automation business sold to MSD Animal Health in 2021; no maker page found.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -16221,6 +18817,32 @@
           <t>https://www.lic.co.nz/products-and-services/automation/protrack-scc/</t>
         </is>
       </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lic.co.nz/</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>LIC page is 404; LIC home shows only a ProTrack login link; automation business sold to MSD Animal Health in 2021; no maker page found.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -16258,6 +18880,32 @@
           <t>https://www.lotek.com/products/activity-sensor/</t>
         </is>
       </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lotek.com/products/activity-sensor/</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Activity Sensor for Lotek Collars</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -16295,6 +18943,36 @@
           <t>https://www.lotek.com/products/?segment=terrestrial</t>
         </is>
       </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lotek.com/products/?segment=terrestrial</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>LiteTrack Iridium 130 - 150</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>The page lists LiteTrack Iridium and other Lotek collars; LiteTrack 330 or 420 is not named.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -16332,6 +19010,28 @@
           <t>https://www.mastiline.com/products/luci/</t>
         </is>
       </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>mastiline.com now redirects to a parked /lander page; searched 'Mastiline Luci' and 'Mastiline' and found no maker site.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -16369,6 +19069,32 @@
           <t>https://www.medria.fr/en/solutions/velphone/</t>
         </is>
       </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>https://medria.com/</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>www.medria.fr fails the SSL handshake; medria.fr redirects to medria.com, which does not name Vel'Phone or a calf temperature bolus.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -16406,6 +19132,32 @@
           <t>https://www.medria.fr/en/solutions/velphone/</t>
         </is>
       </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>https://medria.com/farmlife-livestock</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr"/>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>FarmLife Livestock page describes a connected collar but never names Bouquet or says it replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -16443,6 +19195,32 @@
           <t>https://milkomax.com/en/robomax/</t>
         </is>
       </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>https://milkomax.com/en/robomax/</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>THE SUCCESS OF ROBOMAX IS BASED ON 3 KEY FACTORS</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -16480,6 +19258,36 @@
           <t>http://www.milkrite-interpuls.co.uk/precision-farming.htm</t>
         </is>
       </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>http://www.milkrite-interpuls.co.uk/precision-farming.htm</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>The milkrite | InterPuls Neck Tags offer peace of mind to the farmer</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>Only change is http to https.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -16517,6 +19325,36 @@
           <t>http://www.milkrite-interpuls.co.uk/precision-farming.htm</t>
         </is>
       </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>https://ecommerce-uk.interpuls.com/products/herd-management-2/heat-detection-health-monitoring/set-10x-pedometers-uhf-heat-det-en.html</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>5550242 - Set Leg Pedometer UHF (10X)</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>2021 page now lists neck tags only; leg pedometer found on the InterPuls S.p.A. own web shop.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -16554,6 +19392,28 @@
           <t>https://moonsyst.com/home</t>
         </is>
       </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr"/>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>moonsyst.com refuses connections on every address tried; searched 'Moonsyst smart rumen bolus', only third party pages describe it.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -16591,6 +19451,28 @@
           <t>https://moonsyst.com/collar</t>
         </is>
       </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>moonsyst.com refuses connections; searched 'moonsyst.com smart collar heat detection', no collar found, only the bolus.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -16628,6 +19510,28 @@
           <t>http://moow.farm/</t>
         </is>
       </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr"/>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t>Domain moow.farm no longer resolves; searched 'Moow rumen bolus Hungary' and 'MOOW bolus pH sensor', only directories found.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -16665,6 +19569,36 @@
           <t>https://www.nedap-livestockmanagement.com/wp-content/uploads/2017/07/Nedap-Smarttag-Neck.pdf</t>
         </is>
       </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>https://nedap-livestockmanagement.com/smarttag-neck-ear/</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Nedap SmartTag Neck</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>2021 PDF returns server error 500.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -16706,6 +19640,36 @@
           <t>https://www.nedap-livestockmanagement.com/dairy-farming/solutions/nedap-cowcontrol/</t>
         </is>
       </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>https://nedap-livestockmanagement.com/solutions/nedap-cowcontrol/</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Nedap CowControl</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>Same page also spells the tag 'Smarttag Neck'.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -16747,6 +19711,36 @@
           <t>https://www.nedap-livestockmanagement.com/dairy-farming/solutions/nedap-cowcontrol/</t>
         </is>
       </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>https://nedap-livestockmanagement.com/solutions/nedap-cowcontrol/health-monitoring/</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>The Smarttag Leg does the same for standing, lying and walking</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>2021 link redirects to the CowControl page, which does not name the leg tag.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -16784,6 +19778,32 @@
           <t>https://www.nedap-livestockmanagement.com/dairy-farming/solutions/electronic-concentrate-feeding/</t>
         </is>
       </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>https://nedap-livestockmanagement.com/solutions/nedap-farmcontrol/feeding/</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Nedap Cow Feeding Station</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -16821,6 +19841,36 @@
           <t>https://www.tracks360.com/asset-tracking-solutions/gps-rfid-tracking-industries/cattle-bolus/</t>
         </is>
       </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>https://tracks360.com/cattle-bolus/</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Key Features of ActiveHerd™</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>Same Tracks360 site, now under Smarter Technologies Group; product written ActiveHerd.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -16858,6 +19908,36 @@
           <t>http://www.pearson-international.com/dairy-systems-milking-machines/heat-detection-with-health-monitoring</t>
         </is>
       </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>https://pearsonmilking.com/heat-detection-and-health-monitoring/</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>SmartTag System</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t>The page names the SmartTag System but not the neck version.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -16895,6 +19975,32 @@
           <t>http://www.pearson-international.com/dairy-systems-milking-machines/robotic-milking/astrea-milking-robot</t>
         </is>
       </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>https://pearsonmilking.com/</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr"/>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>Old domain redirects to a malformed address; Pearson site no longer lists robots or Astrea. Third party sources tie Astrea 20.20 to AMS Galaxy.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -16932,6 +20038,36 @@
           <t>http://www.prosagri.net/en/prodotti/alimentazione-computerizzata-per-bovini/stazioni-di-alimentazione/</t>
         </is>
       </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Moved, still works</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prosagri.net/prodotti/alimentazione-computerizzata-per-bovini/stazioni-di-alimentazione/</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>DAP 3: stazione di alimentazione automatica</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>English path now redirects to the Italian page.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -16969,6 +20105,32 @@
           <t>https://sacmilking.com/our-solutions/robotic-dairy-solution/</t>
         </is>
       </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/eu_en/</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>sacmilking.com home now redirects to BouMatic Europe; Futureline not listed there; searched 'SAC Christensen RDS Futureline MAX robot'.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -17006,6 +20168,32 @@
           <t>https://www.agriexpo.online/prod/sac-christensen-co/product-175064-16344.html</t>
         </is>
       </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K115" s="2" t="inlineStr">
+        <is>
+          <t>https://boumatic.com/eu_en/</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr"/>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>2021 link is an AgriExpo marketplace page that blocks scripts (403); FDS3 not found on the maker site, which redirects to BouMatic.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -17043,6 +20231,32 @@
           <t>https://www.sensolus.com/</t>
         </is>
       </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sensolus.com/</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr"/>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>Sensolus home page covers industrial asset trackers only; the source row pairs a SAC robot name with Sensolus.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -17088,6 +20302,28 @@
           <t>https://www.smartbow.com/en/how-it-works.aspx</t>
         </is>
       </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr"/>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>smartbow.com is a parked domain for sale; Zoetis bought Smartbow but its precision livestock page does not name it.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -17125,6 +20361,36 @@
           <t>https://www.smartstock-usa.com/how-smartstock-works-you</t>
         </is>
       </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.smartstock-usa.com/</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>digestive track (rumen) bolus that specifically monitors the health and conditions</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>2021 subpage is 404; home page describes the SmartStock bolus.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -17162,6 +20428,32 @@
           <t>https://smaxtec.com/en/</t>
         </is>
       </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>https://www.smaxtec.com/en/</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr"/>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>Site names Classic Bolus and pH Bolus but never 'basic'; no page says either replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -17203,6 +20495,32 @@
           <t>https://smaxtec.com/en/</t>
         </is>
       </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.smaxtec.com/en/</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>Maker's home page only</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr"/>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>Site names Classic Bolus and pH Bolus but never 'premium'; no page says either replaces it.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -17240,6 +20558,32 @@
           <t>https://www.system-happel.de/en/index.php?pg=fuetterung.php</t>
         </is>
       </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>https://www.system-happel.de/en/index.php?pg=fuetterung.php</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>In the feeding station, each cow is supplied with exactly</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -17277,6 +20621,32 @@
           <t>https://www.system-happel.de/en/index.php?pg=aktivpuls-robot2020.php</t>
         </is>
       </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.system-happel.de/en/index.php?pg=aktivpuls-robot2020.php</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>TIM AktivPuls® Robot</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -17314,6 +20684,32 @@
           <t>https://taggle.com/smart-agriculture/</t>
         </is>
       </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>https://taggle.com/smart-agriculture/</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>Maker's site, product not on it</t>
+        </is>
+      </c>
+      <c r="M123" s="2" t="inlineStr"/>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O123" s="2" t="inlineStr">
+        <is>
+          <t>Page describes Calf Alert, a calving locator read by land based receivers, but never names a radiolocation tracking system.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -17351,6 +20747,36 @@
           <t>http://www.urban-feeder.com/fileadmin/user_upload/mediacenter/alma-pro/en-alma-pro-katalog/index.html#16</t>
         </is>
       </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.urbanonline.de/en/urban-products/detail/urban-alma-pro</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>The Urban Alma Pro supports you with this on all levels.</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>Catalogue redirects to urbanonline.de and returns 404.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -17388,6 +20814,28 @@
           <t>https://angel.co/company/vitalherd</t>
         </is>
       </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M125" s="2" t="inlineStr"/>
+      <c r="N125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>The link redirects to a profile on wellfound.com, a third party site; no VitalHerd site of its own was found.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -17425,6 +20873,36 @@
           <t>https://www.waikatomilking.com/products/automation/rotary-automation/ecr-plus/optional-features/smartd-tect/</t>
         </is>
       </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>https://waikatomilking.com/products/milking-point-products/pulsators/smartd-tect</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>SmartD-TECT performs a health analysis of each quarter of the udder</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>Now filed under pulsators.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -17462,6 +20940,36 @@
           <t>https://workswell-thermal-camera.com/thermal-imaging-camera-smartis-industrial/</t>
         </is>
       </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>https://workswell.eu/thermal-monitoring-of-casting-ladle-during-processes/</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>Enter Workswell's SMARTIS thermographic system</t>
+        </is>
+      </c>
+      <c r="N127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>Only a Workswell case study names SMARTIS; the model 336 is not named.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -17499,6 +21007,36 @@
           <t>https://workswell-thermal-camera.com/workswell-wiris-pro-sc-thermal-inspection-camera-with-ultrazoom/</t>
         </is>
       </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>Wrong page</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>https://workswell.eu/thermal-drone-camera-inspection-wiris-pro/</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>The Workswell WIRIS Pro is a fully radiometric thermal camera</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>Old domain redirects to an unrelated spam site; Workswell now on workswell.eu.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -17536,6 +21074,28 @@
           <t>https://www.zeddy.com/zeddy-500/</t>
         </is>
       </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr"/>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M129" s="2" t="inlineStr"/>
+      <c r="N129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>zeddy.com no longer resolves; searched 'Zeddy calf feeder 500 1250' and 'Zeddy Ellison website', no maker site found.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -17571,6 +21131,28 @@
       <c r="I130" s="2" t="inlineStr">
         <is>
           <t>https://www.zeddy.com/zeddy-1250/</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>Broken</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr"/>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>No maker site found</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr"/>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>zeddy.com no longer resolves; only news coverage of the 1250 found.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit corrections: rule 4.10 tightened, eleven link rows recoded, counts and wording in found_along_the_way.md made exact.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -759,7 +759,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Link (2021) is the link the Stygar team printed in their spreadsheet. On the date in Checked, each was opened again. Works or Moved: it still opens a page that names the product. Wrong page: it opens a page that does not, such as a dealer's page, a parked domain or an unrelated site. Broken: an error or no answer. Link today is the maker's current page for the product where one was found, otherwise the nearest live maker page, as the next column says. 2_research/product_links.csv holds the same, with the rule in 2_research/rules.md, rule 4.10. The links change no grade, count or score.</t>
+          <t>Link (2021) is the link the Stygar team printed in their spreadsheet. On the date in Checked, each was opened again. Works or Moved: it still opens, directly or after being sent on to a new address, a maker's page that names this exact product. Wrong page: it opens a page that does not, such as a page for the product family, a dealer's page, a domain held for sale or an unrelated site. Broken: an error or no answer. Link today is the maker's current page for the product where one was found, otherwise the nearest live maker page, as the next column says. 2_research/product_links.csv holds the same, with the rule in 2_research/rules.md, rule 4.10. The links change no grade, count or score.</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>The sensor evidence is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products, studies and links are as those papers found them; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
+          <t>The sensor evidence is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products and studies are as those papers found them, and so are the links in the column Link (2021); what those links open today is in the Product list sheet; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
         </is>
       </c>
     </row>
@@ -12757,7 +12757,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -12828,10 +12828,14 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>AfiAct III is a smart sensor used to identify</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -12839,7 +12843,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Redirects to Afimilk cow monitoring page, which lists AfiAct III only; page does not say AfiAct III replaces AfiAct II.</t>
+          <t>The page names AfiAct III and does not say it replaces AfiAct II.</t>
         </is>
       </c>
     </row>
@@ -12900,7 +12904,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>AfiCollar is a smart sensor that collects data on each cow's eating</t>
+          <t>AfiCollar is a smart sensor that collects data on each cow’s</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -13155,7 +13159,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
@@ -13352,10 +13356,14 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>the world-renowned Heatime® system for heat detection</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -13363,7 +13371,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Old link redirects via allflex.global/product/heatimepro/ to msd.sensehub.com, which does not name Heatime; MSD page only says Heatime later evolved into SenseTime and then SenseHub, without naming Heatime HR or Hi-Tag.</t>
+          <t>The page names the Heatime system but not the HR LD or the Hi-Tag.</t>
         </is>
       </c>
     </row>
@@ -13809,7 +13817,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
@@ -13872,7 +13880,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
@@ -14073,7 +14081,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
@@ -14266,7 +14274,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>A related page (see note)</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -14281,7 +14289,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ida.io now shows a redirect notice to Datamars Livestock, which bought Ida for Farmers in 2023; no Ida product page found on the Datamars Livestock site.</t>
+          <t>ida.io shows only a notice naming Datamars Livestock and ida before sending visitors to Datamars Livestock; no Ida product page was found there.</t>
         </is>
       </c>
     </row>
@@ -14877,7 +14885,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr"/>
@@ -15740,7 +15748,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr"/>
@@ -15807,7 +15815,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr"/>
@@ -15935,7 +15943,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Works</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -16075,7 +16083,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr"/>
@@ -16128,7 +16136,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Works</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -16205,7 +16213,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr"/>
@@ -16335,7 +16343,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>A related page (see note)</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -16350,7 +16358,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>Livestock page does not name Tellus; home page names Tellus 2 only in its customer login list; no product page found</t>
+          <t>The home page names Tellus 2 only in its list of customer logins; no product page was found.</t>
         </is>
       </c>
     </row>
@@ -16536,7 +16544,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr"/>
@@ -16662,7 +16670,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr"/>
@@ -16725,7 +16733,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr"/>
@@ -16855,7 +16863,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr"/>
@@ -16918,7 +16926,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr"/>
@@ -17046,7 +17054,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Moved, still works</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -17257,7 +17265,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr"/>
@@ -17513,7 +17521,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr"/>
@@ -17889,24 +17897,20 @@
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>Works</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>https://store.calfstar.com/products/automatic-calf-feeders</t>
+          <t>https://www.holm-laue.de/</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>A related page (see note)</t>
-        </is>
-      </c>
-      <c r="M80" s="2" t="inlineStr">
-        <is>
-          <t>The Calf Star Double Jug is connected to the CalfExpert</t>
-        </is>
-      </c>
+          <t>Maker's site, product not named on it</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr"/>
       <c r="N80" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -17914,7 +17918,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>This is the store of Calf Star, a seller of Holm &amp; Laue CalfExpert feeders, not the maker's own site.</t>
+          <t>The 2021 link opens the shop of Calf Star, a seller of Holm &amp; Laue CalfExpert feeders, whose page describes the Calf Star Double Jug; the Holm &amp; Laue home page does not name Calf Star.</t>
         </is>
       </c>
     </row>
@@ -18301,7 +18305,7 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr"/>
@@ -18354,7 +18358,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>Works</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -18369,7 +18373,7 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>The Lely Calm helps dairy farmers achieve optimal growth.</t>
+          <t>The Lely Calm helps dairy farmers achieve optimal growth and development from calf to cow</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
@@ -18436,7 +18440,7 @@
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>The Lely Calm helps dairy farmers achieve optimal growth.</t>
+          <t>The Lely Calm helps dairy farmers achieve optimal growth and development from calf to cow</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
@@ -18569,10 +18573,14 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
-        </is>
-      </c>
-      <c r="M90" s="2" t="inlineStr"/>
+          <t>The product's page</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>8x Astronaut A4</t>
+        </is>
+      </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -18580,7 +18588,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>Astronaut page now sells the Astronaut A5 Next; A4 appears only in a customer quote and the page does not say the A5 replaces it.</t>
+          <t>Named only in a customer reference; the page sells the Astronaut A5 Next and does not say it replaces the A4.</t>
         </is>
       </c>
     </row>
@@ -18703,7 +18711,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr"/>
@@ -18766,7 +18774,7 @@
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr"/>
@@ -18829,7 +18837,7 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr"/>
@@ -18955,12 +18963,12 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>A related page (see note)</t>
+          <t>The product's page</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>LiteTrack Iridium 130 - 150</t>
+          <t>LiteTrack 140</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
@@ -18970,7 +18978,7 @@
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>The page lists LiteTrack Iridium and other Lotek collars; LiteTrack 330 or 420 is not named.</t>
+          <t>The page lists LiteTrack 140 and LiteTrack 330 to 800 among Lotek's collars.</t>
         </is>
       </c>
     </row>
@@ -19081,7 +19089,7 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr"/>
@@ -19144,10 +19152,14 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
-        </is>
-      </c>
-      <c r="M99" s="2" t="inlineStr"/>
+          <t>A related page (see note)</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>FarmLife Livestock</t>
+        </is>
+      </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -19155,7 +19167,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>FarmLife Livestock page describes a connected collar but never names Bouquet or says it replaces it.</t>
+          <t>The page names FarmLife Livestock, a connected collar, but not Bouquet.</t>
         </is>
       </c>
     </row>
@@ -19987,7 +19999,7 @@
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M112" s="2" t="inlineStr"/>
@@ -20117,7 +20129,7 @@
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M114" s="2" t="inlineStr"/>
@@ -20170,7 +20182,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>Broken</t>
+          <t>Wrong page</t>
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr">
@@ -20180,7 +20192,7 @@
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M115" s="2" t="inlineStr"/>
@@ -20191,7 +20203,7 @@
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>2021 link is an AgriExpo marketplace page that blocks scripts (403); FDS3 not found on the maker site, which redirects to BouMatic.</t>
+          <t>The 2021 link is a live page on AgriExpo, a trade marketplace (it refuses scripts and loads in a web browser); FDS3 is not named on the maker's site, which now sends visitors to BouMatic.</t>
         </is>
       </c>
     </row>
@@ -20243,7 +20255,7 @@
       </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M116" s="2" t="inlineStr"/>
@@ -20321,7 +20333,7 @@
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>smartbow.com is a parked domain for sale; Zoetis bought Smartbow but its precision livestock page does not name it.</t>
+          <t>smartbow.com is a domain for sale; no maker page naming Smartbow was found.</t>
         </is>
       </c>
     </row>
@@ -20440,7 +20452,7 @@
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M119" s="2" t="inlineStr"/>
@@ -20507,7 +20519,7 @@
       </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
-          <t>Maker's home page only</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M120" s="2" t="inlineStr"/>
@@ -20696,7 +20708,7 @@
       </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
-          <t>Maker's site, product not on it</t>
+          <t>Maker's site, product not named on it</t>
         </is>
       </c>
       <c r="M123" s="2" t="inlineStr"/>
@@ -20957,7 +20969,7 @@
       </c>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>Enter Workswell's SMARTIS thermographic system</t>
+          <t>Enter Workswell’s SMARTIS thermographic system</t>
         </is>
       </c>
       <c r="N127" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rule 4.10 covers maker addresses that now send visitors elsewhere and redirect notices; six link rows and several notes made exact.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -13107,7 +13107,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>agersens.com redirects through cu-bx.com and fronteer.us to an unrelated restaurant site; Gallagher (acquired Agersens 2021) sells eShepherd on its own site, though the page does not mention Agersens.</t>
+          <t>agersens.com sends visitors through cu-bx.com and fronteer.us to an unrelated restaurant site; Gallagher sells eShepherd under its own name on its own site, though the page does not mention Agersens.</t>
         </is>
       </c>
     </row>
@@ -13564,7 +13564,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>App delisted from Google Play; Bayer Animal Health went to Elanco in 2020 and no current Cowdition page found; bayer.com blocks fetching (403).</t>
+          <t>No current Cowdition page was found; the app is no longer listed on Google Play, and bayer.com refuses scripted requests (403).</t>
         </is>
       </c>
     </row>
@@ -14151,7 +14151,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Domain is a parked page that redirects to /lander; company later renamed Herd-itt and reported as ceased operating; no maker site found.</t>
+          <t>The domain is a parked page; no maker site was found.</t>
         </is>
       </c>
     </row>
@@ -14289,7 +14289,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ida.io shows only a notice naming Datamars Livestock and ida before sending visitors to Datamars Livestock; no Ida product page was found there.</t>
+          <t>The page is only a notice, which names ida as joining forces with Datamars Livestock, before it sends visitors on to Datamars Livestock; it does not describe the product, and no Ida product page was found there.</t>
         </is>
       </c>
     </row>
@@ -15562,7 +15562,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>eiodiagnostics.com now redirects to an unrelated pizza site; press says the product became UdderHealth but no maker page confirms it</t>
+          <t>eiodiagnostics.com now sends visitors to an unrelated gambling page, and the 2021 link itself gives an error; no maker page for FirstLook was found.</t>
         </is>
       </c>
     </row>
@@ -17069,7 +17069,7 @@
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+          <t>GEA DairyFeed F4110 / F4120</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -17079,7 +17079,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>J C400 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+          <t>The page names J C400 only in an image description, "Calf Feeder DairyFeed J C400 , V600 and V640"; its visible text is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
         </is>
       </c>
     </row>
@@ -17136,7 +17136,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+          <t>GEA DairyFeed F4110 / F4120</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -17146,7 +17146,7 @@
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>V600 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+          <t>The page names V600 only in an image description, "Calf Feeder DairyFeed J C400 , V600 and V640"; its visible text is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
         </is>
       </c>
     </row>
@@ -17203,7 +17203,7 @@
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>Calf Feeder DairyFeed J C400 , V600 and V640</t>
+          <t>GEA DairyFeed F4110 / F4120</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
@@ -17213,7 +17213,7 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>V640 appears only in an image description; the page is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
+          <t>The page names V640 only in an image description, "Calf Feeder DairyFeed J C400 , V600 and V640"; its visible text is for DairyFeed F4110 and F4120 and does not say they replace it.</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>licautomation.com refuses connections; LIC sold LIC Automation to MSD Animal Health in 2021 and no maker page for Saber Milk was found.</t>
+          <t>licautomation.com refuses connections; no maker page for Saber Milk was found.</t>
         </is>
       </c>
     </row>
@@ -18785,7 +18785,7 @@
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>LIC page is 404; LIC home shows only a ProTrack login link; automation business sold to MSD Animal Health in 2021; no maker page found.</t>
+          <t>LIC page is 404; LIC home shows only a ProTrack login link; no maker page found.</t>
         </is>
       </c>
     </row>
@@ -18848,7 +18848,7 @@
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>LIC page is 404; LIC home shows only a ProTrack login link; automation business sold to MSD Animal Health in 2021; no maker page found.</t>
+          <t>LIC page is 404; LIC home shows only a ProTrack login link; no maker page found.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Step 2: research_only split into research_demonstrated (2) and theoretically_measurable (22), rules 0.6; company facts with sources in found_along_the_way.md section 10.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Checked for 58 of 58 indicators so far. 7 tested; 1 claimed; 24 research only; 19 nothing found; 7 unclear</t>
+          <t>Checked for 58 of 58 indicators so far. 7 tested; 1 claimed; 2 shown in research; 22 proposed only; 19 nothing found; 7 unclear</t>
         </is>
       </c>
     </row>
@@ -646,156 +646,160 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Sensor: research_only</t>
+          <t>Sensor: research_demonstrated</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Sensor: none</t>
+          <t>Sensor: theoretically_measurable</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Sensor: unsure</t>
+          <t>Sensor: none</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Device needed</t>
+          <t>Sensor: unsure</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>The cheapest kind of equipment that measures it. Classes, in the order the score ranks them: nothing extra (3 points), one device per farm (2), one device per animal (1), a sample or a scoring by a person (0), or no technology named in the sources (0), or unclear when the rules do not settle it (0). 'Nothing extra' can appear where no sensor exists, because the value is already taken from milk or farm records (2_research/rules.md, rule 4.4).</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Vendors naming it</t>
+          <t>Device needed</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>How many of the 129 products in the Stygar list contain one of the indicator's search words in their own description. A count of claims, not of proof. 'Tested products' is a separate column: a product can be tested without its description naming the measure, and the reverse.</t>
+          <t>The cheapest kind of equipment that measures it. Classes, in the order the score ranks them: nothing extra (3 points), one device per farm (2), one device per animal (1), a sample or a scoring by a person (0), or no technology named in the sources (0), or unclear when the rules do not settle it (0). 'Nothing extra' can appear where no sensor exists, because the value is already taken from milk or farm records (2_research/rules.md, rule 4.4).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>EFSA's ratings</t>
+          <t>Vendors naming it</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>For indicators that come from EFSA, how EFSA's own assessment table rates the measure: sensitivity (does it catch the animals that have the problem), specificity (does it avoid flagging animals that do not) and feasibility on farm. High, Medium and Low are EFSA's own words; Mixed means EFSA gives two levels and Not stated means EFSA gives none. 2_research/indicators.csv quotes the passage. Blank for Welfare Quality only indicators, which EFSA does not rate.</t>
+          <t>How many of the 129 products in the Stygar list contain one of the indicator's search words in their own description. A count of claims, not of proof. 'Tested products' is a separate column: a product can be tested without its description naming the measure, and the reverse.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Schemes: 'Unclear'</t>
+          <t>EFSA's ratings</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>A scheme has a requirement that may name the indicator, but the written rules do not settle whether it does. It is not counted as required. Kevin's lists show Unclear for that indicator only where the answer depends on it, for example a list 1 row graded Tested or Claimed that no other scheme requires (see 2_research/rules.md, section 6, and 2_research/open_questions.md).</t>
+          <t>For indicators that come from EFSA, how EFSA's own assessment table rates the measure: sensitivity (does it catch the animals that have the problem), specificity (does it avoid flagging animals that do not) and feasibility on farm. High, Medium and Low are EFSA's own words; Mixed means EFSA gives two levels and Not stated means EFSA gives none. 2_research/indicators.csv quotes the passage. Blank for Welfare Quality only indicators, which EFSA does not rate.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Sensors x products: 'validated'</t>
+          <t>Schemes: 'Unclear'</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>A published study tested this product for this measure (Stygar 2021, Tables 1 and 2).</t>
+          <t>A scheme has a requirement that may name the indicator, but the written rules do not settle whether it does. It is not counted as required. Kevin's lists show Unclear for that indicator only where the answer depends on it, for example a list 1 row graded Tested or Claimed that no other scheme requires (see 2_research/rules.md, section 6, and 2_research/open_questions.md).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Sensors x products: 'named'</t>
+          <t>Sensors x products: 'validated'</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The vendor's own description contains one of the indicator's search words. Not tested.</t>
+          <t>A published study tested this product for this measure (Stygar 2021, Tables 1 and 2).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Product list: links</t>
+          <t>Sensors x products: 'named'</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Link (2021) is the link the Stygar team printed in their spreadsheet. On the date in Checked, each was opened again. Works or Moved: it still opens, directly or after being sent on to a new address, a maker's page that names this exact product. Wrong page: it opens a page that does not, such as a page for the product family, a dealer's page, a domain held for sale or an unrelated site. Broken: an error or no answer. Link today is the maker's current page for the product where one was found, otherwise the nearest live maker page, as the next column says. 2_research/product_links.csv holds the same, with the rule in 2_research/rules.md, rule 4.10. The links change no grade, count or score.</t>
+          <t>The vendor's own description contains one of the indicator's search words. Not tested.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>Product list: links</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Link (2021) is the link the Stygar team printed in their spreadsheet. On the date in Checked, each was opened again. Works or Moved: it still opens, directly or after being sent on to a new address, a maker's page that names this exact product. Wrong page: it opens a page that does not, such as a page for the product family, a dealer's page, a domain held for sale or an unrelated site. Broken: an error or no answer. Link today is the maker's current page for the product where one was found, otherwise the nearest live maker page, as the next column says. 2_research/product_links.csv holds the same, with the rule in 2_research/rules.md, rule 4.10. The links change no grade, count or score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
           <t>Ease of adoption score</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>0 to 15, five factors of 0 to 3 added together (2_research/rules.md, section 5). Ties are sorted by indicator id. A sort order, not a welfare judgement. Score parts are shown in the order: sensor + device + vendors + FARM + schemes.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr"/>
-      <c r="B29" s="2" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>WHAT THIS DOES NOT SHOW</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>The sensor evidence is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products and studies are as those papers found them, and so are the links in the column Link (2021); what those links open today is in the Product list sheet; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr"/>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>'Tested' means a published study tested the product for the measure, as Stygar 2021 coded it; many of those tests fell below Stygar's high performance bar, which the column 'What was tested, and how well' shows.</t>
         </is>
       </c>
     </row>
@@ -803,7 +807,7 @@
       <c r="A32" s="3" t="inlineStr"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>The certification schemes have been read for every indicator.</t>
+          <t>'Tested' means a published study tested the product for the measure, as Stygar 2021 coded it; many of those tests fell below Stygar's high performance bar, which the column 'What was tested, and how well' shows.</t>
         </is>
       </c>
     </row>
@@ -811,45 +815,53 @@
       <c r="A33" s="3" t="inlineStr"/>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no review by a welfare scientist is recorded in the repository.</t>
+          <t>The certification schemes have been read for every indicator.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>The score is a rule of thumb used as a sort order. It is not a welfare judgement, and no review by a welfare scientist is recorded in the repository.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO CHECK ANY CELL</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names and sensor types, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
-        </is>
-      </c>
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Who checked it</t>
+          <t>HOW TO CHECK ANY CELL</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Before each push, an AI auditing agent checks the changes against the source pages; 2_research/audit_log.md lists the versions that passed. The author plans to spot check ten rows after each push; each spot check is logged in 2_research/decision_log.md with its date and the rows read.</t>
+          <t>Every checked row of the Answer sheet has a 'Where to check' column naming the documents, with pages where a passage is cited. The documents are listed in the Sources sheet and in 1_sources/. The rules that turn what a page says into a label are in 2_research/rules.md, and section 2 of that file explains the codes and the abbreviations used in the cells, other than product names and sensor types, which are given as the Stygar list writes them. 2_research/README.md explains the three kinds of check: read the page, apply the rule, or count again.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t>Who checked it</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Before each push, an AI auditing agent checks the changes against the source pages; 2_research/audit_log.md lists the versions that passed. The author plans to spot check ten rows after each push; each spot check is logged in 2_research/decision_log.md with its date and the rows read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>Built from</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>The tables in 2_research/ by 3_code/build_output.py. Do not edit this file by hand; change the tables and run the script.</t>
         </is>
@@ -1291,7 +1303,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -1347,7 +1359,7 @@
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial.</t>
+          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1409,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -1453,7 +1465,7 @@
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>As I004.</t>
+          <t>As I004. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I004: Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1821,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1865,7 +1877,7 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class.</t>
+          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water point measure. A study of the substitute does not demonstrate the indicator, even in cattle.</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1911,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -1955,7 +1967,7 @@
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded.</t>
+          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina only propose turbidity sensors for water cleanliness and cite no study that used them at a water point.</t>
         </is>
       </c>
     </row>
@@ -2515,7 +2527,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
@@ -2719,7 +2731,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -2931,7 +2943,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -3021,7 +3033,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
@@ -3077,7 +3089,7 @@
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says.</t>
+          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no automatic system for cow dirtiness and only propose image analysis adapted from technologies shown on carcasses, which the reference titles give as chicken and poultry carcasses (Windham et al. 2003; Seo et al. 2019). Stygar page 10 also find no available technology for the cleanliness of animals.</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3123,7 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr"/>
@@ -3167,7 +3179,7 @@
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says.</t>
+          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I036: no automatic system for cow dirtiness was found, and the technologies proposed were shown on chicken and poultry carcasses, not live cattle.</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3213,7 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
@@ -3291,7 +3303,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr"/>
@@ -3381,7 +3393,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
@@ -3437,7 +3449,7 @@
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class.</t>
+          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I030: the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water flow at the point.</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3483,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr"/>
@@ -3527,7 +3539,7 @@
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class.</t>
+          <t>Same reading as I030: the substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the measure as defined is the water point, not the intake. Class from the technology proposed, a flowmeter with RFID at the trough, farm_fixed. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I030: the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the functioning of water points.</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3573,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
@@ -3617,7 +3629,7 @@
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says.</t>
+          <t>The proposed technology is a camera, farm_fixed; nothing commercial. The keyword clean alone matches one aim, Cainthus Alus Nutrition, whose aim reads monitors events like feed deliveries, push-ups and clean-outs, feed events, so it is not used. The technology Maroto Molina cite comes from carcass inspection, not live cows, as their text says. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I036: no automatic system for cow dirtiness was found, and the technologies proposed were shown on chicken and poultry carcasses, not live cattle.</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3663,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
@@ -3707,7 +3719,7 @@
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>As on I030, I032 and I033, the substitute measure has commercial products, GEA CowView among them, which the grade does not credit because the measure is the housing system, not where the cow is. Class: among the technologies proposed the cheapest class with a commercial product is the collar (CowView, appendix aim animal location), animal_mounted; the camera alternative has no appendix product for this purpose.</t>
+          <t>As on I030, I032 and I033, the substitute measure has commercial products, GEA CowView among them, which the grade does not credit because the measure is the housing system, not where the cow is. Class: among the technologies proposed the cheapest class with a commercial product is the collar (CowView, appendix aim animal location), animal_mounted; the camera alternative has no appendix product for this purpose. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina offer only a substitute measure, indoor location monitoring, in place of the presence of tethering. The location studies they cite (Tøgersen et al. 2010, Pastell et al. 2018, Dao et al. 2015) measured where cows are, not the housing system.</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3753,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
@@ -3831,7 +3843,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
@@ -3887,7 +3899,7 @@
       </c>
       <c r="X30" s="2" t="inlineStr">
         <is>
-          <t>Calving prediction is a substitute measure, so research_only under rules.md rule 4.2, although two appendix products state calving monitoring; the grade does not credit them, as on I030 and I040, and the search words name dystocia itself, so the two calving aims are not counted. Device needed routine_data under the records rule (rules.md rule 4.4): the Welfare Quality definition takes the value from herd records, and the routine_data class list names calving records. The calving products, both worn, animal_mounted, are the added device alternative for the substitute.</t>
+          <t>Calving prediction is a substitute measure, so research_only under rules.md rule 4.2, although two appendix products state calving monitoring; the grade does not credit them, as on I030 and I040, and the search words name dystocia itself, so the two calving aims are not counted. Device needed routine_data under the records rule (rules.md rule 4.4): the Welfare Quality definition takes the value from herd records, and the routine_data class list names calving records. The calving products, both worn, animal_mounted, are the added device alternative for the substitute. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute, calving prediction (Borchers et al. 2017), which by its title was done in dairy cattle but predicts calving rather than recording calvings that needed major assistance. Maroto Molina also say dystocia is a measure based on farmer records.</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4051,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
@@ -4090,12 +4102,12 @@
       </c>
       <c r="W32" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan of the 129 appendix aims: 0 hits for social, aggress, agonist or interaction. Maroto Molina page 3: social behaviour has not been a priority topic for PLF researchers; top view cameras in the waiting area of automated milking systems with machine learning detect head pressing and body pushing (Guzhva et al. 2016); proximity loggers and location solutions have been used to characterise social network structure.</t>
+          <t>Keyword scan of the 129 appendix aims: 0 hits for social, aggress, agonist or interaction. Maroto Molina page 3: social behaviour has not been a priority topic for PLF researchers; top view cameras in the waiting area of automated milking systems with machine learning detect head pressing and body pushing (Guzhva et al. 2016); proximity loggers and location solutions have been used to characterise social network structure. stygar_2021.pdf page 11 (social competition from feeding and drinking station data, studies 70, 78 and 79) and page 15 (reference 78, Foris et al. 2019).</t>
         </is>
       </c>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>Nothing commercial. Of the technologies proposed the fixed camera is the cheaper class, farm_fixed; proximity loggers are animal mounted. EFSA Table 32 page 53 rates feasibility low.</t>
+          <t>Nothing commercial. Of the technologies proposed the fixed camera is the cheaper class, farm_fixed; proximity loggers are animal mounted. EFSA Table 32 page 53 rates feasibility low. Rule 4.2 split (15 October 2026): research_demonstrated, because Stygar et al. (page 11) cite study 78 for monitoring social competition from feeding and drinking station data, and its title in their reference list (page 15) says it detected feeding and drinking related agonistic behavior in dairy cows; no product's stated aim names agonistic behaviour. Maroto Molina page 3 also cite Guzhva et al. 2016, top view cameras detecting head pressing and body pushing in the waiting area of automatic milking stations.</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4259,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
@@ -4303,7 +4315,7 @@
       </c>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, farm_fixed. Nothing commercial. EFSA Table 33 defines the measure citing Welfare Quality.</t>
+          <t>The proposed technology is a camera, farm_fixed. Nothing commercial. EFSA Table 33 defines the measure citing Welfare Quality. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system that measures the time needed to lie down and only propose camera systems. The studies they cite for those (Porto et al. 2013, Cangar et al. 2008) were in cows but, by their titles, detected lying behaviour and posture, not this measure.</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4361,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr"/>
@@ -4439,7 +4451,7 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
@@ -4495,7 +4507,7 @@
       </c>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>Same passage and same reading as I014: the proposed technology is a camera, farm_fixed; nothing commercial.</t>
+          <t>Same passage and same reading as I014: the proposed technology is a camera, farm_fixed; nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system that measures collisions with equipment and only propose camera systems. The studies they cite for those (Porto et al. 2013, Cangar et al. 2008) detected lying behaviour and posture, not collisions.</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4541,7 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
@@ -4585,7 +4597,7 @@
       </c>
       <c r="X37" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera detecting cows at cubicles, farm_fixed; nothing commercial. Smartbow's appendix row names indoor location in its sensor type and lying behaviour in its aim, neither of which is position relative to the lying area, so it is not cited.</t>
+          <t>The proposed technology is a camera detecting cows at cubicles, farm_fixed; nothing commercial. Smartbow's appendix row names indoor location in its sensor type and lying behaviour in its aim, neither of which is position relative to the lying area, so it is not cited. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for cow positioning in the resting area and only propose cameras that detect cows at cubicles. The study they cite (Porto et al. 2013) detected lying behaviour of dairy cows by its title, not lying outside the lying area.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4631,7 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr"/>
@@ -4675,7 +4687,7 @@
       </c>
       <c r="X38" s="2" t="inlineStr">
         <is>
-          <t>As on I040, the substitute measure has commercial products, which the grade does not credit, because the Welfare Quality measure is whether the farm gives access to an outdoor loafing area or pasture, not where the cow is. Device needed: among the technologies proposed, the only one with appendix products whose aims state the substitute measurement is GPS positioning, and all seven are worn (collars and an ear tag), so animal_mounted; satellite imagery is not a device on the farm and has no appendix row. Four more aims name location or tracking: Boumatic Real Time + RL (appendix row 17, location indoor), CowManager (row 26, location monitor) and GEA CowView (row 64, animal location), all worn, and Taggle (row 123), an RFID radiolocation system whose aim, Tracking system, does not state location; Smartbow (row 117) names indoor location only in its sensor type. None of them changes the class. The records rule of rule 4.4 does not apply, because the definition takes the value from the manager's answers and names no records. IceTag's aim names "pastur activity" with the number of steps, a step count at pasture, not access to it; the search word pasture does not match that spelling, and a reader who searched pastur would count 1. Stygar Table 2 page 7 validates grazing time (MooMonitor+ 29, RumiWatch 29 and 38, research farm, high performance column), a feeding behaviour, not the provision of access, so under rule 4.2 it is not the same measure. I053, the Welfare Quality access to pasture measure under appropriate behaviour, is a separate row.</t>
+          <t>As on I040, the substitute measure has commercial products, which the grade does not credit, because the Welfare Quality measure is whether the farm gives access to an outdoor loafing area or pasture, not where the cow is. Device needed: among the technologies proposed, the only one with appendix products whose aims state the substitute measurement is GPS positioning, and all seven are worn (collars and an ear tag), so animal_mounted; satellite imagery is not a device on the farm and has no appendix row. Four more aims name location or tracking: Boumatic Real Time + RL (appendix row 17, location indoor), CowManager (row 26, location monitor) and GEA CowView (row 64, animal location), all worn, and Taggle (row 123), an RFID radiolocation system whose aim, Tracking system, does not state location; Smartbow (row 117) names indoor location only in its sensor type. None of them changes the class. The records rule of rule 4.4 does not apply, because the definition takes the value from the manager's answers and names no records. IceTag's aim names "pastur activity" with the number of steps, a step count at pasture, not access to it; the search word pasture does not match that spelling, and a reader who searched pastur would count 1. Stygar Table 2 page 7 validates grazing time (MooMonitor+ 29, RumiWatch 29 and 38, research farm, high performance column), a feeding behaviour, not the provision of access, so under rule 4.2 it is not the same measure. I053, the Welfare Quality access to pasture measure under appropriate behaviour, is a separate row. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina say access to an outdoor loafing area or pasture could be substituted by outdoor location monitoring, for which GPS would be the preferred option (Turner et al. 2000). Turner's title names cattle and pasture use but does not say the study recorded the days per year or hours per day on pasture that the protocol asks the manager for, so it is a study of a substitute measure and does not demonstrate the indicator.</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4721,7 @@
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
@@ -4765,7 +4777,7 @@
       </c>
       <c r="X39" s="2" t="inlineStr">
         <is>
-          <t>No appendix aim names hampered respiration, and Maroto Molina propose two technologies, so research_only. HerdInsight's health disorder validation (30), whose footnote names pneumonia, is a health disorder trait, not this measure, the reading applied on I006, so it is not credited. Device needed: nothing commercial for the measure, so the cheapest class among the technologies proposed (rules.md rule 4.4). Image analysis, as Maroto Molina name it, is a camera technology, farm_fixed, and that reading sets the class. The integration of body temperature and intake monitoring is not used for the class, because its own class is unsure (see I043). The class follows Maroto Molina's words, as the cleanliness rows follow their carcass passage; the study they cite for the pigs is, by its title, a laboratory biosensor that detects a virus, not a camera on the animals. If that technology were read as a sample analysis, the class would rest on the unsettled integration of I043; the row follows the image analysis reading only. Sound analysis for coughs is not listed for this measure (the notes column of indicators.csv).</t>
+          <t>No appendix aim names hampered respiration, and Maroto Molina propose two technologies, so research_only. HerdInsight's health disorder validation (30), whose footnote names pneumonia, is a health disorder trait, not this measure, the reading applied on I006, so it is not credited. Device needed: nothing commercial for the measure, so the cheapest class among the technologies proposed (rules.md rule 4.4). Image analysis, as Maroto Molina name it, is a camera technology, farm_fixed, and that reading sets the class. The integration of body temperature and intake monitoring is not used for the class, because its own class is unsure (see I043). The class follows Maroto Molina's words, as the cleanliness rows follow their carcass passage; the study they cite for the pigs is, by its title, a laboratory biosensor that detects a virus, not a camera on the animals. If that technology were read as a sample analysis, the class would rest on the unsettled integration of I043; the row follows the image analysis reading only. Sound analysis for coughs is not listed for this measure (the notes column of indicators.csv). Rule 4.2 split (15 October 2026): theoretically_measurable, because the image analysis Maroto Molina cite for respiratory problems was tested in pigs (Chen et al. 2013, whose title names a porcine virus detected by a biosensor), and the cough sound study in calves (Vandermeulen et al. 2016) measured coughing, a different measure. The body temperature route is only proposed.</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4811,7 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -4855,7 +4867,7 @@
       </c>
       <c r="X40" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is image based, a camera, farm_fixed; nothing commercial. Maroto Molina cite no study for it.</t>
+          <t>The proposed technology is image based, a camera, farm_fixed; nothing commercial. Maroto Molina cite no study for it. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina identified no automatic system for diarrhoea, only propose image based solutions and cite no study.</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4901,7 @@
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
@@ -4979,7 +4991,7 @@
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
@@ -5035,7 +5047,7 @@
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>Nothing commercial, and the sources propose research level technologies, so research_only. Device needed: the cheapest class among the technologies proposed (rules.md rule 4.4): video imaging, infrared thermography and 3D cameras are farm_fixed; the Bluetooth or radio location network uses tags worn by the cows, animal_mounted. So farm_fixed. The four appendix aims that name location (I040) state location, not avoidance distance, so they do not set the class.</t>
+          <t>Nothing commercial, and the sources propose research level technologies, so research_only. Device needed: the cheapest class among the technologies proposed (rules.md rule 4.4): video imaging, infrared thermography and 3D cameras are farm_fixed; the Bluetooth or radio location network uses tags worn by the cows, animal_mounted. So farm_fixed. The four appendix aims that name location (I040) state location, not avoidance distance, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the only study Maroto Molina cite as assessing avoidance distance was in broiler flocks (Johansson et al. 2015), and they say no individual level PLF solution is available. The cattle study they cite (Stewart et al. 2008) measured fear related responses to handling, a substitute.</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5093,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
@@ -5137,7 +5149,7 @@
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>The technologies named are proximity loggers and location solutions, both worn by the animal, animal_mounted. Nothing commercial for grooming: no appendix aim names grooming, social behaviour or proximity. Location is named in four appendix aims (GEA CowView, CowManager, Boumatic Real Time + RL, Sensolus RDS Futureline MAX), and positioning in six more (Cattlewatch, Pellegro Livestock, Tellus Livestock, Ceres Tag, Digitanimal, Lotek). All ten are worn by the animal, as collars or ear tags.</t>
+          <t>The technologies named are proximity loggers and location solutions, both worn by the animal, animal_mounted. Nothing commercial for grooming: no appendix aim names grooming, social behaviour or proximity. Location is named in four appendix aims (GEA CowView, CowManager, Boumatic Real Time + RL, Sensolus RDS Futureline MAX), and positioning in six more (Cattlewatch, Pellegro Livestock, Tellus Livestock, Ceres Tag, Digitanimal, Lotek). All ten are worn by the animal, as collars or ear tags. Rule 4.2 split (15 October 2026): research_demonstrated, because Maroto Molina page 3 say proximity loggers and location solutions detected grooming in dairy herds, citing Boyland et al. 2016, and no product's stated aim names grooming. The reference title names dairy cows but not grooming, so the grade rests on Maroto Molina's own words.</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5183,7 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
@@ -5227,7 +5239,7 @@
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>Nothing commercial, and Maroto Molina name research level technology, so research_only. The technologies named, image and video analysis and sound analysis, are a camera and a microphone, both farm_fixed. Four aims name welfare or wellbeing in general (Ceres Tag and Track a))) Cow, health and welfare monitoring; AfiAct II, wellbing; SenseHub Dairy, wellbeing status); none names the assessment, so they are not counted.</t>
+          <t>Nothing commercial, and Maroto Molina name research level technology, so research_only. The technologies named, image and video analysis and sound analysis, are a camera and a microphone, both farm_fixed. Four aims name welfare or wellbeing in general (Ceres Tag and Track a))) Cow, health and welfare monitoring; AfiAct II, wellbing; SenseHub Dairy, wellbeing status); none names the assessment, so they are not counted. Rule 4.2 split (15 October 2026): theoretically_measurable, because the cattle studies the sources cite used ear posture and eye white (Battini et al. 2019, Maroto Molina page 4) or ear postures and nasal temperature (Stygar references 81 and 82, page 11), substitute measures in place of Qualitative Behaviour Assessment; Maroto Molina only propose image and video analysis to monitor these, and sound analysis for emotional state.</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5363,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -5453,7 +5465,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr"/>
@@ -5555,7 +5567,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr"/>
@@ -5657,7 +5669,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
@@ -5759,7 +5771,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
@@ -5861,7 +5873,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
@@ -5951,7 +5963,7 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr"/>
@@ -6007,7 +6019,7 @@
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>No appendix aim names nasal discharge, and Maroto Molina propose a technology, so research_only. The maroto_molina_technology column of indicators.csv attaches the integration of body temperature sensors with feed and water intake monitoring to this row, and the image analysis tested in pigs to I045 only. HerdInsight's health disorder validation (30) is not the same measure as nasal discharge, the reading already applied on I006, so it is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
+          <t>No appendix aim names nasal discharge, and Maroto Molina propose a technology, so research_only. The maroto_molina_technology column of indicators.csv attaches the integration of body temperature sensors with feed and water intake monitoring to this row, and the image analysis tested in pigs to I045 only. HerdInsight's health disorder validation (30) is not the same measure as nasal discharge, the reading already applied on I006, so it is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md. Rule 4.2 split (15 October 2026): theoretically_measurable, because in their passage on the respiratory signs Maroto Molina cite a cough sound study in calves (Vandermeulen et al. 2016), which measured coughing, and image analysis tested in pigs (Chen et al. 2013), and otherwise only propose integrating body temperature sensors with feed and water intake monitoring, citing no study that did so.</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6053,7 @@
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr"/>
@@ -6097,7 +6109,7 @@
       </c>
       <c r="X53" s="2" t="inlineStr">
         <is>
-          <t>Same passage and same reading as I043 (the maroto_molina_technology column of indicators.csv): no appendix aim names ocular discharge, and Maroto Molina propose the integration of body temperature sensors with intake monitoring, so research_only; HerdInsight's health disorder validation (30) is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md.</t>
+          <t>Same passage and same reading as I043 (the maroto_molina_technology column of indicators.csv): no appendix aim names ocular discharge, and Maroto Molina propose the integration of body temperature sensors with intake monitoring, so research_only; HerdInsight's health disorder validation (30) is not credited. Device needed: no appendix aim states the sign, so no technology is commercial for it, and rules.md rule 4.4 takes the cheapest class among the technologies the sources propose. The integration needs a body temperature sensor and an intake monitoring system. For body temperature the sources name reticular boluses (Maroto Molina pages 2 and 3; Stygar page 11), animal_mounted, and cameras (Stygar page 11; OPTRIS, Table 2 page 7), farm_fixed; for intake they name RFID with flowmeters at the trough (Maroto Molina page 2) and load cells with RFID (Stygar page 11), farm_fixed. So device needed is unsure, with two candidates. farm_fixed: the cheapest combination, a camera from Stygar page 11 with an intake station. animal_mounted: the only body temperature sensors Maroto Molina name are reticular boluses; all ten appendix aims naming temperature belong to worn devices (eight boluses, the Ceres Tag ear tag and the Digitanimal collar), while the thermal cameras' aims name udder health, mastitis, inflammation, fever or lameness, not temperature (the I039 reading); and I030's reasoning classes its bolus option animal_mounted. The missing rule is how a proposed combination of devices is classed, and whether a technology Stygar names only for disease detection in general counts as proposed for the row. Listed in open_questions.md. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I043: the only studies in Maroto Molina's passage on the respiratory signs measured coughing in calves (Vandermeulen et al. 2016) or were in pigs (Chen et al. 2013), and the body temperature route is only proposed.</t>
         </is>
       </c>
     </row>
@@ -6131,7 +6143,7 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
@@ -6187,7 +6199,7 @@
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>A substitute measure, so research_only under rules.md rule 4.2, whatever the products for the substitute; the grade does not credit them, as on I030 and I040. Device needed: the cheapest class with a commercial product for the substitute measurement. Herd Navigator (P012), an inline milk analyser of progesterone, LDH and BHB whose aim states heat measurement, is farm_fixed under the milk analyser line of rule 4.4; the other 30 aims naming heat detection or monitoring are collars, leg tags and ear tags, animal_mounted. The electronic nose analyses a sample and is not automatic, and the human biosensors are worn and under development; neither has an appendix row. So device needed is unsure, with two candidates. farm_fixed, if the appendix word heat is read as oestrus: Maroto Molina use heat duration and oestrus monitoring in the same passage (page 3), and Stygar calls these tools estrus detection (pages 3 and 9); Herd Navigator is then the cheapest. Or, because no aim states oestrus, no commercial product for the substitute, so rule 4.4 takes the cheapest class among the technologies proposed: animal_mounted, for the worn biosensors, although Maroto Molina's oestrus monitoring itself names no technology. The missing rule is whether an aim word that is a common synonym of the measurement states it. Listed in open_questions.md. The 31 heat aims are not counted in vendors naming it, because heat is the substitute, not the measure, the same treatment as water intake on I030.</t>
+          <t>A substitute measure, so research_only under rules.md rule 4.2, whatever the products for the substitute; the grade does not credit them, as on I030 and I040. Device needed: the cheapest class with a commercial product for the substitute measurement. Herd Navigator (P012), an inline milk analyser of progesterone, LDH and BHB whose aim states heat measurement, is farm_fixed under the milk analyser line of rule 4.4; the other 30 aims naming heat detection or monitoring are collars, leg tags and ear tags, animal_mounted. The electronic nose analyses a sample and is not automatic, and the human biosensors are worn and under development; neither has an appendix row. So device needed is unsure, with two candidates. farm_fixed, if the appendix word heat is read as oestrus: Maroto Molina use heat duration and oestrus monitoring in the same passage (page 3), and Stygar calls these tools estrus detection (pages 3 and 9); Herd Navigator is then the cheapest. Or, because no aim states oestrus, no commercial product for the substitute, so rule 4.4 takes the cheapest class among the technologies proposed: animal_mounted, for the worn biosensors, although Maroto Molina's oestrus monitoring itself names no technology. The missing rule is whether an aim word that is a common synonym of the measurement states it. Listed in open_questions.md. The 31 heat aims are not counted in vendors naming it, because heat is the substitute, not the measure, the same treatment as water intake on I030. Rule 4.2 split (15 October 2026): theoretically_measurable, because the one cattle study Maroto Molina cite (Burfeind et al. 2014) analysed vaginal discharge with an electronic nose to diagnose acute puerperal metritis, as its title says, which is a substitute measure and not the presence of vulvar discharge the protocol scores by looking at the cow. Maroto Molina also propose oestrus monitoring as sufficient to detect reproductive problems, another substitute.</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6245,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
@@ -6335,7 +6347,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr"/>
@@ -6437,7 +6449,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr"/>
@@ -6539,7 +6551,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
@@ -6641,7 +6653,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -7589,7 +7601,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7618,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7635,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7652,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7751,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8012,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8029,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
         </is>
       </c>
     </row>
@@ -8143,7 +8155,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8172,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8189,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8206,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8211,7 +8223,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8228,7 +8240,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
         </is>
       </c>
     </row>
@@ -8348,7 +8360,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8404,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8451,7 +8463,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8468,7 +8480,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8497,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8514,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8519,7 +8531,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8548,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8553,7 +8565,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8570,7 +8582,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8587,7 +8599,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8604,7 +8616,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8621,7 +8633,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8667,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8672,7 +8684,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8701,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8706,7 +8718,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8723,7 +8735,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8752,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8757,7 +8769,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8774,7 +8786,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8803,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8820,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8825,7 +8837,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8854,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8859,7 +8871,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8888,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8893,7 +8905,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Research only: no product in the Stygar list claims this measure; researchers propose a method or a substitute measure</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
     </row>
@@ -8910,7 +8922,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -8991,7 +9003,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
     </row>
@@ -12768,7 +12780,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Product not found on i4 Product Design site (design consultancy); Well Cow company listed as out of business; searched 'WellCow bolus pH temperature' and 'i4 product design Well Cow bolus'.</t>
+          <t>The product is not on the site of i4 Product Design, a design firm; searched 'WellCow bolus pH temperature'. What happened to the company is in 4_output/found_along_the_way.md, section 10.</t>
         </is>
       </c>
     </row>
@@ -16874,7 +16886,7 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>gea-cowview.com no longer resolves; no CowView page on gea.com; positioning now sold under CowScout but GEA does not say it replaces CowView</t>
+          <t>gea-cowview.com no longer answers, and no CowView page was found on gea.com. What GEA says about positioning is in 4_output/found_along_the_way.md, section 10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit corrections to the sensor evidence split and section 10 of found_along_the_way.md.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -5329,7 +5329,7 @@
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>The grade rule asks whether a product measures the indicator, and this row has no measure, so the rule does not settle it. Candidates: research_only, since Maroto Molina name technologies for a criterion the protocol leaves undefined and the weather station is not in the appendix; commercial_unvalidated, if rumen or body temperature is taken as the measure, since 10 appendix aims name it; validated_commercial is not available on that reading because KB 3/04 and Optris have no appendix row. Listed in open_questions.md; the missing rule is how to grade a criterion with no measure. Device needed per the unsure rule from the cheapest commercial candidate, where commercial means an appendix product whose aim states the candidate measurement (rules.md rule 4.4, version 0.1.4): the 10 products whose aims name temperature are boluses, ear tags and a collar, all animal_mounted, so animal_mounted. The thermal cameras Stygar page 10 name for thermal comfort do not count, because their appendix aims name udder health, mastitis, inflammation, fever or lameness; a farm_fixed reading would need one whose aim states temperature or thermal comfort. Five of those aims name fever, which is a raised body temperature; the row reads a detection aim as not stating the measure, the literal reading that is one of the two candidates on I006 and I020 (both of which still count detection aims in vendors_naming_it), and a reader may challenge it. The weather station Maroto Molina say commercial farms use is not in the appendix and does not set the class.</t>
+          <t>The grade rule asks whether a product measures the indicator, and this row has no measure, so the rule does not settle it. Candidates: research_only (now research_demonstrated or theoretically_measurable, see below), since Maroto Molina name technologies for a criterion the protocol leaves undefined and the weather station is not in the appendix; commercial_unvalidated, if rumen or body temperature is taken as the measure, since 10 appendix aims name it; validated_commercial is not available on that reading because KB 3/04 and Optris have no appendix row. Listed in open_questions.md; the missing rule is how to grade a criterion with no measure. Device needed per the unsure rule from the cheapest commercial candidate, where commercial means an appendix product whose aim states the candidate measurement (rules.md rule 4.4, version 0.1.4): the 10 products whose aims name temperature are boluses, ear tags and a collar, all animal_mounted, so animal_mounted. The thermal cameras Stygar page 10 name for thermal comfort do not count, because their appendix aims name udder health, mastitis, inflammation, fever or lameness; a farm_fixed reading would need one whose aim states temperature or thermal comfort. Five of those aims name fever, which is a raised body temperature; the row reads a detection aim as not stating the measure, the literal reading that is one of the two candidates on I006 and I020 (both of which still count detection aims in vendors_naming_it), and a reader may challenge it. The weather station Maroto Molina say commercial farms use is not in the appendix and does not set the class. Rule 4.2 split (15 October 2026): the first candidate is now research_demonstrated or theoretically_measurable, since Maroto Molina page 3 cite studies of heat stress in dairy cows (Abeni and Galli 2017; Bewley and Schutz 2010) for a criterion the protocol gives no measure; which of the two applies is left open with the rest of the question, and the cell stays unsure.</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>No product states access to pasture, and Maroto Molina do not discuss the measure, so none under rules.md rule 4.2. Their outdoor location passage on page 3 is assigned to I041, access to an outdoor loafing area or pasture (decision_log.md, 2 October 2026), although the Welfare Quality method for I041 also asks for days and hours on pasture; a reader who carried it over would grade this row research_only, animal_mounted. Grazing time is a feeding behaviour measured on the cow, not the provision of access, so under rule 4.2 it is not the same measure. Device needed none: no technology is named for the row, and the definition takes the value from the manager's answers, not records. IceTag's aim names "pastur activity" with the number of steps; it does not match the search word and is not access to pasture.</t>
+          <t>No product states access to pasture, and Maroto Molina do not discuss the measure, so none under rules.md rule 4.2. Their outdoor location passage on page 3 is assigned to I041, access to an outdoor loafing area or pasture (decision_log.md, 2 October 2026), although the Welfare Quality method for I041 also asks for days and hours on pasture; a reader who carried it over would grade this row theoretically_measurable (a substitute measure), animal_mounted. Grazing time is a feeding behaviour measured on the cow, not the provision of access, so under rule 4.2 it is not the same measure. Device needed none: no technology is named for the row, and the definition takes the value from the manager's answers, not records. IceTag's aim names "pastur activity" with the number of steps; it does not match the search word and is not access to pasture.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit corrections to the evidence since 2021: I021/I025 tested (ICAR Brolis), I058 unsure, exact stronger-grade rule, records and prose fixed.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work in progress. Every indicator has a sensor row and four scheme rows. The sensor grades rest on the 2021 baseline (Stygar and colleagues 2021, Maroto Molina and colleagues 2020); the dated pass for later studies, from Kevin's change request of 7 October 2026, is still to come, so the ranking is provisional. A row whose Row status is 'Not yet checked' would have no row in 2_research/sensor_coverage.csv.</t>
+          <t>Work in progress. Every indicator has a sensor row and four scheme rows. The sensor grades rest on the 2021 baseline (Stygar and colleagues 2021, Maroto Molina and colleagues 2020) and, since 16 October 2026, on a second grade from studies and makers' pages since 2021 (2_research/rules.md, rule 4.11); two points of that rule are provisional until Kevin answers, so the ranking is provisional. A row whose Row status is 'Not yet checked' would have no row in 2_research/sensor_coverage.csv.</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Studies and maker pages since 2021, read in October 2026: 7 tested; 6 claimed; 4 shown in research; 8 proposed only; 28 nothing found; 5 unclear. The stronger of the two grades, used for the score and Kevin's lists: 10 tested; 3 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 6 unclear.</t>
+          <t>Studies and maker pages since 2021, read in October 2026: 8 tested; 4 claimed; 4 shown in research; 8 proposed only; 28 nothing found; 6 unclear. The stronger of the two grades, used for the score and Kevin's lists: 9 tested; 3 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 7 unclear.</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Siachos et al. 2024 tested the CattleEye body condition scores against an experienced assessor (weighted kappa 0.69) with a CattleEye author, which the provisional rule records as maker involvement; Swartz et al. 2025 and CattleEye's own page confirm it is on sale. Read as an abstract.</t>
+          <t>Siachos et al. 2024 tested the CattleEye body condition scores against an experienced assessor (weighted kappa 0.69) with a CattleEye author, which the provisional rule records as maker involvement; Swartz et al. 2025 and CattleEye's own page confirm it is on sale. Read as an abstract; the abstract does not name the product, which Swartz et al. 2025 identify as CattleEye in their full text, and the Europe PMC record gives one author's affiliation as CattleEye Ltd.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -1371,7 +1371,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1450,20 +1450,24 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>I058</t>
+          <t>I004</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mastitis: Individual cow somatic cell count (SCC)</t>
+          <t>Locomotory disorders: Hock alterations</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>EFSA only</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>EFSA and Welfare Quality</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Integument alterations</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -1471,12 +1475,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Not stated by EFSA</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1486,50 +1490,46 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Hubner2023LactiCyte;Maker:pagepedersen_lacticyte_hd;Maker:delaval_milk_cell_analysis</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>As on I057: the LactiCyte HD was tested against flow cytometry on individual cow samples, with independent authors.</t>
+          <t>Nothing on hock alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Named in FARM, with a number to meet</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>Nothing extra: already in milk records or farm records</t>
-        </is>
-      </c>
-      <c r="S5" s="2" t="inlineStr">
-        <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector checks farm records</t>
+          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
@@ -1539,15 +1539,15 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>Yes: RSPCA Assured (UK)</t>
+          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="X5" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>3 + 3 + 2 + 1 + 1</t>
+          <t>1 + 2 + 0 + 3 + 2</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
@@ -1557,12 +1557,12 @@
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>EFSA Table 27 (continued), PDF page 44: the ABM is "Specified increases in individual cow SCC values between consecutive monthly recordings (or in case of AMS between milkings) to indicate a new infection has occurred"; feasibility high, "but information not routinely available in all farms" (even fewer farms with AMS). Keyword scan: 3 aims name somatic cells or SCC: Lely MQC-C (appendix sheet 1 row 91, milk quality sensors, conductivity, spectrometer and viscosity, aim milk yield and somatic cell count of each cow every 3 milkings, validation flag yes), LIC Protrack SCC (row 94, viscosity, individual somatic cell count in real time during milking, no flag) and Gea M6850 (row 71, permittivity sensor, SCC on each udder quarter during milking, no flag). Stygar Table 2 page 7 has no somatic cell count trait; it lists the Lely on line California mastitis test (43) under Mastitis detection, commercial farm, lower performance column, and Table 1 page 6 gives it a viscosity meter, with 43 in the independent validation column by text position. Stygar page 4 describes study 43 as an experiment "testing performance of online somatic cell count (SCC) estimation in automatic milking system" with above 4,000 milking cows; reference 43 (page 14) is Deng et al. 2020, "Performance of online somatic cell count estimation in automatic milking systems"; appendix sheet 2 codes Deng et al. commercial herds, 4829 cows, external independent validation. Why 43 is MQC-C: MQC-C is the only one of the six Lely rows with a validation flag, and its viscosity sensor matches Table 1 (I006). Maroto Molina page 3: "Milk somatic cell count can be monitored by near infrared spectroscopy (NIRS), even for the individual cow by incorporating this technology into milking robots" (Kawasaki et al. 2008), rated partial (indicators.csv). Stygar page 11: commercially available systems such as milking robots provide data on SCC.</t>
+          <t>Keyword scan: 0 hits. Maroto Molina page 3: sensor systems for detecting integument alterations have not been found in literature, computer vision systems for skin problems in humans could be adapted (indicators.csv I004, partial).</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>Candidates as on I057: validated_commercial, because study 43 tested online somatic cell count estimation in automatic milking systems on commercial farms, the AMS case EFSA names, with the product MQC-C, whose aim states somatic cell count of each cow, and Stygar page 8 says "real-time milk analyzers agreed moderately with SCC (43)"; commercial_unvalidated, because Table 2 files study 43 under Mastitis detection and rule 4.2 counts a trait only when its name is the same measure, while three aims state somatic cell count. Listed in open_questions.md. The missing rule is whether a study that, by Stygar's own text and the reference title, tested the indicator's measure counts when Table 2 files it under another trait name. products names the three appendix products whose aims state somatic cell count; P018, the Ekomilk analyser in products.csv, is on the ICAR list and not in the Stygar list, so it is outside this 2021 baseline. Device needed routine_data under the records rule (rules.md rule 4.4): EFSA's definition takes the values from consecutive monthly recordings, which is milk recording, and the class list names somatic cell count from records. EFSA's feasibility line says the information is not routinely available in all farms; I025 is routine_data under the same rule although EFSA writes that it "would require all farmers to participate in milk recording" (Table 46, PDF page 76). In the AMS case the per milking value needs an inline sensor such as MQC-C, Protrack SCC or M6850, farm_fixed, the added device alternative.</t>
+          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>I004</t>
+          <t>I005</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Locomotory disorders: Hock alterations</t>
+          <t>Locomotory disorders: Knee alterations</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1619,13 +1619,13 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Nothing on hock alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
+          <t>Nothing on knee alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 0 hits. Maroto Molina page 3: sensor systems for detecting integument alterations have not been found in literature, computer vision systems for skin problems in humans could be adapted (indicators.csv I004, partial).</t>
+          <t>As I004; EFSA Table 18 lists hock and knee alterations separately, Maroto Molina treat integument alterations as one measure.</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
+          <t>As I004. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I004: Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -1694,24 +1694,20 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>I005</t>
+          <t>I006</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Locomotory disorders: Knee alterations</t>
+          <t>Mastitis: Clinical cases</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>EFSA and Welfare Quality</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Integument alterations</t>
-        </is>
-      </c>
+          <t>EFSA only</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -1734,29 +1730,33 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Bausewein2022AMS</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Nothing on knee alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
+          <t>Bausewein et al. 2022 tested the mastitis alerts of four makers' milking robots against a clinical udder examination of 7096 cows on 114 farms (sensitivity 61.4% to 78.2%, specificity 79.2% to 92.2%), with independent authors, though the makers advised on the alerts and supplied data. It detects cases at one visit, while EFSA's measure is the incidence rate of clinical mastitis, the same open question that keeps the 2021 grade unsure, so this grade is unsure too: validated_commercial if detection counts, otherwise theoretically_measurable. Listed in open_questions.md.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Named in FARM, with a number to meet</t>
+          <t>FARM has only a related housing, equipment or practice rule</t>
         </is>
       </c>
       <c r="T7" s="2" t="n">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
+          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): inspector checks farm records</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
+          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US)</t>
         </is>
       </c>
       <c r="X7" s="2" t="n">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 3 + 2</t>
+          <t>0 + 2 + 3 + 1 + 2</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr">
@@ -1801,12 +1801,12 @@
       </c>
       <c r="AA7" s="2" t="inlineStr">
         <is>
-          <t>As I004; EFSA Table 18 lists hock and knee alterations separately, Maroto Molina treat integument alterations as one measure.</t>
+          <t>Stygar Table 2 page 7 lists Lely on line CMT (43) under Mastitis detection, commercial farm, lower performance column; Table 1 page 6 places 43 in the independent column. HerdInsight (30, Brassel et al. 2019, health disorder alarms) is listed under Health disorder (footnote d: e.g., mastitis or pneumonia) and its appendix aim names heat detection, health and feeding behaviour, not mastitis; under rules factor 1 a health disorder trait is not the same measure as clinical mastitis cases, so 30 does not count for I006. Appendix aims: FirstLook Mastitis system names mastitis identification; ten aims name udder health. Maroto Molina do not discuss clinical mastitis incidence (I006). Why Stygar's Lely on line CMT (43) is the appendix product MQC-C: in stygar_2021_supplementary.xlsx, sheet Appendix table 1, row 91, MQC-C (provider Lely) has sensor type milk quality sensors (conductivity, spectrometer, viscosity), aim milk yield and somatic cell count of each cow every 3 milkings, and validation flag yes. It is the only one of the six Lely rows (Qwes HR-LD, Lely Calm Compact +, Lely Calm Vario +, Cosmix, Astronaut A4, MQC-C) with a validation flag, and its viscosity sensor matches the sensor Table 1 page 6 gives for the Lely on line California mastitis test, a viscosity meter. MQC-C is an inline milk sensor fitted at the milking point, so its class is farm_fixed.</t>
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>As I004. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I004: Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
+          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), farm_fixed under rule 4.4 (an analyser at the milking point is one installation per parlour; DeLaval DCC, a cytometry camera whose appendix row does not place it at the milking point, is farm_fixed as a camera), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
         </is>
       </c>
     </row>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>I006</t>
+          <t>I008</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Mastitis: Clinical cases</t>
+          <t>Restriction of movement and resting problems: Step activity</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1842,47 +1842,55 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Cow Manager; IceTag; RumiWatch; CowScout S</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Active behavior (walking, no. of steps), Table 2 page 7, research and commercial farms, lower performance column for every product listed</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Bausewein2022AMS</t>
+          <t>Charlton2022IceQube</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Bausewein et al. 2022 tested the mastitis alerts of four makers' milking robots against a clinical udder examination of 7096 cows on 114 farms (sensitivity 61.4% to 78.2%, specificity 79.2% to 92.2%), with independent authors. It detects cases at one visit, while EFSA's measure is the incidence rate of clinical mastitis, the same open question that keeps the 2021 grade unsure, so this grade is unsure too: validated_commercial if detection counts, otherwise theoretically_measurable. Listed in open_questions.md.</t>
+          <t>Charlton et al. 2022 tested step counts of the CowAlert IceQube, a commercial leg sensor, against live observation in three housing systems, with independent authors (step count agreement CCC 0.55 to 0.68 indoors, up to 0.93 at pasture on the back leg).</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
+          <t>One device per animal (collar, ear tag, bolus)</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1891,21 +1899,21 @@
         </is>
       </c>
       <c r="T8" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): inspector checks farm records</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US)</t>
         </is>
       </c>
       <c r="X8" s="2" t="n">
@@ -1913,7 +1921,7 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>0 + 2 + 3 + 1 + 2</t>
+          <t>3 + 1 + 3 + 1 + 0</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -1923,12 +1931,12 @@
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7 lists Lely on line CMT (43) under Mastitis detection, commercial farm, lower performance column; Table 1 page 6 places 43 in the independent column. HerdInsight (30, Brassel et al. 2019, health disorder alarms) is listed under Health disorder (footnote d: e.g., mastitis or pneumonia) and its appendix aim names heat detection, health and feeding behaviour, not mastitis; under rules factor 1 a health disorder trait is not the same measure as clinical mastitis cases, so 30 does not count for I006. Appendix aims: FirstLook Mastitis system names mastitis identification; ten aims name udder health. Maroto Molina do not discuss clinical mastitis incidence (I006). Why Stygar's Lely on line CMT (43) is the appendix product MQC-C: in stygar_2021_supplementary.xlsx, sheet Appendix table 1, row 91, MQC-C (provider Lely) has sensor type milk quality sensors (conductivity, spectrometer, viscosity), aim milk yield and somatic cell count of each cow every 3 milkings, and validation flag yes. It is the only one of the six Lely rows (Qwes HR-LD, Lely Calm Compact +, Lely Calm Vario +, Cosmix, Astronaut A4, MQC-C) with a validation flag, and its viscosity sensor matches the sensor Table 1 page 6 gives for the Lely on line California mastitis test, a viscosity meter. MQC-C is an inline milk sensor fitted at the milking point, so its class is farm_fixed.</t>
+          <t>Stygar Table 2 page 7, Active behavior (walking, no. of steps): every entry sits in the lower performance column, research farms CowManager SensOor (17, 39, 40), IceTag (28), Lely activity (42), RumiWatch (38), commercial farms CowScout Leg (27), IceTag (26, 27); page 6 text: for active behavior, lower performance of tools was reported. Table 1 page 6 columns: 39, 40, 28 and 26 independent; 17 and 38 self; on the IceTag row 21 and 26 to 28 sit in the independent column while the supplementary table codes 27 (Nielsen 2018) self, and on the CowScout Leg row 27 sits in the self column, so for P013 both sources agree on self. Appendix aims naming steps or walking: IceTag, IceQube, CowScout S.</t>
         </is>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), farm_fixed under rule 4.4 (an analyser at the milking point is one installation per parlour; DeLaval DCC, a cytometry camera whose appendix row does not place it at the milking point, is farm_fixed as a camera), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
+          <t>The keyword activity matches 39 aims. 28 of them name heat detection, and five are rumen boluses (eBolus, Moow Rumen bolus, smaXtec basic, smaXtec premium, VitalHerd). Only IceTag's aim names steps, and only IceTag, IceQube and CowScout S name walking; with the keywords step; walking the count would be 3. The count is reported as is and the keywords are visible. EFSA Table 31 rates on farm feasibility low; the appendix shows the opposite for the market. Table 1 also lists Lely activity (42, Elischer 2013, independent) but no appendix row is named Lely activity and no Lely row other than MQC-C carries a validation flag, so ref 42 is not attached to a product here. RumiWatch is not in products.csv and is cited as an appendix product. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. CowAlert IceQube (P016) names walking in its appendix aim, but Table 2 page 7 does not list it under Active behavior, so it is not among the products behind this grade.</t>
         </is>
       </c>
     </row>
@@ -1938,12 +1946,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>I008</t>
+          <t>I021</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Restriction of movement and resting problems: Step activity</t>
+          <t>Metabolic disorders: Subclinical ketosis: individual cow milk constituents</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1959,19 +1967,19 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
@@ -1979,27 +1987,27 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Cow Manager; IceTag; RumiWatch; CowScout S</t>
+          <t>AfiLab</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Active behavior (walking, no. of steps), Table 2 page 7, research and commercial farms, lower performance column for every product listed</t>
+          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Charlton2022IceQube</t>
+          <t>ICAR2025Brolis;Maker:brolis_herdline_home;Maker:brolis_herdline;Ponzo2026AMS;Maker:lely_astronaut_a5_next;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2023FPR</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Charlton et al. 2022 tested step counts of the CowAlert IceQube, a commercial leg sensor, against live observation in three housing systems, with independent authors (step count agreement CCC 0.55 to 0.68 indoors, up to 0.93 at pasture on the back leg).</t>
+          <t>ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; the robot is on sale, though Lely's page does not claim this measurement. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2008,11 +2016,11 @@
         </is>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>One device per animal (collar, ear tag, bolus)</t>
+          <t>Nothing extra: already in milk records or farm records</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -2043,7 +2051,7 @@
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>3 + 1 + 3 + 1 + 0</t>
+          <t>3 + 3 + 1 + 1 + 0</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -2053,12 +2061,12 @@
       </c>
       <c r="AA9" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Active behavior (walking, no. of steps): every entry sits in the lower performance column, research farms CowManager SensOor (17, 39, 40), IceTag (28), Lely activity (42), RumiWatch (38), commercial farms CowScout Leg (27), IceTag (26, 27); page 6 text: for active behavior, lower performance of tools was reported. Table 1 page 6 columns: 39, 40, 28 and 26 independent; 17 and 38 self; on the IceTag row 21 and 26 to 28 sit in the independent column while the supplementary table codes 27 (Nielsen 2018) self, and on the CowScout Leg row 27 sits in the self column, so for P013 both sources agree on self. Appendix aims naming steps or walking: IceTag, IceQube, CowScout S.</t>
+          <t>EFSA Table 46 page 75 defines the ABM as the individual milk fat to protein ratio or early lactation fat percentage monitored at routine milk recording. Stygar Table 2 page 7 lists AfiLab real time milk analyzer (25) under Milk quality, research farm, lower performance column; footnote e reads fat, lactose and protein as indicator for mastitis. Ref 25, Kaniyamattam and De Vries, agreement between milk fat, protein and lactose observations from DHIA and a real time milk analyzer, coded external independent validation in the supplementary study table. Appendix row AfiLab: milk quality sensors (spectrometer), aim milk composition analysis, monitoring general health and udder health, validation flag yes.</t>
         </is>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>The keyword activity matches 39 aims. 28 of them name heat detection, and five are rumen boluses (eBolus, Moow Rumen bolus, smaXtec basic, smaXtec premium, VitalHerd). Only IceTag's aim names steps, and only IceTag, IceQube and CowScout S name walking; with the keywords step; walking the count would be 3. The count is reported as is and the keywords are visible. EFSA Table 31 rates on farm feasibility low; the appendix shows the opposite for the market. Table 1 also lists Lely activity (42, Elischer 2013, independent) but no appendix row is named Lely activity and no Lely row other than MQC-C carries a validation flag, so ref 42 is not attached to a product here. RumiWatch is not in products.csv and is cited as an appendix product. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. CowAlert IceQube (P016) names walking in its appendix aim, but Table 2 page 7 does not list it under Active behavior, so it is not among the products behind this grade.</t>
+          <t>The measure is the same, individual cow milk fat and protein; Stygar record its validation as an indicator for mastitis, so the purpose differs and the note says so. The EFSA definition takes the value at routine milk recording, which the farm already has, so the class is routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser is the added device alternative, farm_fixed. Keyword fat and protein return 0 aims because the appendix describes these products as milk composition analysis.</t>
         </is>
       </c>
     </row>
@@ -2068,104 +2076,80 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>I021</t>
+          <t>I030</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Subclinical ketosis: individual cow milk constituents</t>
+          <t>Water provision</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>EFSA only</t>
+          <t>Welfare Quality only</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+          <t>About the housing or equipment</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>AfiLab</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
-        </is>
-      </c>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Maker:brolis_herdline;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2023FPR;Ponzo2025AMS</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>The makers' own pages say the Brolis HerdLine, DeLaval Milk Solids Analysis and Lemmer-Fullwood M²erlin measure milk fat and protein for each cow. No study since 2021 tested the fat to protein ratio of a product confirmed on sale against a reference: Antanaitis et al. 2023 used HerdLine without a reference, and Ponzo et al. 2025 compared Lely robot fat and protein with official recording (r 0.52 and 0.48), but Lely's current page claims no fat or protein measurement.</t>
+          <t>No source read since 2021 covers water points.</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Nothing extra: already in milk records or farm records</t>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
+          <t>Named in FARM</t>
         </is>
       </c>
       <c r="T10" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: FARM v5 (US industry)</t>
         </is>
       </c>
       <c r="X10" s="2" t="n">
@@ -2173,7 +2157,7 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>3 + 3 + 1 + 1 + 0</t>
+          <t>1 + 2 + 0 + 2 + 3</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
@@ -2183,12 +2167,12 @@
       </c>
       <c r="AA10" s="2" t="inlineStr">
         <is>
-          <t>EFSA Table 46 page 75 defines the ABM as the individual milk fat to protein ratio or early lactation fat percentage monitored at routine milk recording. Stygar Table 2 page 7 lists AfiLab real time milk analyzer (25) under Milk quality, research farm, lower performance column; footnote e reads fat, lactose and protein as indicator for mastitis. Ref 25, Kaniyamattam and De Vries, agreement between milk fat, protein and lactose observations from DHIA and a real time milk analyzer, coded external independent validation in the supplementary study table. Appendix row AfiLab: milk quality sensors (spectrometer), aim milk composition analysis, monitoring general health and udder health, validation flag yes.</t>
+          <t>Maroto Molina page 2: monitoring the number and status of water points has no relevance from a PLF perspective, since water consumption of every cow can be measured by a combination of RFID and flowmeters (Cardot et al. 2008), or indirectly by reticular temperature boluses. The Welfare Quality measure is the provision of water points, a resource measure, so this is a substitute measure and the grade is research_only under rules.md rule 4.2. Stygar Table 2 page 7 lists Insentec (45) under Water intake, research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation; the appendix row is Hokofarm Group RIC (Insentec, now Hokofarm), load cells and RFID, aim measures individual feed and water intake, flag yes.</t>
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>The measure is the same, individual cow milk fat and protein; Stygar record its validation as an indicator for mastitis, so the purpose differs and the note says so. The EFSA definition takes the value at routine milk recording, which the farm already has, so the class is routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser is the added device alternative, farm_fixed. Keyword fat and protein return 0 aims because the appendix describes these products as milk composition analysis.</t>
+          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water point measure. A study of the substitute does not demonstrate the indicator, even in cattle.</t>
         </is>
       </c>
     </row>
@@ -2198,12 +2182,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>I030</t>
+          <t>I031</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Water provision</t>
+          <t>Cleanliness of water points</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2229,7 +2213,7 @@
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
@@ -2289,12 +2273,12 @@
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>Maroto Molina page 2: monitoring the number and status of water points has no relevance from a PLF perspective, since water consumption of every cow can be measured by a combination of RFID and flowmeters (Cardot et al. 2008), or indirectly by reticular temperature boluses. The Welfare Quality measure is the provision of water points, a resource measure, so this is a substitute measure and the grade is research_only under rules.md rule 4.2. Stygar Table 2 page 7 lists Insentec (45) under Water intake, research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation; the appendix row is Hokofarm Group RIC (Insentec, now Hokofarm), load cells and RFID, aim measures individual feed and water intake, flag yes.</t>
+          <t>Welfare Quality PDF page 24 (printed 23): a resource based measure; the assessor checks the inner side of the bowl or trough for old or fresh dirt and staining of the water; clean when there is no evidence of crusts of dirt or decayed food residues. Maroto Molina page 2: as regards water quality, there are turbidity sensors able to measure water cleanliness, but it could be assumed to be adequate if water intake is normal. Keyword scan: 0 aims name turbidity, water quality or water cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: regarding the thirst criterion only resource based indicators are evaluated.</t>
         </is>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water point measure. A study of the substitute does not demonstrate the indicator, even in cattle.</t>
+          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina only propose turbidity sensors for water cleanliness and cite no study that used them at a water point.</t>
         </is>
       </c>
     </row>
@@ -2304,88 +2288,112 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>I031</t>
+          <t>I012</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Cleanliness of water points</t>
+          <t>Restriction of movement and resting problems: Lying time</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality only</t>
+          <t>EFSA only</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>About the housing or equipment</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>Observed or recorded on the animal</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>AfiAct II; IceQube, cowAlert; Cow Manager; Track a))) Cow; RumiWatch; MooMonitor +; CowScout S; IceTag</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Non-active behavior (lying, lying and standing), Table 2 page 7: high performance column for AfiAct Pedometer Plus (21), AfiTagII (22), CowAlert IceQube (21), CowManager SensOor (17, 39), Track A Cow (21) and RumiWatch (38) on research farms and for CowScout Leg (27) and Ice Tag (26, 27) on commercial farms; lower performance column for CowManager SensOor (40), MooMonitor+ (18) and Pedometer Plus (23) on research farms</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr"/>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Charlton2022IceQube;Pichlbauer2024pasture</t>
+        </is>
+      </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>No source read since 2021 covers water points.</t>
+          <t>Charlton et al. 2022 tested CowAlert IceQube lying time against live observation (CCC 0.99 to 1.00), and Pichlbauer et al. 2024 tested the RumiWatch pedometer (CCC above 0.99) and the SMARTBOW ear tag (0.55) on pasture against drone video; authors independent of the makers (Smartbow supplied the ear tag data).</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>One device per animal (collar, ear tag, bolus)</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>FARM has only a related housing, equipment or practice rule</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
-        </is>
-      </c>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>Named in FARM</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="W12" s="2" t="inlineStr">
-        <is>
-          <t>Yes: FARM v5 (US industry)</t>
-        </is>
-      </c>
       <c r="X12" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 2 + 3</t>
+          <t>3 + 1 + 2 + 1 + 0</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
@@ -2395,12 +2403,12 @@
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality PDF page 24 (printed 23): a resource based measure; the assessor checks the inner side of the bowl or trough for old or fresh dirt and staining of the water; clean when there is no evidence of crusts of dirt or decayed food residues. Maroto Molina page 2: as regards water quality, there are turbidity sensors able to measure water cleanliness, but it could be assumed to be adequate if water intake is normal. Keyword scan: 0 aims name turbidity, water quality or water cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: regarding the thirst criterion only resource based indicators are evaluated.</t>
+          <t>Stygar Table 2 page 7, Non-active behavior (lying, lying and standing): high performance on research farms for AfiAct Pedometer Plus (21), AfiTagII (22), CowAlert IceQube (21), CowManager SensOor (17, 39), Track A Cow (21) and RumiWatch (38), and on commercial farms for CowScout Leg (27), IceTag (26, 27) and a prototype (59); lower performance for CowManager SensOor (40), Lely activity (42), MooMonitor+ (18) and Pedometer Plus (23). Supplementary study table: 21, 22, 23, 26, 39, 40 and 18 are external independent validation; 17, 27 and 38 external self validation. Maroto Molina page 3: pedometers and accelerometers provide data on lying time and lying bouts.</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina only propose turbidity sensors for water cleanliness and cite no study that used them at a water point.</t>
+          <t>Non active behaviour is the trait Stygar report as most often validated, 20 trials. EFSA Table 33 page 54 rates on farm feasibility low because validated activity monitors are not widely available. The appendix product AfiAct II (P001) corresponds to the Table 1 row AfiAct Pedometer Plus, AfiTagII, Pedometer Plus. Lely activity (42) has no appendix row and is not cited as a product. Track A Cow, RumiWatch and MooMonitor+ are not in products.csv and are cited as appendix products. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. Stygar's trait pools lying with lying and standing, and Table 2 page 7 does not say which trial measured lying alone; the decision_log entry of 29 September maps the trait to lying time (rules.md rule 4.2).</t>
         </is>
       </c>
     </row>
@@ -2410,12 +2418,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>I012</t>
+          <t>I020</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Restriction of movement and resting problems: Lying time</t>
+          <t>Metabolic disorders: Clinical ketosis: clinical case incidence rate</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2431,60 +2439,52 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>AfiAct II; IceQube, cowAlert; Cow Manager; Track a))) Cow; RumiWatch; MooMonitor +; CowScout S; IceTag</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Non-active behavior (lying, lying and standing), Table 2 page 7: high performance column for AfiAct Pedometer Plus (21), AfiTagII (22), CowAlert IceQube (21), CowManager SensOor (17, 39), Track A Cow (21) and RumiWatch (38) on research farms and for CowScout Leg (27) and Ice Tag (26, 27) on commercial farms; lower performance column for CowManager SensOor (40), MooMonitor+ (18) and Pedometer Plus (23) on research farms</t>
-        </is>
-      </c>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Charlton2022IceQube;Pichlbauer2024pasture</t>
+          <t>RoblesTrillo2026ketosis</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Charlton et al. 2022 tested CowAlert IceQube lying time against live observation (CCC 0.99 to 1.00), and Pichlbauer et al. 2024 tested the RumiWatch pedometer (CCC above 0.99) and the SMARTBOW ear tag (0.55) on pasture against drone video; authors independent of the makers.</t>
+          <t>Robles-Trillo et al. 2026 predicted ketosis from collar and conductivity data, a substitute measure; no study since 2021 measured the incidence of clinical ketosis itself.</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>One device per animal (collar, ear tag, bolus)</t>
+          <t>Nothing extra: already in milk records or farm records</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -2493,21 +2493,21 @@
         </is>
       </c>
       <c r="T13" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="X13" s="2" t="n">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>3 + 1 + 2 + 1 + 0</t>
+          <t>0 + 3 + 1 + 1 + 2</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
@@ -2525,12 +2525,12 @@
       </c>
       <c r="AA13" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Non-active behavior (lying, lying and standing): high performance on research farms for AfiAct Pedometer Plus (21), AfiTagII (22), CowAlert IceQube (21), CowManager SensOor (17, 39), Track A Cow (21) and RumiWatch (38), and on commercial farms for CowScout Leg (27), IceTag (26, 27) and a prototype (59); lower performance for CowManager SensOor (40), Lely activity (42), MooMonitor+ (18) and Pedometer Plus (23). Supplementary study table: 21, 22, 23, 26, 39, 40 and 18 are external independent validation; 17, 27 and 38 external self validation. Maroto Molina page 3: pedometers and accelerometers provide data on lying time and lying bouts.</t>
+          <t>Keyword scan: 1 aim names ketosis, Afimilk AfiMilk MPC, milk quality sensor (spectrometer), aim Ketosis and SARA detection, no validation flag in the appendix. Stygar Table 2 lists no ketosis trait. Maroto Molina do not discuss ketosis (indicators.csv I020).</t>
         </is>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>Non active behaviour is the trait Stygar report as most often validated, 20 trials. EFSA Table 33 page 54 rates on farm feasibility low because validated activity monitors are not widely available. The appendix product AfiAct II (P001) corresponds to the Table 1 row AfiAct Pedometer Plus, AfiTagII, Pedometer Plus. Lely activity (42) has no appendix row and is not cited as a product. Track A Cow, RumiWatch and MooMonitor+ are not in products.csv and are cited as appendix products. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. Stygar's trait pools lying with lying and standing, and Table 2 page 7 does not say which trial measured lying alone; the decision_log entry of 29 September maps the trait to lying time (rules.md rule 4.2).</t>
+          <t>Candidates: commercial_unvalidated, a product states ketosis detection; none, the EFSA ABM is the incidence rate of clinical cases from veterinary or farm records, not detection. Same question as I006. Listed in open_questions.md. Device needed routine_data under the records rule (rules.md rule 4.4, first written in version 0.1.3, applied to unsure rows since version 0.2): EFSA Table 46 (PDF page 75) defines the ABM as the incidence rate of clinical ketosis estimated from veterinary diagnoses, farm records or national databases. The added device alternative is the candidate product AfiMilk MPC, an inline milk analyser (spectrometer) installed in the parlour, farm_fixed. The appendix aim dates from 2021 and has not been re-verified; the row follows the appendix as the rule requires.</t>
         </is>
       </c>
     </row>
@@ -2540,12 +2540,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>I020</t>
+          <t>I024</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Clinical ketosis: clinical case incidence rate</t>
+          <t>Metabolic disorders: Left displaced abomasum: clinical case incidence rate</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2561,12 +2561,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -2576,33 +2576,33 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>RoblesTrillo2026ketosis</t>
+          <t>Suzuki2026LDA</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Robles-Trillo et al. 2026 predicted ketosis from collar and conductivity data, a substitute measure; no study since 2021 measured the incidence of clinical ketosis itself.</t>
+          <t>Suzuki et al. 2026 predicted left displaced abomasum from rumination data, a substitute measure.</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>0 + 3 + 1 + 1 + 2</t>
+          <t>1 + 3 + 0 + 1 + 2</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr">
@@ -2647,12 +2647,12 @@
       </c>
       <c r="AA14" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 1 aim names ketosis, Afimilk AfiMilk MPC, milk quality sensor (spectrometer), aim Ketosis and SARA detection, no validation flag in the appendix. Stygar Table 2 lists no ketosis trait. Maroto Molina do not discuss ketosis (indicators.csv I020).</t>
+          <t>Keyword scan: 0 aims name abomasum or displacement. Stygar Table 2 lists no such trait. Maroto Molina do not discuss it. EFSA Table 46 page 75 defines the ABM as the incidence rate from veterinary diagnoses, farm records or national databases.</t>
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>Candidates: commercial_unvalidated, a product states ketosis detection; none, the EFSA ABM is the incidence rate of clinical cases from veterinary or farm records, not detection. Same question as I006. Listed in open_questions.md. Device needed routine_data under the records rule (rules.md rule 4.4, first written in version 0.1.3, applied to unsure rows since version 0.2): EFSA Table 46 (PDF page 75) defines the ABM as the incidence rate of clinical ketosis estimated from veterinary diagnoses, farm records or national databases. The added device alternative is the candidate product AfiMilk MPC, an inline milk analyser (spectrometer) installed in the parlour, farm_fixed. The appendix aim dates from 2021 and has not been re-verified; the row follows the appendix as the rule requires.</t>
+          <t>No product, so the detection versus incidence question does not arise here. Device needed routine_data under the records rule (rules.md rule 4.4, version 0.1.3): EFSA Table 46 (PDF page 75) takes the incidence rate of left displaced abomasum from veterinary diagnoses, farm records or national databases, so the value exists with no added device. No added device is named by Stygar or Maroto Molina.</t>
         </is>
       </c>
     </row>
@@ -2662,12 +2662,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>I024</t>
+          <t>I025</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Left displaced abomasum: clinical case incidence rate</t>
+          <t>Metabolic disorders: Subacute ruminal acidosis: individual cow milk constituents</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2683,75 +2683,83 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>AfiLab</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Suzuki2026LDA</t>
+          <t>ICAR2025Brolis;Maker:brolis_herdline_home;Maker:brolis_herdline;Ponzo2026AMS;Maker:lely_astronaut_a5_next;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2024SARA;Grige2026SARA</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Suzuki et al. 2026 predicted left displaced abomasum from rumination data, a substitute measure.</t>
+          <t>As on I021: ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; the robot is on sale, though Lely's page does not claim this measurement. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Nothing extra: already in milk records or farm records</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>Not named in FARM</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="R15" s="2" t="inlineStr">
-        <is>
-          <t>Nothing extra: already in milk records or farm records</t>
-        </is>
-      </c>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="W15" s="2" t="inlineStr">
-        <is>
-          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="X15" s="2" t="n">
@@ -2759,7 +2767,7 @@
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>1 + 3 + 0 + 1 + 2</t>
+          <t>3 + 3 + 1 + 0 + 0</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">
@@ -2769,12 +2777,12 @@
       </c>
       <c r="AA15" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 0 aims name abomasum or displacement. Stygar Table 2 lists no such trait. Maroto Molina do not discuss it. EFSA Table 46 page 75 defines the ABM as the incidence rate from veterinary diagnoses, farm records or national databases.</t>
+          <t>EFSA Table 46 page 76 defines the ABM as individual milk fat percentage and fat to protein ratio monitored at routine milk recording, as a sign of subacute ruminal acidosis. The same milk constituents as I021, measured by the same validated analyser: AfiLab (25), Stygar Table 2 page 7, Milk quality, research farm, lower performance column; ref 25 external independent validation.</t>
         </is>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>No product, so the detection versus incidence question does not arise here. Device needed routine_data under the records rule (rules.md rule 4.4, version 0.1.3): EFSA Table 46 (PDF page 75) takes the incidence rate of left displaced abomasum from veterinary diagnoses, farm records or national databases, so the value exists with no added device. No added device is named by Stygar or Maroto Molina.</t>
+          <t>Same evidence as I021; the indicator differs only in which disorder the constituents point to. AfiMilk MPC states ketosis and SARA detection in its aim with no validation flag and is not needed for the grade. Class routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser AfiLab, farm_fixed, is the added device alternative.</t>
         </is>
       </c>
     </row>
@@ -2784,12 +2792,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>I025</t>
+          <t>I028</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Subacute ruminal acidosis: individual cow milk constituents</t>
+          <t>Metabolic disorders: Clinical hypocalcaemia: clinical case incidence rate</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2805,12 +2813,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2820,41 +2828,33 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>AfiLab</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
-        </is>
-      </c>
+          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Maker:brolis_herdline;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2024SARA;Ponzo2025AMS</t>
+          <t>Gleissenberger2025motility</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>As on I021: three makers' pages claim milk fat and protein for each cow, and no study since 2021 tested the fat to protein ratio of a product confirmed on sale against a reference.</t>
+          <t>Gleissenberger et al. 2025 predicted low calcium from bolus rumination and motility data, a substitute measure, with smaXtec employees among the authors.</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
@@ -2863,25 +2863,25 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Not named in FARM</t>
+          <t>FARM has only a related housing, equipment or practice rule</t>
         </is>
       </c>
       <c r="T16" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="X16" s="2" t="n">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>3 + 3 + 1 + 0 + 0</t>
+          <t>1 + 3 + 0 + 1 + 2</t>
         </is>
       </c>
       <c r="Z16" s="2" t="inlineStr">
@@ -2899,12 +2899,12 @@
       </c>
       <c r="AA16" s="2" t="inlineStr">
         <is>
-          <t>EFSA Table 46 page 76 defines the ABM as individual milk fat percentage and fat to protein ratio monitored at routine milk recording, as a sign of subacute ruminal acidosis. The same milk constituents as I021, measured by the same validated analyser: AfiLab (25), Stygar Table 2 page 7, Milk quality, research farm, lower performance column; ref 25 external independent validation.</t>
+          <t>Keyword scan: 0 aims. Stygar Table 2 lists no such trait. Maroto Molina do not discuss it. EFSA Table 46 page 76 defines the ABM as the incidence rate of clinical hypocalcaemia from veterinary diagnoses, farm records or national databases.</t>
         </is>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>Same evidence as I021; the indicator differs only in which disorder the constituents point to. AfiMilk MPC states ketosis and SARA detection in its aim with no validation flag and is not needed for the grade. Class routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser AfiLab, farm_fixed, is the added device alternative.</t>
+          <t>Device needed routine_data under the records rule (rules.md rule 4.4, version 0.1.3): EFSA Table 46 (PDF page 76) takes the incidence rate of clinical hypocalcaemia from veterinary diagnoses, farm records or national databases, so the value exists with no added device. No added device is named by Stygar or Maroto Molina.</t>
         </is>
       </c>
     </row>
@@ -2914,12 +2914,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>I028</t>
+          <t>I058</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Clinical hypocalcaemia: clinical case incidence rate</t>
+          <t>Mastitis: Individual cow somatic cell count (SCC)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2935,48 +2935,48 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Not stated by EFSA</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Gleissenberger2025motility</t>
+          <t>Hubner2023LactiCyte;Maker:pagepedersen_lacticyte_hd;Maker:delaval_milk_cell_analysis</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Gleissenberger et al. 2025 predicted low calcium from bolus rumination and motility data, a substitute measure, with smaXtec employees among the authors.</t>
+          <t>As on I057, the LactiCyte HD was tested against flow cytometry on single samples, with independent authors. EFSA's measure for this row is a specified increase in a cow's cell count between consecutive recordings, which signals a new infection. Whether a device that measures each cow's count at each recording measures that increase is the same kind of question as on I006, so the grade is unsure: validated_commercial if it does, otherwise theoretically_measurable. Listed in open_questions.md.</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
@@ -2989,11 +2989,11 @@
         </is>
       </c>
       <c r="T17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>RSPCA Assured (UK): inspector checks farm records</t>
         </is>
       </c>
       <c r="V17" s="2" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US)</t>
+          <t>Yes: RSPCA Assured (UK)</t>
         </is>
       </c>
       <c r="X17" s="2" t="n">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>1 + 3 + 0 + 1 + 2</t>
+          <t>0 + 3 + 2 + 1 + 1</t>
         </is>
       </c>
       <c r="Z17" s="2" t="inlineStr">
@@ -3021,12 +3021,12 @@
       </c>
       <c r="AA17" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 0 aims. Stygar Table 2 lists no such trait. Maroto Molina do not discuss it. EFSA Table 46 page 76 defines the ABM as the incidence rate of clinical hypocalcaemia from veterinary diagnoses, farm records or national databases.</t>
+          <t>EFSA Table 27 (continued), PDF page 44: the ABM is "Specified increases in individual cow SCC values between consecutive monthly recordings (or in case of AMS between milkings) to indicate a new infection has occurred"; feasibility high, "but information not routinely available in all farms" (even fewer farms with AMS). Keyword scan: 3 aims name somatic cells or SCC: Lely MQC-C (appendix sheet 1 row 91, milk quality sensors, conductivity, spectrometer and viscosity, aim milk yield and somatic cell count of each cow every 3 milkings, validation flag yes), LIC Protrack SCC (row 94, viscosity, individual somatic cell count in real time during milking, no flag) and Gea M6850 (row 71, permittivity sensor, SCC on each udder quarter during milking, no flag). Stygar Table 2 page 7 has no somatic cell count trait; it lists the Lely on line California mastitis test (43) under Mastitis detection, commercial farm, lower performance column, and Table 1 page 6 gives it a viscosity meter, with 43 in the independent validation column by text position. Stygar page 4 describes study 43 as an experiment "testing performance of online somatic cell count (SCC) estimation in automatic milking system" with above 4,000 milking cows; reference 43 (page 14) is Deng et al. 2020, "Performance of online somatic cell count estimation in automatic milking systems"; appendix sheet 2 codes Deng et al. commercial herds, 4829 cows, external independent validation. Why 43 is MQC-C: MQC-C is the only one of the six Lely rows with a validation flag, and its viscosity sensor matches Table 1 (I006). Maroto Molina page 3: "Milk somatic cell count can be monitored by near infrared spectroscopy (NIRS), even for the individual cow by incorporating this technology into milking robots" (Kawasaki et al. 2008), rated partial (indicators.csv). Stygar page 11: commercially available systems such as milking robots provide data on SCC.</t>
         </is>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>Device needed routine_data under the records rule (rules.md rule 4.4, version 0.1.3): EFSA Table 46 (PDF page 76) takes the incidence rate of clinical hypocalcaemia from veterinary diagnoses, farm records or national databases, so the value exists with no added device. No added device is named by Stygar or Maroto Molina.</t>
+          <t>Candidates as on I057: validated_commercial, because study 43 tested online somatic cell count estimation in automatic milking systems on commercial farms, the AMS case EFSA names, with the product MQC-C, whose aim states somatic cell count of each cow, and Stygar page 8 says "real-time milk analyzers agreed moderately with SCC (43)"; commercial_unvalidated, because Table 2 files study 43 under Mastitis detection and rule 4.2 counts a trait only when its name is the same measure, while three aims state somatic cell count. Listed in open_questions.md. The missing rule is whether a study that, by Stygar's own text and the reference title, tested the indicator's measure counts when Table 2 files it under another trait name. products names the three appendix products whose aims state somatic cell count; P018, the Ekomilk analyser in products.csv, is on the ICAR list and not in the Stygar list, so it is outside this 2021 baseline. Device needed routine_data under the records rule (rules.md rule 4.4): EFSA's definition takes the values from consecutive monthly recordings, which is milk recording, and the class list names somatic cell count from records. EFSA's feasibility line says the information is not routinely available in all farms; I025 is routine_data under the same rule although EFSA writes that it "would require all farmers to participate in milk recording" (Table 46, PDF page 76). In the AMS case the per milking value needs an inline sensor such as MQC-C, Protrack SCC or M6850, farm_fixed, the added device alternative.</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
@@ -3197,7 +3197,7 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Peacock Technology's page lists Lying Bouts as an output of its IDS i-QUBE leg sensor; no independent test of lying bouts as such was found. Charlton et al. 2022 tested the IceQube's lying and standing transitions per hour (CCC 0.81 to 0.96) and Kroese et al. 2024 detected lying to standing transitions by camera; whether a count of transitions is the frequency of lying bouts is not settled, so they are recorded without raising the grade.</t>
+          <t>Peacock Technology's page lists Lying Bouts as an output of its IDS i-QUBE leg sensor; no test of lying bouts as such against a reference was found. Charlton et al. 2022 tested the IceQube's lying and standing transitions per hour (CCC 0.81 to 0.96) and Kroese et al. 2024 detected lying to standing transitions by camera; whether a count of transitions is the frequency of lying bouts is not settled, so they are recorded without raising the grade. The i-QUBE appears to be the current form of the IceQube, product P016 in the 2021 list; no page says so.</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -3319,7 +3319,7 @@
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -3559,7 +3559,7 @@
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr"/>
@@ -3665,7 +3665,7 @@
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr"/>
@@ -3877,7 +3877,7 @@
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr"/>
@@ -3995,7 +3995,7 @@
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -4105,7 +4105,7 @@
       <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
@@ -4211,7 +4211,7 @@
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr"/>
@@ -4317,7 +4317,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr"/>
@@ -4423,7 +4423,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
@@ -4529,7 +4529,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr"/>
@@ -4635,7 +4635,7 @@
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr"/>
@@ -4753,7 +4753,7 @@
       <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
+          <t>Shown in research: a study since 2021 measured it in cattle, with no product sold for it</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -4879,7 +4879,7 @@
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
+          <t>Shown in research: a study since 2021 measured it in cattle, with no product sold for it</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -5005,7 +5005,7 @@
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -5115,7 +5115,7 @@
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr"/>
@@ -5221,7 +5221,7 @@
       <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -5331,7 +5331,7 @@
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr"/>
@@ -5547,7 +5547,7 @@
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr"/>
@@ -5653,7 +5653,7 @@
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr"/>
@@ -5759,7 +5759,7 @@
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr"/>
@@ -5877,7 +5877,7 @@
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -5999,7 +5999,7 @@
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Hoofcount's own page says PediVue images are analysed by computer vision to detect early signs of digital dermatitis per cow; no independent test of it was found. The studies since 2021 in the sources read measure foot temperature, a substitute (Spadola et al. 2026). A thermal camera study of digital dermatitis (Feighelstein et al. 2024) was found two steps through the reviews, beyond the one step the provisional rule allows, so it is not counted.</t>
+          <t>Hoofcount's own page says PediVue images are analysed by computer vision to detect early signs of digital dermatitis per cow; no test of it against a reference was found. The studies since 2021 in the sources read measure foot temperature, a substitute (Spadola et al. 2026). A thermal camera study of digital dermatitis (Feighelstein et al. 2024) was found two steps through the reviews, beyond the one step the provisional rule allows, so it is not counted.</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -6121,7 +6121,7 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
+          <t>Shown in research: a study since 2021 measured it in cattle, with no product sold for it</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -6231,7 +6231,7 @@
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr"/>
@@ -6349,7 +6349,7 @@
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -6471,7 +6471,7 @@
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -6593,7 +6593,7 @@
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Shown in research: no product in the Stygar list claims this measure, but a study the sensor sources cite measured it in cattle</t>
+          <t>Shown in research: a study since 2021 measured it in cattle, with no product sold for it</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
@@ -6813,7 +6813,7 @@
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr"/>
@@ -7041,7 +7041,7 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Proposed only: the sources since 2021 only propose a method, show one in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr"/>
@@ -7147,7 +7147,7 @@
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr"/>
@@ -7253,7 +7253,7 @@
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr"/>
@@ -7381,7 +7381,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>Suzuki et al. 2021 and Cao et al. 2025 tested the HORIBA LAQUAtwin Ca-11C, which HORIBA's page offers for cow side use, against laboratory analysers with independent authors, but it measures ionised calcium in whole blood, while EFSA's measure is serum calcium; and a hand held meter on a blood sample may not belong in this sensor column. Listed in open_questions.md.</t>
+          <t>Suzuki et al. 2021 and Cao et al. 2025 tested the HORIBA LAQUAtwin Ca-11C, which HORIBA's page offers for cow side use and Cao et al. call commercially available, against a benchtop blood gas analyser and the handheld i-STAT 1, with independent authors; it measures ionised calcium in whole blood, while EFSA's measure is total serum calcium. Leal Yepes et al. 2023 tested an ARKRAY point of care analyser on serum total calcium against a laboratory analyser (serum sensitivity 64.7%), with devices supplied by the maker; no source says it is on sale. So the grade is validated_commercial if ionised whole blood calcium counts as EFSA's measure, otherwise research_demonstrated. Listed in open_questions.md.</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -7493,7 +7493,7 @@
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr"/>
@@ -7611,7 +7611,7 @@
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr"/>
@@ -7729,7 +7729,7 @@
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Nothing found: neither sensor source names a product or a method for it, as of their dates (2020 and 2021)</t>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr"/>
@@ -22276,7 +22276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -22593,7 +22593,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G4.json record 35; primary/antanaitis_2023_PMC10603915.xml</t>
+          <t>bounded search group G4 record 35 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G4.json record 37; primary/antanaitis_2024_PMC11240606.xml</t>
+          <t>bounded search group G4 record 37 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -22870,7 +22870,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>none stated</t>
+          <t>makers consulted on which alerts to use; makers' service teams provided herds, AMS data and support (Acknowledgments)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results G1.json record 29; A1.json record 12; full text primary/bausewein_2022_PMC9405299.xml</t>
+          <t>bounded search group G1 record 29; group A1 record 12 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -22947,7 +22947,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>not_stated</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -22997,7 +22997,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G7.json record 14; primary/cao_2025_PMC11758346.xml</t>
+          <t>bounded search group G7 record 14 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -23095,7 +23095,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>lee_supp/lee_2025_dataset.xlsx sheet 'Sifted articles' row 40 (Behaviors Detected includes self-grooming); full text primary/carslake_2021_PMC7795166.xml</t>
+          <t>lee_2025_dataset.xlsx sheet 'Sifted articles' row 40 (Behaviors Detected includes self-grooming)</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -23197,7 +23197,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>lee_2025_wearables.pdf Table 4 (PDF page 9, row Charlton, G. 2022) and reference list; full text primary/charlton_2022_PMC8909491.xml</t>
+          <t>lee_2025_wearables.pdf Table 4 (PDF page 9, row Charlton, G. 2022) and reference list</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -23299,7 +23299,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G4.json record 34; primary/dejong_2023_PMC10663411.xml</t>
+          <t>bounded search group G4 record 34 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -23357,7 +23357,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>commercial_farm</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -23499,7 +23499,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G7.json record 4; primary/gleissenberger_2025_PMC12649405.xml</t>
+          <t>bounded search group G7 record 4 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G6.json record 1 and A6.json record 1; primary/grige_2026_PMC13454269.xml</t>
+          <t>bounded search group G6 record 1 and group A6 record 1 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -23703,7 +23703,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results A2.json record 9; full text primary/lacticyte_2023_PMC10692336.xml</t>
+          <t>bounded search group A2 record 9 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -24059,7 +24059,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>laboratory</t>
+          <t>commercial_farm</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -24074,7 +24074,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>none stated</t>
+          <t>the maker supplied the devices and test strips (Acknowledgments)</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -24099,7 +24099,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G7.json record 31; primary/lealyepes_2023_PMC10505766.xml</t>
+          <t>bounded search group G7 record 31 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
@@ -24109,7 +24109,7 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>Samples from commercial farms stored at -80 C and run in the laboratory. ARKRAY provided the devices and test strips; one author at Boehringer Ingelheim Animal Health, none at ARKRAY; "The authors have not stated any conflicts of interest".</t>
+          <t>Samples from commercial farms stored at -80 C and run in the laboratory. ARKRAY provided the devices and test strips; one author at Boehringer Ingelheim Animal Health, none at ARKRAY; "The authors have not stated any conflicts of interest". Samples from one commercial farm, analysed in a laboratory.</t>
         </is>
       </c>
     </row>
@@ -24397,7 +24397,7 @@
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>lee_2025_wearables.pdf text, PDF page 4 (section Precision, reproducibility, accuracy and bias: 'Pichlbauer et al., 2024') and reference list; one step from Lee (decision 1 of 16 October 2026); full text primary/pichlbauer_2024_PMC11644843.xml</t>
+          <t>lee_2025_wearables.pdf text, PDF page 4 (section Precision, reproducibility, accuracy and bias: 'Pichlbauer et al., 2024') and reference list; one step from Lee (decision 1 of 16 October 2026)</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr">
@@ -24414,7 +24414,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Ponzo2025AMS</t>
+          <t>Ponzo2026AMS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -24424,7 +24424,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Ponzo E, Moretti R, Masia F, Vrieze E, Sacchi P, Chessa S (2025). Assessing the Reliability of Automatic Milking Systems Data to Support Genetic Improvement in Dairy Cattle. Animals (Basel) 16(1): 1</t>
+          <t>Ponzo E, Moretti R, Masia F, Vrieze E, Sacchi P, Chessa S (2026). Assessing the Reliability of Automatic Milking Systems Data to Support Genetic Improvement in Dairy Cattle. Animals (Basel) 16(1): 1</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -24434,7 +24434,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>not_stated</t>
+          <t>commercial_farm</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -24499,7 +24499,7 @@
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results G2.json record 19; full text primary/ponzo_2025_PMC12785074.xml</t>
+          <t>bounded search group G2 record 19 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
@@ -24509,7 +24509,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>COI: 'Fernando Masia and Elisa Vrieze are employed by the company Lely International N.V.' Text says AMS 'could also be equipped with sensors performing somatic cell count' and that external calibration data were not entered on these farms. Farms not stated as commercial. Bausewein 2022 names Lely's SCC system as MQC-C. Licence CC BY.</t>
+          <t>COI: 'Fernando Masia and Elisa Vrieze are employed by the company Lely International N.V.' Text says AMS 'could also be equipped with sensors performing somatic cell count' and that external calibration data were not entered on these farms. Bausewein 2022 names Lely's SCC system as MQC-C. Licence CC BY. Published online on 19 December 2025 in the 2026 volume; the year of the journal issue is used.</t>
         </is>
       </c>
     </row>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>not_stated (grants listed by Europe PMC: Conseil Regional des Pays de la Loire, Association nationale de la recherche technique)</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>lee_supp/lee_2025_dataset.xlsx sheet 'Sifted articles' row 102 (Behaviors Detected lists distance travelled and duration before lying down in the pasture); abstract from Europe PMC (PMID 34092420)</t>
+          <t>lee_2025_dataset.xlsx sheet 'Sifted articles' row 102 (Behaviors Detected lists distance travelled and duration before lying down in the pasture); abstract from Europe PMC (PMID 34092420)</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -24699,7 +24699,7 @@
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G4.json record 14</t>
+          <t>bounded search group G4 record 14 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr">
@@ -24801,7 +24801,7 @@
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results G3.json record 13; A1.json record 17; full text primary/saila_2023_PMC10382826.xml</t>
+          <t>bounded search group G3 record 13; group A1 record 17 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr">
@@ -25011,7 +25011,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>Author M Lennox affiliated with CattleEye Ltd, so not independent of the maker. Test on 4 dairy farms (training data from 7). Full text not in Europe PMC</t>
+          <t>The abstract does not name the product; Swartz et al. 2025 identify it as CattleEye and cite this study as its body condition validation. The Europe PMC record, kept in the source file, gives author M Lennox's affiliation as CattleEye Ltd. Author M Lennox affiliated with CattleEye Ltd, so not independent of the maker. Test on 4 dairy farms (training data from 7). Full text not in Europe PMC</t>
         </is>
       </c>
     </row>
@@ -25054,7 +25054,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Handheld infrared thermography camera (FLIR ThermaCam P25)</t>
+          <t>infrared thermography camera (FLIR ThermaCam P25)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -25201,7 +25201,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G7.json record 37; primary/suzuki_2021_PMC8182322.xml</t>
+          <t>bounded search group G7 record 37 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -25303,7 +25303,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>milkmeta_results/G5.json record 3; primary/suzuki_2026_PMC13000433.xml</t>
+          <t>bounded search group G5 record 3 (2_research/bounded_search_2026-10-16.md)</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>The maker page names CattleEye, offers it for sale with prices, and claims daily mobility scores for lameness detection.; The maker page names CattleEye, offers it for sale, and claims automatic body condition scoring of each cow.</t>
+          <t>The maker page names CattleEye, offers a Starter Kit for purchase online (UK only), and claims daily mobility scores and automatic body condition scoring of each cow.</t>
         </is>
       </c>
     </row>
@@ -26729,7 +26729,7 @@
       </c>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>Page and Pedersen, which designs and sells LactiCyte HD and owns the lacticyte.com domain, lists it with price on request and claims somatic cell counts for individual cow milk.</t>
+          <t>The page names LactiCyte HD, says results from individual cows, bulk tanks and tanker trucks are reported, and asks buyers to contact the company for the price.</t>
         </is>
       </c>
     </row>
@@ -26815,7 +26815,7 @@
       </c>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>The maker page for this rear leg sensor lists lying bouts by name among its outputs, though i-QUBE appears to be the current form of IceQube, already a Stygar product (P016), so check before treating it as new; search tried: dairy cow sensor lying bouts lying time monitoring product.</t>
+          <t>The maker page for this rear leg sensor lists lying bouts by name among its outputs, though i-QUBE appears to be the current form of IceQube, already a Stygar product (P016), so check before treating it as new; search tried: dairy cow sensor lying bouts lying time monitoring product. On 17 October 2026 the address redirects to https://www.peacocktechnology.com/ids-i-qube.</t>
         </is>
       </c>
     </row>
@@ -26902,6 +26902,280 @@
       <c r="T48" s="2" t="inlineStr">
         <is>
           <t>The maker page sells the pH bolus for 6 to 10 percent of the herd and claims continuous pH and SARA detection, though the bolus sits in the reticulum rather than the rumen and accuracy is stated only to day 150.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ICAR2025Brolis</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>ICAR Measuring, Recording and Sampling Devices Sub-Committee 2025, Brolis BLH01: Validation of Principle for an Inline Analyser for Milk Fat and Protein, fact sheet and summary of ICAR validation test findings, 26 June 2025</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.icar.org/wp-content/uploads/documents/Brolis-BLH01-Validation-Test-Summary-Fact-Sheet-Final-Website.pdf</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>I021;I025</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Brolis BLH01 in line analyser (Brolis HerdLine)</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>in line spectroscopic milk analyser in an automatic milking system</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>not_stated</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>105 measurements on each of two devices</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>fat and protein content of individual cows' milk at each milking</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>reference values under ICAR's validation test (bias and regression against them are reported)</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>bias -0.002 and -0.006 g/100 g for fat and protein on a BouMatic Gemini, -0.08 and -0.02 on a DeLaval V300; RMSPE for milk fat 2.6% with R2 98.2%</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="inlineStr">
+        <is>
+          <t>full text (three pages)</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>ICAR validated sensor systems page in 1_sources; the Brolis home page calls its analyser ICAR-validated</t>
+        </is>
+      </c>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>icar_brolis_report.pdf</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>An ICAR test report rather than a journal article. On sale per the maker's home page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Maker:brolis_herdline_home</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>maker_page</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Brolis Sensor Technology, Brolis HerdLine (maker's home page)</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>https://brolisherdline.com/</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>I021;I025</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Brolis HerdLine</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>the maker's own page</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>The first and only ICAR-validated In-line Milk analyzer; Receive more information about our product, pricing</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr"/>
+      <c r="Q50" s="2" t="inlineStr">
+        <is>
+          <t>maker page</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Vendor check of 16 and 17 October 2026</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>maker_brolis_herdline_home.txt</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Shows the analyser on sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Maker:lely_astronaut_a5_next</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>maker_page</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Lely, Astronaut A5 Next (maker's page)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/milking/astronaut/</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>I021;I025</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Lely Astronaut A5 Next</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>the maker's own page</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>The page offers the Astronaut A5 Next robot and names no fat or protein measurement</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr"/>
+      <c r="P51" s="2" t="inlineStr"/>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>maker page</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>Vendor check of 16 and 17 October 2026</t>
+        </is>
+      </c>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>maker_lely_astronaut_a5_next.txt</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>Shows the robot on sale; it is the product Ponzo et al. 2026 tested, and the page does not claim the fat and protein measurement.</t>
         </is>
       </c>
     </row>
@@ -26916,7 +27190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -29911,6 +30185,174 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Lely, Astronaut A5 Next: maker's web page, saved 16 October 2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>maker_lely_astronaut_a5_next.txt</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Vendor check since 2021: I021, I025 (the robot is on sale; the page claims no fat or protein measurement)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>© the maker, no licence stated</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/milking/astronaut/</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lely.com/solutions/milking/astronaut/</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Brolis HerdLine: maker's home page, saved 17 October 2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>maker_brolis_herdline_home.txt</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Vendor check since 2021: I021, I025 (on sale, ICAR validated)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>© the maker, no licence stated</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>https://brolisherdline.com/</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>https://brolisherdline.com/</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Meckbach C et al. 2021, Sensors 21:7585 (full text, Europe PMC)</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>ref_meckbach2021gps.xml</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>found_along_the_way.md section 11 (a sensor name in the Lee 2025 dataset)</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>cc by</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s21227585</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8624045/fullTextXML</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Yu et al. 2024, Animals 14:458 (full text, Europe PMC)</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>ref_yu2024standing.xml</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>found_along_the_way.md section 11 (a figure in Islam 2026 Table 7)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>cc by</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ani14030458</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10854845/fullTextXML</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Second round of audit corrections: ICAR test reports admitted through a maker's page, Lely A5 Next wording, record fixes, rules 0.7.1, source check fixes for three stable documents.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -2007,7 +2007,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; the robot is on sale, though Lely's page does not claim this measurement. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
+          <t>ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; Lely's page now sells the A5 Next, which it says builds on the A5, and does not claim this measurement, so this test is recorded but the grade rests on the ICAR test. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>As on I021: ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; the robot is on sale, though Lely's page does not claim this measurement. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
+          <t>As on I021: ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; Lely's page now sells the A5 Next, which it says builds on the A5, and does not claim this measurement, so this test is recorded but the grade rests on the ICAR test. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow. Grige et al. 2026 used HerdLine data in a classifier for acidosis against bolus pH, not a fat or protein test.</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -22870,7 +22870,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>makers consulted on which alerts to use; makers' service teams provided herds, AMS data and support (Acknowledgments)</t>
+          <t>makers consulted on which alerts to use; makers' service teams provided herds, AMS data and support (Methods and Acknowledgments)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -24059,7 +24059,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>commercial_farm</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -24109,7 +24109,7 @@
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>Samples from commercial farms stored at -80 C and run in the laboratory. ARKRAY provided the devices and test strips; one author at Boehringer Ingelheim Animal Health, none at ARKRAY; "The authors have not stated any conflicts of interest". Samples from one commercial farm, analysed in a laboratory.</t>
+          <t>Samples from one commercial farm stored at -80 C and run in the laboratory. ARKRAY provided the devices and test strips; one author at Boehringer Ingelheim Animal Health, none at ARKRAY; "The authors have not stated any conflicts of interest". Blood was collected on the farm and measured in a laboratory.</t>
         </is>
       </c>
     </row>
@@ -24504,7 +24504,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>ev_ponzo2025ams.xml</t>
+          <t>ev_ponzo2026ams.xml</t>
         </is>
       </c>
       <c r="T22" s="2" t="inlineStr">
@@ -25011,7 +25011,7 @@
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
-          <t>The abstract does not name the product; Swartz et al. 2025 identify it as CattleEye and cite this study as its body condition validation. The Europe PMC record, kept in the source file, gives author M Lennox's affiliation as CattleEye Ltd. Author M Lennox affiliated with CattleEye Ltd, so not independent of the maker. Test on 4 dairy farms (training data from 7). Full text not in Europe PMC</t>
+          <t>The abstract does not name the product; Swartz et al. 2025 identify it as CattleEye and cite this study as its body condition validation. The Europe PMC record, kept in the source file, gives author M Lennox's affiliation as CattleEye Ltd, so the authors are not independent of the maker. Test on 4 dairy farms (training data from 7). Full text not in Europe PMC</t>
         </is>
       </c>
     </row>
@@ -26993,7 +26993,7 @@
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>ICAR validated sensor systems page in 1_sources; the Brolis home page calls its analyser ICAR-validated</t>
+          <t>Vendor check: the maker's home page (Maker:brolis_herdline_home) calls the analyser ICAR-validated; ICAR's report is in 1_sources</t>
         </is>
       </c>
       <c r="S49" s="2" t="inlineStr">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="T51" s="2" t="inlineStr">
         <is>
-          <t>Shows the robot on sale; it is the product Ponzo et al. 2026 tested, and the page does not claim the fat and protein measurement.</t>
+          <t>Shows the Astronaut A5 Next on sale; the page says it builds on the Astronaut A5, the robot Ponzo et al. 2026 tested, with a new operating system and updated features, and it claims no fat or protein measurement.</t>
         </is>
       </c>
     </row>
@@ -28723,7 +28723,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>ev_ponzo2025ams.xml</t>
+          <t>ev_ponzo2026ams.xml</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -30146,12 +30146,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Leliveld and Provolo 2020, supplementary Tables S1 to S3 (Europe PMC supplementary files)</t>
+          <t>Leliveld and Provolo 2020, supplementary Tables S1 to S3 (the archive inside Europe PMC's supplementary files zip)</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>leliveld_provolo_2020_supplementary.zip</t>
+          <t>leliveld_provolo_2020_supplementary.7z</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit corrections to step 4: I082 unsure for RSPCA and Certified Humane, I067/I082 management based, I065 supported, I066/I072 unsure on column 1, I068/I082 unsure and I075 claimed since 2021, records and prose fixed.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>48 established; 10 established input; 11 supported; 5 indirect or contested; 4 no welfare validation; 3 not framed as welfare. On the sensor side alone: 11 supported; 5 indirect or contested; 4 no welfare validation; 3 not framed as welfare.</t>
+          <t>48 established; 10 established input; 12 supported; 4 indirect or contested; 3 no welfare validation; 2 not framed as welfare; 2 unclear. On the sensor side alone: 12 supported; 4 indirect or contested; 3 no welfare validation; 2 not framed as welfare; 2 unclear.</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Studies and maker pages since 2021, read in October 2026: 14 tested; 17 claimed; 5 shown in research; 8 proposed only; 28 nothing found; 9 unclear. The stronger of the two grades, used for the score and Kevin's lists: 18 tested; 17 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 7 unclear.</t>
+          <t>Studies and maker pages since 2021, read in October 2026: 12 tested; 17 claimed; 5 shown in research; 8 proposed only; 28 nothing found; 11 unclear. The stronger of the two grades, used for the score and Kevin's lists: 16 tested; 19 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 7 unclear.</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Indirect or contested: one of those three sources says its link to welfare is indirect, insufficient on its own, inconsistent or debated</t>
+          <t>Indirect or contested: one of those three sources says its link to welfare is indirect, insufficient on its own, weak, inconsistent, unclear or not fully understood</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>No welfare validation: a product's description frames it as about health or welfare, or a scheme requires it, but none of the three sources links it to welfare</t>
+          <t>No welfare validation: none of the three sources links it to welfare, but a product's description says it is for health, welfare or a named condition, or it is itself a health or condition status, or a scheme requires it</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
+          <t>About farm management</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>The three sources were searched (EFSA 2023, Welfare Quality v3.2, Linstädt et al. 2024) and none links it to welfare in its own words. All three leave calves out of scope: EFSA 2023 covers dairy cows, the Welfare Quality text read is the dairy cow protocol, and Linstädt et al. 2024 sorted out calves as a wrong life stage. The one EFSA passage on automatic milk feeders compares rearing methods, not the milk each calf is given (section 4.4.8, PDF 74). No product aim says it is for health or welfare, but all four schemes require a minimum milk feeding for each calf (crosswalk.csv), and the four schemes are animal welfare standards, so they frame it as part of welfare.</t>
+          <t>The three sources were searched (EFSA 2023, Welfare Quality v3.2, Linstädt et al. 2024) and none links it to welfare in its own words. All three leave calves out of scope: EFSA 2023 covers dairy cows, the Welfare Quality text read is the dairy cow protocol, and Linstädt et al. 2024 sorted out calves as a wrong life stage. The one EFSA passage on automatic milk feeders compares rearing methods, not the milk each calf is given (section 4.4.8, PDF 74). No product aim says it is for health or welfare, but FARM v5 and Global Animal Partnership require that each calf is given milk or milk replacer (crosswalk.csv; for RSPCA Assured and Certified Humane it is unsure), and the four schemes are animal welfare standards, so they frame it as part of welfare.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -1608,7 +1608,7 @@
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Carslake 2021 (ev_carslake2021calves.xml, section 2.1) says an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan, and Lee Table 3 lists Forster Technik Compact Smart among its commercial products. No source since 2021 tests the milk a feeder gives each calf against a reference; Carslake does not say the feeder records the amounts, and it was published online in December 2020 in the January 2021 issue.</t>
+          <t>Carslake 2021 (ev_carslake2021calves.xml, section 2.1) says an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan, but it does not say the feeder measures or records the milk each calf is given, nor that the feeder is on sale; it was published online in December 2020 in the January 2021 issue. Lee Table 3 lists Forster Technik Compact Smart as an ear worn wearable, which is not the feeder. Candidate readings: commercial_unvalidated, if dispensing on an individual plan counts as measuring the milk fed, or none. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -1640,11 +1640,11 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector checks farm records; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>FARM v5 (US industry): inspector checks farm records; Global Animal Partnership (US): required, but the scheme does not say how it is checked; unclear whether RSPCA Assured (UK), Certified Humane (US) requires it</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -1658,11 +1658,11 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>2 + 2 + 3 + 2 + 3</t>
+          <t>2 + 2 + 3 + 2 + 2</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
@@ -1828,7 +1828,7 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
+          <t>About farm management</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1981,12 +1981,12 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Cow Manager; MooMonitor +; RumiWatch; Track a))) Cow; GrowSafe feed alley</t>
+          <t>Cow Manager; MooMonitor +; RumiWatch; Track a))) Cow; GrowSafe feed alley; RIC</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Feeding time, Table 2 page 7: lower performance on research farms for CowManager SensOor (17, 21, 39, 40), MooMonitor+ (18), RumiWatch (33, 34) and Track A Cow (21), high performance on a commercial farm for RumiWatch V0.7.3.2 (36) and lower for RumiWatch V0.7.2.0 (36); Presence at the feeder (animal identification and time), high performance on research farms for GrowSafe (44); Grazing time, high performance on research farms for MooMonitor+ (29) and RumiWatch (29, 38)</t>
+          <t>Feeding time, Table 2 page 7: lower performance on research farms for CowManager SensOor (17, 21, 39, 40), MooMonitor+ (18), RumiWatch (33, 34) and Track A Cow (21), high performance on a commercial farm for RumiWatch V0.7.3.2 (36) and lower for a prototype (59) and RumiWatch V0.7.2.0 (36); Presence at the feeder (animal identification and time), high performance on research farms for GrowSafe (44), Insentec (45) and Intergado (46, no row in the Stygar list); Grazing time, high performance on research farms for MooMonitor+ (29) and RumiWatch (29, 38)</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, rows Feeding time, Presence at the feeder and Grazing time, as in validated_trait. Table 1 page 6: GrowSafe (44) independent validation, RFID neck collar and load cell. The Stygar list row GrowSafe feed alley states Feeding duration. Stygar list AIM column: 20 products name feeding times, feeding behaviour, feeding duration or grazing (search words in search_words); every one is marked on the Sensors x products sheet.</t>
+          <t>Stygar Table 2 page 7, rows Feeding time, Presence at the feeder and Grazing time, as in validated_trait. Table 1 page 6: GrowSafe (44) independent validation, RFID neck collar and load cell; Insentec (45) independent validation, RFID ear tag and load cell, the Stygar list row Hokofarm Group RIC. The Stygar list row GrowSafe feed alley states Feeding duration. Stygar list AIM column: 20 products name feeding times, feeding behaviour, feeding duration or grazing (search words in search_words); every one is marked on the Sensors x products sheet.</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
         <is>
-          <t>The cheapest commercial class is farm_fixed: the GrowSafe feed alley, a feed alley with RFID and load cells, like the trough with RFID that rule 4.4 lists as farm_fixed. The other products whose aims name it are animal mounted collars and tags. Stygar's footnote defines presence at the feeder as animal identification and time, which is time spent at the feeder, the measure the GrowSafe aim calls feeding duration. Grazing time is counted here because MooMonitor+'s aim names grazing behaviour beside feeding times.</t>
+          <t>The cheapest commercial class is farm_fixed: the GrowSafe feed alley, a feed alley with RFID and load cells, like the trough with RFID that rule 4.4 lists as farm_fixed. The other products whose aims name it are animal mounted collars and tags. Stygar's footnote defines presence at the feeder as animal identification and time, which is time spent at the feeder, the measure the GrowSafe aim calls feeding duration. Grazing time is counted here because MooMonitor+'s aim names grazing behaviour beside feeding times. RIC is credited for presence at the feeder (45), as a tested product whose aim names feed intake, not feeding time, under the same reading as GrowSafe.</t>
         </is>
       </c>
     </row>
@@ -2203,12 +2203,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>I068</t>
+          <t>I071</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Oestrus (heat) detection (sensor side)</t>
+          <t>General health status and health alerts (sensor side)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2224,17 +2224,17 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Oestrus (heat) detection</t>
+          <t>General health status and health alerts</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Indirect or contested</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Links: EFSA 2023, section 6.2.3 (PDF 99): "Tethering imposes severe restriction of movement ... it particularly restricts ... oestrus, calving and social behaviour"; Linstädt et al. 2024 (PDF 14): "Oestrus intensity was linked to good welfare"; (PDF 7): clinical lameness "has an effect on reproductive hormones and sexual behavior". No passage questions the link.</t>
+          <t>Question: Linstädt et al. 2024 (PDF 13): "evaluating animal welfare requires a multidisciplinary approach, and health assessment alone falls short of determining overall well-being". Links as well: Welfare Quality protocol v3.2 (PDF 15, printed 14): "Animals should be free from disease"; Linstädt et al. 2024 (PDF 2): "Less diseases would also mean a better welfare." A question decides the grade (rule 4.14).</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
@@ -2242,24 +2242,32 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>HerdInsights</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Health disorder (for example mastitis or pneumonia), Table 2 page 7, commercial farm, lower performance column: HerdInsight (30)</t>
+        </is>
+      </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Schilkowsky2021SmartBow</t>
+          <t>Maker:smaxtec_ph_bolus;Maker:msd_sensehub_dairy;Maker:cowmed_smart_collar</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, which evaluated the oestrus alerts of the SmartBow ear tag in 216 lactating cows against the HeatWatch System, with sensitivity and specificity; Lee Table 3 and its discussion (PDF page 10) count Smartbow among the commercial wearables. The comparison is another system, which Lee treats as a comparison standard (cross validation against another sensor, PDF page 6); if that is not read as a reference method, the grade is commercial_unvalidated on the Herd Navigator, smaXtec, SenseHub, Cowmed and i-QUBE pages.</t>
+          <t>The smaXtec page says the bolus lets you monitor each cow's health status, the SenseHub page (maker_msd_sensehub_dairy.txt) offers health reports and alerts for cows needing attention, and the Cowmed page offers three level health alerts. The health studies from 2021 on in Lee's dataset (rows 5, 8, 18, 34) test alerts for named diseases (metritis, respiratory disease, diarrhoea), so none tests a general health alert.</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -2268,7 +2276,7 @@
         </is>
       </c>
       <c r="T9" s="2" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
@@ -2285,17 +2293,17 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>No scheme requires it (4 of 4 read); unclear whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear: whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it (see open questions)</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unclear: whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it (see open questions)</t>
         </is>
       </c>
       <c r="AA9" s="2" t="n">
@@ -2313,12 +2321,12 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>Stygar list AIM column: 31 products name heat (heat detection, or heat measurement for Herd Navigator), or progesterone (search words in search_words); every one is marked on the Sensors x products sheet. Stygar Table 2 page 7 has no oestrus trait, and rule 4.2 says activity is not oestrus.</t>
+          <t>Stygar Table 2 page 7, Health disorder: HerdInsight (30), commercial farm, lower performance. Table 1 page 6: HerdInsights, Alanya Ltd., Cork, accelerometer collar, independent validation (30). Page 7 text: the only validated study on the accelerometer based system used for health alarms (30) reported a high number of false positives, but the true health disorders were alerted before the farmer noticed them. Stygar list AIM column: 39 products name health in a general sense (search words in search_words, chosen so that udder health alone does not match); every one is marked on the Sensors x products sheet.</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
         <is>
-          <t>The cheapest commercial class is farm_fixed: DeLaval Herd Navigator, a milk analyser at the milking point (rule 4.4, milk analysers), whose aim names progesterone and heat measurement. The other 30 products are animal mounted activity collars and tags.</t>
+          <t>The cheapest commercial class is farm_fixed: AfiLab, an inline milk analyser whose aim names monitoring general health, and Herd Navigator, whose aim names milk analysis for health. The other products are animal mounted. Aims that name only udder health are on I006, not here.</t>
         </is>
       </c>
     </row>
@@ -2328,20 +2336,24 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>I071</t>
+          <t>I004</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>General health status and health alerts (sensor side)</t>
+          <t>Locomotory disorders: Hock alterations</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Sensor side only</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>EFSA and Welfare Quality</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Integument alterations</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -2349,59 +2361,59 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>General health status and health alerts</t>
+          <t>Integument alterations</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Indirect or contested</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Question: Linstädt et al. 2024 (PDF 13): "evaluating animal welfare requires a multidisciplinary approach, and health assessment alone falls short of determining overall well-being". Links as well: Welfare Quality protocol v3.2 (PDF 15, printed 14): "Animals should be free from disease"; Linstädt et al. 2024 (PDF 2): "Less diseases would also mean a better welfare." A question decides the grade (rule 4.14).</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>EFSA 2023, Table 18, PDF 33, lists it as an animal based measure; the Welfare Quality protocol v3.2 lists Integument alterations under the criterion Absence of injuries (overview, PDF 22, printed 21). Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>HerdInsights</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>Health disorder (for example mastitis or pneumonia), Table 2 page 7, commercial farm, lower performance column: HerdInsight (30)</t>
-        </is>
-      </c>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>Maker:smaxtec_ph_bolus;Maker:msd_sensehub_dairy;Maker:cowmed_smart_collar</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>The smaXtec page says the bolus lets you monitor each cow's health status, the SenseHub page (maker_msd_sensehub_dairy.txt) offers health reports and alerts for cows needing attention, and the Cowmed page offers three level health alerts. The health studies from 2021 on in Lee's dataset (rows 5, 8, 18, 34) test alerts for named diseases (metritis, respiratory disease, diarrhoea), so none tests a general health alert.</t>
+          <t>Nothing on hock alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="T10" s="2" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
@@ -2410,33 +2422,33 @@
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
+          <t>Named in FARM, with a number to meet</t>
         </is>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read); unclear whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it</t>
+          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>Unclear: whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it (see open questions)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>Unclear: whether RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US) requires it (see open questions)</t>
+          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="AA10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>3 + 2 + 3 + 1 + 0</t>
+          <t>1 + 2 + 0 + 3 + 2</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -2446,12 +2458,12 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Health disorder: HerdInsight (30), commercial farm, lower performance. Table 1 page 6: HerdInsights, Alanya Ltd., Cork, accelerometer collar, independent validation (30). Page 7 text: the only validated study on the accelerometer based system used for health alarms (30) reported a high number of false positives, but the true health disorders were alerted before the farmer noticed them. Stygar list AIM column: 39 products name health in a general sense (search words in search_words, chosen so that udder health alone does not match); every one is marked on the Sensors x products sheet.</t>
+          <t>Keyword scan: 0 hits. Maroto Molina page 3: sensor systems for detecting integument alterations have not been found in literature, computer vision systems for skin problems in humans could be adapted (indicators.csv I004, partial).</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
         <is>
-          <t>The cheapest commercial class is farm_fixed: AfiLab, an inline milk analyser whose aim names monitoring general health, and Herd Navigator, whose aim names milk analysis for health. The other products are animal mounted. Aims that name only udder health are on I006, not here.</t>
+          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -2461,20 +2473,24 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>I075</t>
+          <t>I005</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Milk yield (sensor side)</t>
+          <t>Locomotory disorders: Knee alterations</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Sensor side only</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>EFSA and Welfare Quality</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Integument alterations</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -2482,86 +2498,94 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Milk yield</t>
+          <t>Integument alterations</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Indirect or contested</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Questions: Linstädt et al. 2024 (PDF 12): "relying solely on milk yield is insufficient for gauging the comprehensive welfare of the herd"; (PDF 1): "high milk production alone does not indicate good welfare"; EFSA 2023, section 5.7 (PDF 80): "there is no clear evidence that herd size or milk yield could be useful characteristics to identify farms at risk of poor welfare". Links as well: EFSA 2023, section 4.1.1.2 (PDF 30): cows with septic arthritis show "reduced milk yield"; Linstädt et al. 2024 (PDF 7): poor mobility is linked to lower milk yields. A question decides the grade (rule 4.14).</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>EFSA 2023, Table 18, PDF 33, lists it as an animal based measure; the Welfare Quality protocol v3.2 lists Integument alterations under the criterion Absence of injuries (overview, PDF 22, printed 21). Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t>Ponzo2026AMS;Bausewein2022AMS</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records; two authors are Lely employees. Bausewein 2022 (ev_bausewein2022ams.xml) treats Lely and the other robots as commercial systems recording milk yield (kg). The paper does not say how the official recording weighed the milk.</t>
+          <t>Nothing on knee alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="T11" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>Nothing extra: already in milk records or farm records</t>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
         </is>
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>Not named in FARM</t>
+          <t>Named in FARM, with a number to meet</t>
         </is>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read); unclear whether RSPCA Assured (UK), Certified Humane (US) requires it</t>
+          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>Unclear: whether RSPCA Assured (UK), Certified Humane (US) requires it (see open questions)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>Unclear: whether RSPCA Assured (UK), Certified Humane (US) requires it (see open questions)</t>
+          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>3 + 3 + 3 + 0 + 0</t>
+          <t>1 + 2 + 0 + 3 + 2</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -2571,12 +2595,12 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>Stygar list AIM column: 13 milking robots, aim monitor and analyse the milk production performance; Lely MQC-C, Milk yield and somatic cells count; LIC Saber Milk, Milk yield, composition and conductivity. Stygar Table 2 page 7 has no milk yield trait. ICAR's list of validated sensor systems (1_sources/icar_validated_sensors.html) names the Panazoo MMI sensor (P020) for milk yield; it is not in the Stygar list, so it does not change this grade.</t>
+          <t>As I004; EFSA Table 18 lists hock and knee alterations separately, Maroto Molina treat integument alterations as one measure.</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
         <is>
-          <t>Rule 4.4 lists milk yield under routine_data, a value the milking system already collects with no new device, and the milking robots' aims say they monitor milk production.</t>
+          <t>As I004. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I004: Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
         </is>
       </c>
     </row>
@@ -2586,24 +2610,20 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>I004</t>
+          <t>I006</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Locomotory disorders: Hock alterations</t>
+          <t>Mastitis: Clinical cases</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>EFSA and Welfare Quality</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Integument alterations</t>
-        </is>
-      </c>
+          <t>EFSA only</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -2611,7 +2631,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Integument alterations</t>
+          <t>Mastitis</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -2621,7 +2641,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>EFSA 2023, Table 18, PDF 33, lists it as an animal based measure; the Welfare Quality protocol v3.2 lists Integument alterations under the criterion Absence of injuries (overview, PDF 22, printed 21). Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
+          <t>EFSA 2023, Table 27, PDF 43, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -2641,29 +2661,33 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr"/>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Bausewein2022AMS</t>
+        </is>
+      </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>Nothing on hock alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
+          <t>Bausewein et al. 2022 tested the mastitis alerts of four makers' milking robots against a clinical udder examination of 7096 cows on 114 farms (sensitivity 61.4% to 78.2%, specificity 79.2% to 92.2%), with independent authors, though the makers advised on the alerts and supplied data. It detects cases at one visit, while EFSA's measure is the incidence rate of clinical mastitis, the same open question that keeps the 2021 grade unsure, so this grade is unsure too: validated_commercial if detection counts, otherwise theoretically_measurable. Listed in open_questions.md.</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="T12" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
@@ -2672,7 +2696,7 @@
       </c>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>Named in FARM, with a number to meet</t>
+          <t>FARM has only a related housing, equipment or practice rule</t>
         </is>
       </c>
       <c r="W12" s="2" t="n">
@@ -2680,7 +2704,7 @@
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
+          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): inspector checks farm records</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -2690,7 +2714,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
+          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US)</t>
         </is>
       </c>
       <c r="AA12" s="2" t="n">
@@ -2698,7 +2722,7 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 3 + 2</t>
+          <t>0 + 2 + 3 + 1 + 2</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -2708,12 +2732,12 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>Keyword scan: 0 hits. Maroto Molina page 3: sensor systems for detecting integument alterations have not been found in literature, computer vision systems for skin problems in humans could be adapted (indicators.csv I004, partial).</t>
+          <t>Stygar Table 2 page 7 lists Lely on line CMT (43) under Mastitis detection, commercial farm, lower performance column; Table 1 page 6 places 43 in the independent column. HerdInsight (30, Brassel et al. 2019, health disorder alarms) is listed under Health disorder (footnote d: e.g., mastitis or pneumonia) and its appendix aim names heat detection, health and feeding behaviour, not mastitis; under rules factor 1 a health disorder trait is not the same measure as clinical mastitis cases, so 30 does not count for I006. Appendix aims: FirstLook Mastitis system names mastitis identification; ten aims name udder health. Maroto Molina do not discuss clinical mastitis incidence (I006). Why Stygar's Lely on line CMT (43) is the appendix product MQC-C: in stygar_2021_supplementary.xlsx, sheet Appendix table 1, row 91, MQC-C (provider Lely) has sensor type milk quality sensors (conductivity, spectrometer, viscosity), aim milk yield and somatic cell count of each cow every 3 milkings, and validation flag yes. It is the only one of the six Lely rows (Qwes HR-LD, Lely Calm Compact +, Lely Calm Vario +, Cosmix, Astronaut A4, MQC-C) with a validation flag, and its viscosity sensor matches the sensor Table 1 page 6 gives for the Lely on line California mastitis test, a viscosity meter. MQC-C is an inline milk sensor fitted at the milking point, so its class is farm_fixed.</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
         <is>
-          <t>The proposed technology is a camera, so the class of the proposal is farm_fixed. Nothing commercial. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
+          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), farm_fixed under rule 4.4 (an analyser at the milking point is one installation per parlour; DeLaval DCC, a cytometry camera whose appendix row does not place it at the milking point, is farm_fixed as a camera), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
         </is>
       </c>
     </row>
@@ -2723,24 +2747,20 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>I005</t>
+          <t>I008</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Locomotory disorders: Knee alterations</t>
+          <t>Restriction of movement and resting problems: Step activity</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>EFSA and Welfare Quality</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Integument alterations</t>
-        </is>
-      </c>
+          <t>EFSA only</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Observed or recorded on the animal</t>
@@ -2748,7 +2768,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Integument alterations</t>
+          <t>Restriction of movement (locomotion)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -2758,7 +2778,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>EFSA 2023, Table 18, PDF 33, lists it as an animal based measure; the Welfare Quality protocol v3.2 lists Integument alterations under the criterion Absence of injuries (overview, PDF 22, printed 21). Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
+          <t>EFSA 2023, Table 31, PDF 52, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -2768,66 +2788,78 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Cow Manager; IceTag; RumiWatch; CowScout S</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Active behavior (walking, no. of steps), Table 2 page 7, research and commercial farms, lower performance column for every product listed</t>
+        </is>
+      </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr"/>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Charlton2022IceQube</t>
+        </is>
+      </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Nothing on knee alterations in Hudson 2026, Silva 2021 or Islam 2026.</t>
+          <t>Charlton et al. 2022 tested step counts of the CowAlert IceQube, a commercial leg sensor, against live observation in three housing systems, with independent authors (step count agreement CCC 0.55 to 0.68 indoors, up to 0.93 at pasture on the back leg).</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="T13" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>One device per animal (collar, ear tag, bolus)</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>FARM has only a related housing, equipment or practice rule</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U13" s="2" t="inlineStr">
-        <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
-        </is>
-      </c>
-      <c r="V13" s="2" t="inlineStr">
-        <is>
-          <t>Named in FARM, with a number to meet</t>
-        </is>
-      </c>
-      <c r="W13" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector looks at the animals; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): inspector looks at the animals</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="Z13" s="2" t="inlineStr">
-        <is>
-          <t>Yes: RSPCA Assured (UK), FARM v5 (US industry), Global Animal Partnership (US)</t>
         </is>
       </c>
       <c r="AA13" s="2" t="n">
@@ -2835,7 +2867,7 @@
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 3 + 2</t>
+          <t>3 + 1 + 3 + 1 + 0</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
@@ -2845,12 +2877,12 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>As I004; EFSA Table 18 lists hock and knee alterations separately, Maroto Molina treat integument alterations as one measure.</t>
+          <t>Stygar Table 2 page 7, Active behavior (walking, no. of steps): every entry sits in the lower performance column, research farms CowManager SensOor (17, 39, 40), IceTag (28), Lely activity (42), RumiWatch (38), commercial farms CowScout Leg (27), IceTag (26, 27); page 6 text: for active behavior, lower performance of tools was reported. Table 1 page 6 columns: 39, 40, 28 and 26 independent; 17 and 38 self; on the IceTag row 21 and 26 to 28 sit in the independent column while the supplementary table codes 27 (Nielsen 2018) self, and on the CowScout Leg row 27 sits in the self column, so for P013 both sources agree on self. Appendix aims naming steps or walking: IceTag, IceQube, CowScout S.</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
         <is>
-          <t>As I004. Rule 4.2 split (15 October 2026): theoretically_measurable, as on I004: Maroto Molina found no sensor system for integument alterations and the only technology they cite was shown on human skin (Wei et al. 2018), not on cattle.</t>
+          <t>The keyword activity matches 39 aims. 28 of them name heat detection, and five are rumen boluses (eBolus, Moow Rumen bolus, smaXtec basic, smaXtec premium, VitalHerd). Only IceTag's aim names steps, and only IceTag, IceQube and CowScout S name walking; with the keywords step; walking the count would be 3. The count is reported as is and the keywords are visible. EFSA Table 31 rates on farm feasibility low; the appendix shows the opposite for the market. Table 1 also lists Lely activity (42, Elischer 2013, independent) but no appendix row is named Lely activity and no Lely row other than MQC-C carries a validation flag, so ref 42 is not attached to a product here. RumiWatch is not in products.csv and is cited as an appendix product. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. CowAlert IceQube (P016) names walking in its appendix aim, but Table 2 page 7 does not list it under Active behavior, so it is not among the products behind this grade.</t>
         </is>
       </c>
     </row>
@@ -2860,12 +2892,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>I006</t>
+          <t>I021</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Mastitis: Clinical cases</t>
+          <t>Metabolic disorders: Subclinical ketosis: individual cow milk constituents</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2881,7 +2913,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Mastitis</t>
+          <t>Subclinical ketosis</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2891,57 +2923,65 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>EFSA 2023, Table 27, PDF 43, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
+          <t>EFSA 2023, Table 46, PDF 75 to 76, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>AfiLab</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
+        </is>
+      </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Unclear: the written rules do not settle it (see open questions)</t>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Bausewein2022AMS</t>
+          <t>ICAR2025Brolis;Maker:brolis_herdline_home;Maker:brolis_herdline;Ponzo2026AMS;Maker:lely_astronaut_a5_next;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2023FPR</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Bausewein et al. 2022 tested the mastitis alerts of four makers' milking robots against a clinical udder examination of 7096 cows on 114 farms (sensitivity 61.4% to 78.2%, specificity 79.2% to 92.2%), with independent authors, though the makers advised on the alerts and supplied data. It detects cases at one visit, while EFSA's measure is the incidence rate of clinical mastitis, the same open question that keeps the 2021 grade unsure, so this grade is unsure too: validated_commercial if detection counts, otherwise theoretically_measurable. Listed in open_questions.md.</t>
+          <t>ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; Lely's page now sells the A5 Next, which it says builds on the A5, and does not claim this measurement, so this test is recorded but the grade rests on the ICAR test. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="T14" s="2" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
+          <t>Nothing extra: already in milk records or farm records</t>
         </is>
       </c>
       <c r="V14" s="2" t="inlineStr">
@@ -2950,21 +2990,21 @@
         </is>
       </c>
       <c r="W14" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): inspector checks farm records; Global Animal Partnership (US): inspector checks farm records; Certified Humane (US): inspector checks farm records</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="Z14" s="2" t="inlineStr">
-        <is>
-          <t>Yes: RSPCA Assured (UK), Global Animal Partnership (US), Certified Humane (US)</t>
         </is>
       </c>
       <c r="AA14" s="2" t="n">
@@ -2972,7 +3012,7 @@
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>0 + 2 + 3 + 1 + 2</t>
+          <t>3 + 3 + 1 + 1 + 0</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
@@ -2982,12 +3022,12 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7 lists Lely on line CMT (43) under Mastitis detection, commercial farm, lower performance column; Table 1 page 6 places 43 in the independent column. HerdInsight (30, Brassel et al. 2019, health disorder alarms) is listed under Health disorder (footnote d: e.g., mastitis or pneumonia) and its appendix aim names heat detection, health and feeding behaviour, not mastitis; under rules factor 1 a health disorder trait is not the same measure as clinical mastitis cases, so 30 does not count for I006. Appendix aims: FirstLook Mastitis system names mastitis identification; ten aims name udder health. Maroto Molina do not discuss clinical mastitis incidence (I006). Why Stygar's Lely on line CMT (43) is the appendix product MQC-C: in stygar_2021_supplementary.xlsx, sheet Appendix table 1, row 91, MQC-C (provider Lely) has sensor type milk quality sensors (conductivity, spectrometer, viscosity), aim milk yield and somatic cell count of each cow every 3 milkings, and validation flag yes. It is the only one of the six Lely rows (Qwes HR-LD, Lely Calm Compact +, Lely Calm Vario +, Cosmix, Astronaut A4, MQC-C) with a validation flag, and its viscosity sensor matches the sensor Table 1 page 6 gives for the Lely on line California mastitis test, a viscosity meter. MQC-C is an inline milk sensor fitted at the milking point, so its class is farm_fixed.</t>
+          <t>EFSA Table 46 page 75 defines the ABM as the individual milk fat to protein ratio or early lactation fat percentage monitored at routine milk recording. Stygar Table 2 page 7 lists AfiLab real time milk analyzer (25) under Milk quality, research farm, lower performance column; footnote e reads fat, lactose and protein as indicator for mastitis. Ref 25, Kaniyamattam and De Vries, agreement between milk fat, protein and lactose observations from DHIA and a real time milk analyzer, coded external independent validation in the supplementary study table. Appendix row AfiLab: milk quality sensors (spectrometer), aim milk composition analysis, monitoring general health and udder health, validation flag yes.</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
         <is>
-          <t>Candidates: validated_commercial, because Stygar validate mastitis detection (study 43) on a commercial farm; none, because the EFSA ABM is the incidence rate of clinical mastitis, not detection. Listed in open_questions.md. Device needed follows the unsure fill of rules.md rule 4.4: the cheapest class among the commercial candidates whose aim states the measurement. The records rule does not apply: EFSA Table 27 (PDF page 43) defines the measure as the incidence rate of clinical mastitis, and vet or farm records appear only in its feasibility line (high, although dependent on availability and accuracy of vet/farm records). The candidates are the 13 products whose aims match the search words, among them Lely MQC-C, the product behind study 43: milk quality sensors (AfiLab, DeLaval DCC and OCC, MQC-C, LIC Protrack SCC, SmartD-TECT Sensor), farm_fixed under rule 4.4 (an analyser at the milking point is one installation per parlour; DeLaval DCC, a cytometry camera whose appendix row does not place it at the milking point, is farm_fixed as a camera), and thermal cameras (Agricam CaDDi Mastitis, FirstLook Mastitis system, two Flir rows, Fluke IR FlexCam Pro, Smartis 336, WirisPro), also one device per farm. All are farm_fixed, so the class is farm_fixed. The routine_data class given on 2 October was withdrawn on 3 October (decision_log.md).</t>
+          <t>The measure is the same, individual cow milk fat and protein; Stygar record its validation as an indicator for mastitis, so the purpose differs and the note says so. The EFSA definition takes the value at routine milk recording, which the farm already has, so the class is routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser is the added device alternative, farm_fixed. Keyword fat and protein return 0 aims because the appendix describes these products as milk composition analysis.</t>
         </is>
       </c>
     </row>
@@ -2997,119 +3037,95 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>I008</t>
+          <t>I030</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Restriction of movement and resting problems: Step activity</t>
+          <t>Water provision</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>EFSA only</t>
+          <t>Welfare Quality only</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
+          <t>About the housing or equipment</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Restriction of movement (locomotion)</t>
+          <t>Absence of prolonged thirst</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Established input</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>EFSA 2023, Table 31, PDF 52, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+          <t>The Welfare Quality protocol v3.2 lists Water provision under the criterion Absence of prolonged thirst (overview, PDF 22, printed 21) as a resource based measure, about the housing or equipment. Graded by rule 4.14 from the measure type.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>Cow Manager; IceTag; RumiWatch; CowScout S</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>Active behavior (walking, no. of steps), Table 2 page 7, research and commercial farms, lower performance column for every product listed</t>
-        </is>
-      </c>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
-        </is>
-      </c>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>Charlton2022IceQube</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Charlton et al. 2022 tested step counts of the CowAlert IceQube, a commercial leg sensor, against live observation in three housing systems, with independent authors (step count agreement CCC 0.55 to 0.68 indoors, up to 0.93 at pasture on the back leg).</t>
+          <t>No source read since 2021 covers water points.</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="T15" s="2" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>One device per animal (collar, ear tag, bolus)</t>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
         </is>
       </c>
       <c r="V15" s="2" t="inlineStr">
         <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
+          <t>Named in FARM</t>
         </is>
       </c>
       <c r="W15" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: FARM v5 (US industry)</t>
         </is>
       </c>
       <c r="AA15" s="2" t="n">
@@ -3117,7 +3133,7 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>3 + 1 + 3 + 1 + 0</t>
+          <t>1 + 2 + 0 + 2 + 3</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -3127,12 +3143,12 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Active behavior (walking, no. of steps): every entry sits in the lower performance column, research farms CowManager SensOor (17, 39, 40), IceTag (28), Lely activity (42), RumiWatch (38), commercial farms CowScout Leg (27), IceTag (26, 27); page 6 text: for active behavior, lower performance of tools was reported. Table 1 page 6 columns: 39, 40, 28 and 26 independent; 17 and 38 self; on the IceTag row 21 and 26 to 28 sit in the independent column while the supplementary table codes 27 (Nielsen 2018) self, and on the CowScout Leg row 27 sits in the self column, so for P013 both sources agree on self. Appendix aims naming steps or walking: IceTag, IceQube, CowScout S.</t>
+          <t>Maroto Molina page 2: monitoring the number and status of water points has no relevance from a PLF perspective, since water consumption of every cow can be measured by a combination of RFID and flowmeters (Cardot et al. 2008), or indirectly by reticular temperature boluses. The Welfare Quality measure is the provision of water points, a resource measure, so this is a substitute measure and the grade is research_only under rules.md rule 4.2. Stygar Table 2 page 7 lists Insentec (45) under Water intake, research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation; the appendix row is Hokofarm Group RIC (Insentec, now Hokofarm), load cells and RFID, aim measures individual feed and water intake, flag yes.</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
         <is>
-          <t>The keyword activity matches 39 aims. 28 of them name heat detection, and five are rumen boluses (eBolus, Moow Rumen bolus, smaXtec basic, smaXtec premium, VitalHerd). Only IceTag's aim names steps, and only IceTag, IceQube and CowScout S name walking; with the keywords step; walking the count would be 3. The count is reported as is and the keywords are visible. EFSA Table 31 rates on farm feasibility low; the appendix shows the opposite for the market. Table 1 also lists Lely activity (42, Elischer 2013, independent) but no appendix row is named Lely activity and no Lely row other than MQC-C carries a validation flag, so ref 42 is not attached to a product here. RumiWatch is not in products.csv and is cited as an appendix product. IceTag is its own appendix row, separate from IceQube and CowAlert (P016), and is cited as an appendix product for the references Table 2 places against it. CowAlert IceQube (P016) names walking in its appendix aim, but Table 2 page 7 does not list it under Active behavior, so it is not among the products behind this grade.</t>
+          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water point measure. A study of the substitute does not demonstrate the indicator, even in cattle.</t>
         </is>
       </c>
     </row>
@@ -3142,119 +3158,95 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>I021</t>
+          <t>I031</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Metabolic disorders: Subclinical ketosis: individual cow milk constituents</t>
+          <t>Cleanliness of water points</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>EFSA only</t>
+          <t>Welfare Quality only</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Observed or recorded on the animal</t>
+          <t>About the housing or equipment</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Subclinical ketosis</t>
+          <t>Absence of prolonged thirst</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Established input</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>EFSA 2023, Table 46, PDF 75 to 76, lists it as an animal based measure. Graded by rule 4.14 from the measure type; EFSA's own ratings are in efsa_sensitivity, efsa_specificity and efsa_feasibility.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+          <t>The Welfare Quality protocol v3.2 lists Cleanliness of water points under the criterion Absence of prolonged thirst (overview, PDF 22, printed 21) as a resource based measure, about the housing or equipment. Graded by rule 4.14 from the measure type.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>AfiLab</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>Milk quality (fat, lactose and protein), Table 2 page 7, research farm, lower performance column</t>
-        </is>
-      </c>
+          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
-        </is>
-      </c>
-      <c r="Q16" s="2" t="inlineStr">
-        <is>
-          <t>ICAR2025Brolis;Maker:brolis_herdline_home;Maker:brolis_herdline;Ponzo2026AMS;Maker:lely_astronaut_a5_next;Maker:delaval_vms_v300;Maker:lemmer_fullwood_m2erlin;Antanaitis2023FPR</t>
-        </is>
-      </c>
+          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>ICAR's validation test of 26 June 2025 tested the Brolis BLH01 in line analyser, sold as Brolis HerdLine, for individual cow milk fat and protein at each milking against reference values (bias -0.002 to -0.08 g per 100 g, 105 measurements on each of two devices); the maker's home page offers it and calls it ICAR-validated. Ponzo et al. 2026 compared Lely Astronaut A5 fat and protein with official milk recording on five commercial farms (r 0.52 and 0.48), with Lely employees among the authors; Lely's page now sells the A5 Next, which it says builds on the A5, and does not claim this measurement, so this test is recorded but the grade rests on the ICAR test. As in the 2021 grade, the measure read is individual cow milk fat and protein, from which the ratio is computed. DeLaval and Lemmer-Fullwood pages also claim fat and protein for each cow.</t>
+          <t>No source read since 2021 covers water points.</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Proposed only</t>
         </is>
       </c>
       <c r="T16" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>Nothing extra: already in milk records or farm records</t>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
         </is>
       </c>
       <c r="V16" s="2" t="inlineStr">
         <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
+          <t>Named in FARM</t>
         </is>
       </c>
       <c r="W16" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: FARM v5 (US industry)</t>
         </is>
       </c>
       <c r="AA16" s="2" t="n">
@@ -3262,7 +3254,7 @@
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>3 + 3 + 1 + 1 + 0</t>
+          <t>1 + 2 + 0 + 2 + 3</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
@@ -3272,12 +3264,12 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>EFSA Table 46 page 75 defines the ABM as the individual milk fat to protein ratio or early lactation fat percentage monitored at routine milk recording. Stygar Table 2 page 7 lists AfiLab real time milk analyzer (25) under Milk quality, research farm, lower performance column; footnote e reads fat, lactose and protein as indicator for mastitis. Ref 25, Kaniyamattam and De Vries, agreement between milk fat, protein and lactose observations from DHIA and a real time milk analyzer, coded external independent validation in the supplementary study table. Appendix row AfiLab: milk quality sensors (spectrometer), aim milk composition analysis, monitoring general health and udder health, validation flag yes.</t>
+          <t>Welfare Quality PDF page 24 (printed 23): a resource based measure; the assessor checks the inner side of the bowl or trough for old or fresh dirt and staining of the water; clean when there is no evidence of crusts of dirt or decayed food residues. Maroto Molina page 2: as regards water quality, there are turbidity sensors able to measure water cleanliness, but it could be assumed to be adequate if water intake is normal. Keyword scan: 0 aims name turbidity, water quality or water cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: regarding the thirst criterion only resource based indicators are evaluated.</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
         <is>
-          <t>The measure is the same, individual cow milk fat and protein; Stygar record its validation as an indicator for mastitis, so the purpose differs and the note says so. The EFSA definition takes the value at routine milk recording, which the farm already has, so the class is routine_data under the records rule (rules.md rule 4.4, version 0.1.3); the inline analyser is the added device alternative, farm_fixed. Keyword fat and protein return 0 aims because the appendix describes these products as milk composition analysis.</t>
+          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina only propose turbidity sensors for water cleanliness and cite no study that used them at a water point.</t>
         </is>
       </c>
     </row>
@@ -3287,38 +3279,38 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>I030</t>
+          <t>I060</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Water provision</t>
+          <t>Rumination (sensor side)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality only</t>
+          <t>Sensor side only</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>About the housing or equipment</t>
+          <t>Observed or recorded on the animal</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Absence of prolonged thirst</t>
+          <t>Rumination</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Established input</t>
+          <t>Supported</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>The Welfare Quality protocol v3.2 lists Water provision under the criterion Absence of prolonged thirst (overview, PDF 22, printed 21) as a resource based measure, about the housing or equipment. Graded by rule 4.14 from the measure type.</t>
+          <t>Links: EFSA 2023, section 4.4.8 (PDF 74): cows fed fresh TMR on alternate days spent more time grooming themselves, "which, together with changes in the circadian variation in sleeping and lying ruminating, was interpreted as an indication of less disturbance and thus impaired welfare". Linstädt et al. 2024 (PDF 9): "As the Temperature-Humidity Index increased, feeding, rumination, and resting times decreased"; (PDF 8): lameness in high yield cows in an AMS "affects feeding, rumination, and AMS visits". No passage questions the link.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
@@ -3326,56 +3318,68 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr"/>
-      <c r="O17" s="2" t="inlineStr"/>
+          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Cow Manager; MooMonitor +; RumiWatch; SMARTBOW; Heatime HR LD (Hi-Tag)</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Rumination, Table 2 page 7: high performance on research farms for CowManager SensOor (17), MooMonitor+ (18, 29), RumiWatch (29, 33 to 35, 38), Smartbow (21) and Hi-Tag (31), and on commercial farms for RumiWatch (36) and a prototype (59); lower performance on research farms for CowManager SensOor (21, 39, 40) and Lely activity (42)</t>
+        </is>
+      </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr"/>
+          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Leso2021AfiCollar;Iqbal2021AfiCollar;Borchers2021Nedap;Pereira2021RumiWatch</t>
+        </is>
+      </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>No source read since 2021 covers water points.</t>
+          <t>Lee's dataset (lee_2025_dataset.xlsx, sheet Sifted articles, rows 28, 29, 36 and 37) lists four studies from 2021 that compared rumination from a named product with video: AfiCollar (Leso 2021, n 20; Iqbal 2021, n 48), Nedap SmartTag Neck (Borchers 2021, n 36) and RumiWatch (Pereira 2021, n 12). Lee Table 4 (PDF page 9) gives their precision, from CCC 0.86 with significant bias for Leso (rumination underestimated, Lee text PDF page 4) to CCC 0.93 to 0.98 for Borchers, and Lee Table 3 (PDF page 8) counts all three products among its commercial wearables. Borchers had maker funding, per the Europe PMC grant list recorded in step 3.</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Tested</t>
         </is>
       </c>
       <c r="T17" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>One device per animal (collar, ear tag, bolus)</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>FARM has only a related housing, equipment or practice rule</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U17" s="2" t="inlineStr">
-        <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
-        </is>
-      </c>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>Named in FARM</t>
-        </is>
-      </c>
-      <c r="W17" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="Z17" s="2" t="inlineStr">
-        <is>
-          <t>Yes: FARM v5 (US industry)</t>
         </is>
       </c>
       <c r="AA17" s="2" t="n">
@@ -3383,7 +3387,7 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 2 + 3</t>
+          <t>3 + 1 + 3 + 1 + 0</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
@@ -3393,12 +3397,12 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>Maroto Molina page 2: monitoring the number and status of water points has no relevance from a PLF perspective, since water consumption of every cow can be measured by a combination of RFID and flowmeters (Cardot et al. 2008), or indirectly by reticular temperature boluses. The Welfare Quality measure is the provision of water points, a resource measure, so this is a substitute measure and the grade is research_only under rules.md rule 4.2. Stygar Table 2 page 7 lists Insentec (45) under Water intake, research farm, high performance column; ref 45 Chapinal et al. 2007, external independent validation; the appendix row is Hokofarm Group RIC (Insentec, now Hokofarm), load cells and RFID, aim measures individual feed and water intake, flag yes.</t>
+          <t>Stygar Table 2 page 7, Rumination row, as in validated_trait. Table 1 page 6: independent validation for CowManager SensOor (21, 39 to 41), MooMonitor+ (18, 29), Smartbow (21), Hi-Tag (31, 32) and RumiWatch (34, 35); self validation for CowManager SensOor (17) and RumiWatch (29, 33, 36 to 38). Table 1 names Hi-Tag's provider SCR Engineers, currently Allflex; the Stygar list row is Allflex Heatime HR LD (Hi-Tag). Stygar list AIM column: 14 products name rumination (search word ruminat).</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
         <is>
-          <t>The substitute measure, individual water intake, has a validated commercial product, which the grade rule does not credit because the indicator as defined is the water point, not the intake. Recorded so the write up can say it. Class from the technology, a trough with RFID and flowmeter or load cells, farm_fixed. The keyword water alone matches one aim, Hokofarm RIC, whose aim is individual feed and water intake, the substitute measure, so it is not counted in vendors naming it, the same as on I031. Other technologies Maroto Molina (page 2) name for water intake: reticular temperature boluses, which they say would need data from weather stations or thermometers in water troughs because the rumen temperature drop is correlated to water temperature, and indoor radio based location (CowView, which they describe as commercialised by GEA). Both are animal_mounted. Their appendix rows (the bolus products; CowView, accelerometer collar, aim animal location) have aims that do not state water intake, so they do not set the class. Rule 4.2 split (15 October 2026): theoretically_measurable, because the sources offer only a substitute measure, individual water intake by RFID and flowmeters (Cardot et al. 2008), in place of the water point measure. A study of the substitute does not demonstrate the indicator, even in cattle.</t>
+          <t>Every product whose aim names rumination is an animal mounted collar, ear tag, leg tag or halter, so the class is animal_mounted. Lely activity (42) has no row in the Stygar list and is not cited as a product, as on I008 and I012.</t>
         </is>
       </c>
     </row>
@@ -3408,38 +3412,38 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>I031</t>
+          <t>I064</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Cleanliness of water points</t>
+          <t>Body temperature (sensor side)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality only</t>
+          <t>Sensor side only</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>About the housing or equipment</t>
+          <t>Observed or recorded on the animal</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Absence of prolonged thirst</t>
+          <t>Body temperature</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Established input</t>
+          <t>Supported</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>The Welfare Quality protocol v3.2 lists Cleanliness of water points under the criterion Absence of prolonged thirst (overview, PDF 22, printed 21) as a resource based measure, about the housing or equipment. Graded by rule 4.14 from the measure type.</t>
+          <t>Link: EFSA 2023, Table 26 (PDF 42), measures used for assessment of mastitis: severe clinical mastitis includes "systemic signs of illness such as apathy, anorexia, dehydration, or fever". No passage questions the link. Linstädt et al. 2024 (PDF 15) discusses nasal surface temperature and emotional state, a different parameter, not counted. Nasal temperature is excluded as a different parameter: Linstädt et al. 2024 (PDF 15) treat the temperature of the nose, a local skin temperature, as a sign of emotional state; the class counts the thermal cameras only for their claim to detect fever, a raised body temperature, not for local skin temperature.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -3447,56 +3451,60 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Proposed only: no product claims it; the sources only propose a method, report one shown in another species or setting, or offer a substitute measure</t>
+          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Nothing found in the sources read since 2021 (rules.md, rule 4.11)</t>
-        </is>
-      </c>
-      <c r="Q18" s="2" t="inlineStr"/>
+          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Maker:smaxtec_ph_bolus</t>
+        </is>
+      </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>No source read since 2021 covers water points.</t>
+          <t>The smaXtec page (maker_smaxtec_ph_bolus.txt) says the Classic Bolus continuously measures each cow's inner body temperature in the reticulum, to plus or minus 0.01 °C. No test of a product's body temperature against a reference since 2021 was found: the temperature rows from 2021 on in Lee's dataset are Arshad 2022 (row 17, a research GPS device, n 3) and Borghart 2021 (row 39, MooMonitor+, compared with lameness scoring, not with temperature).</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Proposed only</t>
+          <t>Claimed</t>
         </is>
       </c>
       <c r="T18" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>FARM has only a related housing, equipment or practice rule</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U18" s="2" t="inlineStr">
-        <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
-        </is>
-      </c>
-      <c r="V18" s="2" t="inlineStr">
-        <is>
-          <t>Named in FARM</t>
-        </is>
-      </c>
-      <c r="W18" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector looks at the animals; Global Animal Partnership (US): required, but the scheme does not say how it is checked; Certified Humane (US): required, but the scheme does not say how it is checked</t>
+          <t>No scheme requires it (4 of 4 read)</t>
         </is>
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="Z18" s="2" t="inlineStr">
-        <is>
-          <t>Yes: FARM v5 (US industry)</t>
         </is>
       </c>
       <c r="AA18" s="2" t="n">
@@ -3504,7 +3512,7 @@
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>1 + 2 + 0 + 2 + 3</t>
+          <t>2 + 2 + 3 + 1 + 0</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
@@ -3514,12 +3522,12 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>Welfare Quality PDF page 24 (printed 23): a resource based measure; the assessor checks the inner side of the bowl or trough for old or fresh dirt and staining of the water; clean when there is no evidence of crusts of dirt or decayed food residues. Maroto Molina page 2: as regards water quality, there are turbidity sensors able to measure water cleanliness, but it could be assumed to be adequate if water intake is normal. Keyword scan: 0 aims name turbidity, water quality or water cleanliness. Stygar Table 2 page 7 lists no such trait; page 10: regarding the thirst criterion only resource based indicators are evaluated.</t>
+          <t>Stygar Table 2 page 7, Body temperature: KB 3/04 bolus (52, Kahne Limited, New Zealand) and OPTRIS (55, Optris, Berlin), research farm, lower performance. Neither has a row in the Stygar list, so no product in the list has a coded study on this trait. Stygar list AIM column: 16 products name temperature, febrile responses or fever (search words in search_words); every one is marked on the Sensors x products sheet.</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
         <is>
-          <t>The technology named is a turbidity sensor in the water point, farm_fixed; nothing commercial in the appendix. The keyword water alone matches one aim, Hokofarm RIC, which measures water intake, not cleanliness, so it is not used. Maroto Molina's alternative, assuming cleanliness from normal intake, is an inference, not a measurement, and is not graded. Rule 4.2 split (15 October 2026): theoretically_measurable, because Maroto Molina only propose turbidity sensors for water cleanliness and cite no study that used them at a water point.</t>
+          <t>The cheapest commercial class is farm_fixed: five thermal cameras whose aims name fever. The other products are rumen boluses, ear tags and collars, animal_mounted. Rumen temperature and fever are counted as body temperature because the class is defined as the temperature of the cow's body however it is read; rule 4.2's trait rule then applies to this class as defined. CowManager's sensor type names a body temperature sensor, but its aim does not name temperature, so it is not counted.</t>
         </is>
       </c>
     </row>
@@ -3529,12 +3537,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>I060</t>
+          <t>I068</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Rumination (sensor side)</t>
+          <t>Oestrus (heat) detection (sensor side)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -3550,7 +3558,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Rumination</t>
+          <t>Oestrus (heat) detection</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -3560,7 +3568,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Links: EFSA 2023, section 4.4.8 (PDF 74): changes in "the circadian variation in sleeping and lying ruminating" in cows fed fresh TMR on alternate days were, with more self grooming, interpreted as an indication of impaired welfare. Linstädt et al. 2024 (PDF 9): "As the Temperature-Humidity Index increased, feeding, rumination, and resting times decreased"; (PDF 8): lameness in high yield cows in an AMS "affects feeding, rumination, and AMS visits". No passage questions the link.</t>
+          <t>Links: EFSA 2023, section 6.2.3 (PDF 99): "Tethering imposes severe restriction of movement ... it particularly restricts ... oestrus, calving and social behaviour"; Linstädt et al. 2024 (PDF 14): "Oestrus intensity was linked to good welfare"; (PDF 7): clinical lameness "has an effect on reproductive hormones and sexual behavior". No passage questions the link.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
@@ -3568,45 +3576,37 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product in the Stygar list was tested for this in a published study; the Answer sheet column 'What was tested, and how well' says how it did</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Cow Manager; MooMonitor +; RumiWatch; SMARTBOW; Heatime HR LD (Hi-Tag)</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>Rumination, Table 2 page 7: high performance on research farms for CowManager SensOor (17), MooMonitor+ (18, 29), RumiWatch (29, 33 to 35, 38), Smartbow (21) and Hi-Tag (31), and on commercial farms for RumiWatch (36) and a prototype (59); lower performance on research farms for CowManager SensOor (21, 39, 40) and Lely activity (42)</t>
-        </is>
-      </c>
+          <t>Claimed: a product's own description names it; Stygar 2021 coded no validation study</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Tested: a product on sale was tested against a reference method in a study since 2021 (see the sheet Evidence since 2021)</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Leso2021AfiCollar;Iqbal2021AfiCollar;Borchers2021Nedap;Pereira2021RumiWatch</t>
+          <t>Schilkowsky2021SmartBow;Maker:delaval_herd_navigator;Maker:smaxtec_ph_bolus;Maker:msd_sensehub_dairy;Maker:cowmed_smart_collar;Maker:peacock_ids_i_qube</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset (lee_2025_dataset.xlsx, sheet Sifted articles, rows 28, 29, 36 and 37) lists four studies from 2021 that compared rumination from a named product with video: AfiCollar (Leso 2021, n 20; Iqbal 2021, n 48), Nedap SmartTag Neck (Borchers 2021, n 36) and RumiWatch (Pereira 2021, n 12). Lee Table 4 (PDF page 9) gives their precision, from CCC 0.86 with significant bias for Leso (rumination underestimated, Lee text PDF page 4) to CCC 0.93 to 0.98 for Borchers, and Lee Table 3 (PDF page 8) counts all three products among its commercial wearables. Borchers had maker funding, per the Europe PMC grant list recorded in step 3.</t>
+          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, titled an evaluation of the estrus alerts of the SmartBow ear tag in 216 cows, compared with the HeatWatch System, another electronic system; the row codes the behaviours detected as physical activity and rumination time, and no result values are on disk. Rule 4.11 does not say whether another system is a reference method, and Lee (PDF page 2) gives a laboratory assay as the gold standard for oestrus. The maker pages of Herd Navigator, smaXtec, SenseHub, Cowmed and IDS i-QUBE claim heat or oestrus detection. Candidate readings: validated_commercial if the oestrus alerts and the HeatWatch comparison count, or commercial_unvalidated on the maker pages. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Tested</t>
+          <t>Claimed</t>
         </is>
       </c>
       <c r="T19" s="2" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>One device per animal (collar, ear tag, bolus)</t>
+          <t>One device per farm or barn (camera, scale, trough meter)</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>3 + 1 + 3 + 1 + 0</t>
+          <t>2 + 2 + 3 + 1 + 0</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
@@ -3647,12 +3647,12 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Rumination row, as in validated_trait. Table 1 page 6: independent validation for CowManager SensOor (21, 39 to 41), MooMonitor+ (18, 29), Smartbow (21), Hi-Tag (31, 32) and RumiWatch (34, 35); self validation for CowManager SensOor (17) and RumiWatch (29, 33, 36 to 38). Table 1 names Hi-Tag's provider SCR Engineers, currently Allflex; the Stygar list row is Allflex Heatime HR LD (Hi-Tag). Stygar list AIM column: 14 products name rumination (search word ruminat).</t>
+          <t>Stygar list AIM column: 31 products name heat (heat detection, or heat measurement for Herd Navigator), or progesterone (search words in search_words); every one is marked on the Sensors x products sheet. Stygar Table 2 page 7 has no oestrus trait, and rule 4.2 says activity is not oestrus.</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
         <is>
-          <t>Every product whose aim names rumination is an animal mounted collar, ear tag, leg tag or halter, so the class is animal_mounted. Lely activity (42) has no row in the Stygar list and is not cited as a product, as on I008 and I012.</t>
+          <t>The cheapest commercial class is farm_fixed: DeLaval Herd Navigator, a milk analyser at the milking point (rule 4.4, milk analysers), whose aim names progesterone and heat measurement. The other 30 products are animal mounted activity collars and tags.</t>
         </is>
       </c>
     </row>
@@ -3662,12 +3662,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>I064</t>
+          <t>I075</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Body temperature (sensor side)</t>
+          <t>Milk yield (sensor side)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -3683,17 +3683,17 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Body temperature</t>
+          <t>Milk yield</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Supported</t>
+          <t>Indirect or contested</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Link: EFSA 2023, Table 26 (PDF 42), measures used for assessment of mastitis: severe clinical mastitis includes "systemic signs of illness such as apathy, anorexia, dehydration, or fever". No passage questions the link. Linstädt et al. 2024 (PDF 15) discusses nasal surface temperature and emotional state, a different parameter, not counted.</t>
+          <t>Questions: Linstädt et al. 2024 (PDF 12): "relying solely on milk yield is insufficient for gauging the comprehensive welfare of the herd"; (PDF 1): "high milk production alone does not indicate good welfare"; EFSA 2023, section 5.7 (PDF 80): "there is no clear evidence that herd size or milk yield could be useful characteristics to identify farms at risk of poor welfare". Links as well: EFSA 2023, section 4.1.1.2 (PDF 30): cows with septic arthritis show "reduced milk yield"; Linstädt et al. 2024 (PDF 7): poor mobility is linked to lower milk yields. A question decides the grade (rule 4.14).</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -3713,12 +3713,12 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Maker:smaxtec_ph_bolus</t>
+          <t>Ponzo2026AMS;Bausewein2022AMS</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>The smaXtec page (maker_smaxtec_ph_bolus.txt) says the Classic Bolus continuously measures each cow's inner body temperature in the reticulum, to plus or minus 0.01 °C. No test of a product's body temperature against a reference since 2021 was found: the temperature rows from 2021 on in Lee's dataset are Arshad 2022 (row 17, a research GPS device, n 3) and Borghart 2021 (row 39, MooMonitor+, compared with lameness scoring, not with temperature).</t>
+          <t>Bausewein 2022 (ev_bausewein2022ams.xml) says the commercially available sensor systems in automatic milking systems provide milk yield. Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records, with two Lely employees among the authors; but no source since 2021 says the Astronaut A5 is on sale (Lely's page sells the Astronaut A5 Next), so, as for fat and protein on I021 and I025, the test is recorded and the grade is commercial_unvalidated.</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
@@ -3727,16 +3727,16 @@
         </is>
       </c>
       <c r="T20" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>One device per farm or barn (camera, scale, trough meter)</t>
+          <t>Nothing extra: already in milk records or farm records</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
         <is>
-          <t>FARM has only a related housing, equipment or practice rule</t>
+          <t>Not named in FARM</t>
         </is>
       </c>
       <c r="W20" s="2" t="n">
@@ -3744,17 +3744,17 @@
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>No scheme requires it (4 of 4 read)</t>
+          <t>No scheme requires it (4 of 4 read); unclear whether RSPCA Assured (UK), Certified Humane (US) requires it</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear: whether RSPCA Assured (UK), Certified Humane (US) requires it (see open questions)</t>
         </is>
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unclear: whether RSPCA Assured (UK), Certified Humane (US) requires it (see open questions)</t>
         </is>
       </c>
       <c r="AA20" s="2" t="n">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>2 + 2 + 3 + 1 + 0</t>
+          <t>2 + 3 + 3 + 0 + 0</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>Stygar Table 2 page 7, Body temperature: KB 3/04 bolus (52, Kahne Limited, New Zealand) and OPTRIS (55, Optris, Berlin), research farm, lower performance. Neither has a row in the Stygar list, so no product in the list has a coded study on this trait. Stygar list AIM column: 16 products name temperature, febrile responses or fever (search words in search_words); every one is marked on the Sensors x products sheet.</t>
+          <t>Stygar list AIM column: 13 milking robots, aim monitor and analyse the milk production performance; Lely MQC-C, Milk yield and somatic cells count; LIC Saber Milk, Milk yield, composition and conductivity. Stygar Table 2 page 7 has no milk yield trait. ICAR's list of validated sensor systems (1_sources/icar_validated_sensors.html) names the Panazoo MMI sensor (P020) for milk yield; it is not in the Stygar list, so it does not change this grade.</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
         <is>
-          <t>The cheapest commercial class is farm_fixed: five thermal cameras whose aims name fever. The other products are rumen boluses, ear tags and collars, animal_mounted. Rumen temperature and fever are counted as body temperature because the class is defined as the temperature of the cow's body however it is read; rule 4.2's trait rule then applies to this class as defined. CowManager's sensor type names a body temperature sensor, but its aim does not name temperature, so it is not counted.</t>
+          <t>Rule 4.4 lists milk yield under routine_data, a value the milking system already collects with no new device, and the milking robots' aims say they monitor milk production.</t>
         </is>
       </c>
     </row>
@@ -5945,12 +5945,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>No welfare validation</t>
+          <t>Supported</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>The three sources were searched (EFSA 2023, Welfare Quality v3.2, Linstädt et al. 2024) and none links it to welfare in its own words. The five thermal camera aims say they are "to detect inflammation, fever… Udder health or lamenesse", and inflammation is itself a condition, so a product frames it as about health.</t>
+          <t>Links: EFSA 2023, section 4.1.1 (PDF 29): "Tissue damage and associated inflammation lead to the stimulation of nociceptors and release of e.g. pain mediators"; section 4.2.1 (PDF 42): mastitis is a disease characterised by inflammation of the mammary gland. No passage questions the link. The five thermal camera aims also say they are "to detect inflammation, fever… Udder health or lamenesse".</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Spadola 2026 (ev_spadola2026irt.xml) imaged the hind feet of 15 cows with a FLIR ThermaCam P25 and found higher foot surface temperatures in cows with foot lesions than in healthy cows, and Hudson 2026 (section 3.2.3) says such increases 'may reflect inflammation', while its Table 2 lists no thermography study reporting accuracy. Neither source tests the camera against a reference for inflammation, and the existing record calls the temperature a substitute for the lesions. Candidate readings: research_demonstrated if foot temperature in lesioned cows counts as inflammation found by thermal imaging, theoretically_measurable if it is a substitute.</t>
+          <t>Spadola 2026 (ev_spadola2026irt.xml) imaged the hind feet of 15 cows with a FLIR ThermaCam P25 and found higher foot surface temperatures in cows with foot lesions than in healthy cows; its stated aim includes assessing "the evolution of inflammation over time", and its abstract ties higher temperatures to inflamed areas alongside systemic inflammatory markers, and Hudson 2026 (section 3.2.3) says such increases 'may reflect inflammation', while its Table 2 lists no thermography study reporting accuracy. Neither source tests the camera against a reference for inflammation, and the existing record calls the temperature a substitute for the lesions. Candidate readings: research_demonstrated if foot temperature in lesioned cows counts as inflammation found by thermal imaging, theoretically_measurable if it is a substitute.</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
@@ -6070,12 +6070,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Not framed as welfare</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>The three sources were searched (EFSA 2023, Welfare Quality v3.2, Linstädt et al. 2024) and none links it to welfare in its own words. EFSA 2023 names GPS only as one way to measure walking speed (Table 31, PDF 52), a different parameter. No product aim says location is for health or welfare: they name it for herd management, herd counting, theft alerts or a virtual fence, or list it beside other functions. No scheme requires it.</t>
+          <t>Unsure under rule 4.14. The three sources were searched (EFSA 2023, Welfare Quality v3.2, Linstädt et al. 2024) and none links location to welfare in its own words; EFSA names GPS only as a way to measure locomotor activity and walking speed (PDF 51 and Table 31, PDF 52), a different parameter. No scheme requires it. The grade turns on one product aim: GEA CowView, "Animal location for big herds gestion, Health and Fertility Management". Read one way, location is for herd management and health and fertility management are separate functions, so no aim says location is for health and the row is not_welfare_relevant; read the other way, the aim offers location for health management, so it is no_welfare_validation. The other aims name location for herd counting, theft alerts or a virtual fence, or list it beside other functions. See open_questions.md.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -7466,12 +7466,12 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>Maker:smaxtec_ph_bolus;Pfeiffer2021tail</t>
+          <t>Maker:smaxtec_ph_bolus</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>The smaXtec page (maker_smaxtec_ph_bolus.txt) lists calving detection for both boluses. Pfeiffer 2021 (Lee dataset row 32, full text read from the step 3 copy) used the Moocall and CalveSense tail sensors for early calving detection and calls them commercially available, but tested only cow behaviour after attaching them, not calving detection against a reference.</t>
+          <t>The smaXtec page (maker_smaxtec_ph_bolus.txt) lists calving detection for both boluses. No study since 2021 on disk tests calving detection by a product against a reference.</t>
         </is>
       </c>
       <c r="S49" s="2" t="inlineStr">
@@ -7566,12 +7566,12 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Indirect or contested</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Questions: Linstädt et al. 2024 (PDF 16): "Precision Livestock Farming offers real-time welfare assessment, but validation is important."; (PDF 12): PLF technologies "currently have limited potential for assessing appropriate behavior in dairy cows, necessitating further validation studies". Link as well: Linstädt et al. 2024 (PDF 8): combining automatic indicators "offers the potential for an early warning system in addressing welfare problems". A question decides the grade (rule 4.14).</t>
+          <t>Unsure under rule 4.14. Link: Linstädt et al. 2024 (PDF 8): combining automatic indicators "offers the potential for an early warning system in addressing welfare problems". Possible questions: Linstädt et al. 2024 (PDF 16): "Precision Livestock Farming offers real-time welfare assessment, but validation is important."; (PDF 12): PLF technologies "currently have limited potential for assessing appropriate behavior in dairy cows, necessitating further validation studies". These two say that sensor based welfare assessment still needs validation; they do not use rule 4.14's words for a question (indirect, insufficient on its own, weak, inconsistent, unclear or not fully understood), and validation of a technology belongs to column (a), but the parameter is itself a sensor based welfare assessment. Candidate readings: supported (the PDF 8 link, with no question) or indirect_or_contested (the validation passages as questions). See open_questions.md.</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -13283,7 +13283,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>No welfare validation</t>
+          <t>Supported</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Not framed as welfare</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -13438,7 +13438,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>I068 Tested</t>
+          <t>I068 Claimed</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Indirect or contested</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>I075 Tested</t>
+          <t>I075 Claimed</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -16584,6 +16584,11 @@
           <t>named</t>
         </is>
       </c>
+      <c r="CB62" s="6" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
       <c r="CH62" s="6" t="inlineStr">
         <is>
           <t>validated</t>
@@ -21503,7 +21508,7 @@
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Searched for rumination, ruminat, cud and chewing. No standard names rumination or rumination time. The word appears only in the rationale of the resting area standard, "Cattle have increased lying time in well-bedded environments, which reduces the risk for lameness, improves rumination, production, and health outcomes." (Chapter 3, Resting Areas, PDF 44), and in reference titles about calves (PDF 31 and PDF 101). Rationale text is not a standard (rule 2). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), a housing provision that does not name an animal measure (rule 10).</t>
+          <t>Searched for rumination, ruminat, cud and chewing. No standard names rumination or rumination time. The word appears only in the rationale of the resting area standard, "Cattle have increased lying time in well-bedded environments, which reduces the risk for lameness, improves rumination, production, and health outcomes." (Chapter 3, Resting Areas, PDF 44), and in reference titles about calves (PDF 31, PDF 93 and PDF 101). Rationale text is not a standard (rule 2). Related requirement: "All age classes of animals have a resting area that is clean, dry, provides adequate cushion at all times, and does not pose risk of injury." (Chapter 3, Resting Areas, PDF 44), a housing provision that does not name an animal measure (rule 10).</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -21570,7 +21575,7 @@
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Searched for feeding behaviour, feeding time, feeding duration, eating, grazing and graze. No standard names how long or when a cow feeds or grazes. Related: 6.B.23, all Steps (PDF 40, printed 30), "Feed must be available to all cows for at least 18 hours each day.", a provision of feed, so under rule 10 it does not name the cow's feeding time (it bears on feed availability, I080). Info notes 6.B.8b (PDF 39, printed 29) and 6.B.18b (PDF 40, printed 30) mention feeding time and feeding behaviour of Calves and Heifers as research background; they are guidance (rule 2) and other animals (rule 6). Info notes 4.A.1 and 4.A.2 (PDF 26, printed 16) say observation can take place during feeding, which is general observation, not a feeding measure. Pasture time for lactating cows, 8.W.2 and 8.W.3 (PDF 53, printed 43), is marked only at Steps 4 to 5+, so it is not counted (rule 14), and it is time on Pasture, not grazing time.</t>
+          <t>Searched for feeding behaviour, feeding time, feeding duration, eating, grazing and graze. No standard names how long or when a cow feeds or grazes. Related: 6.B.23, all Steps (PDF 40, printed 30), "Feed must be available to all cows for at least 18 hours each day.", a provision of feed, so under rule 10 it does not name the cow's feeding time (it bears on feed availability, I080). Info notes 6.B.8b (PDF 39, printed 29) and 6.B.18b (PDF 40, printed 30) mention feeding time and feeding behaviour of Calves and Heifers as research background; they are guidance (rule 2) and other animals (rule 6). Info notes 4.A.1 and 4.A.2 (PDF 26, printed 16) say observation can take place during feeding, which is general observation, not a feeding measure. Pasture time for lactating cows, 8.W.2, Steps 4 to 5+, and 8.W.3, Steps 4 and 5 (PDF 53, printed 43), is not counted (rule 14), and it is time on Pasture, not grazing time.</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -21671,7 +21676,7 @@
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Searched for water intake, drink, intake and water. No standard names the amount of water each cow drinks. Related requirement: "Apart from pre-weaned calves, all other age classes of animals have access to clean water appropriate for climatic conditions." (Chapter 3, Access to Water, PDF 30), which names water provision (row I030) and is a provision for this row under rule 10; it sets no amount per animal. Water intake appears only in the rationale and reference titles (PDF 30 and PDF 31). For pre-weaned calves, access to water by day 3 (Chapter 5, PDF 91) is a provision and other animals (rule 6). Non-ambulatory animals are provided access to water (Chapter 6, PDF 116), also a provision.</t>
+          <t>Searched for water intake, drink, intake and water. No standard names the amount of water each cow drinks. Related requirement: "Apart from pre-weaned calves, all other age classes of animals have access to clean water appropriate for climatic conditions." (Chapter 3, Access to Water, PDF 30), which names water provision (row I030) and is a provision for this row under rule 10; it sets no amount per animal. Water intake appears only in the rationale and reference titles (PDF 30, PDF 31 and PDF 93). For pre-weaned calves, access to water by day 3 (Chapter 5, PDF 91) is a provision and other animals (rule 6). Non-ambulatory animals are provided access to water (Chapter 6, PDF 116), also a provision.</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -21884,7 +21889,7 @@
       <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "Managers must: e) develop and implement a transport plan to a slaughterhouse which: i. includes a method of identification of animals (see standard M 5.2)" (M 2.3 e) i., PDF 31 (printed 29)). Candidate: M 2.3 e) i. requires every farm's transport plan to a slaughterhouse to include a method of identification of animals. Reading one: animal identification is a management measure, and under rule 7 a requirement that names a management measure names it; the plan applies to every certified farm, so the row is required. Reading two: the requirement names identification only within a transport plan for animals going to slaughter, not identification of every animal on the farm, so it is narrower than the row and under rule 6 is not a direct synonym. Rules 6 and 7 do not settle whether identification for a stated purpose, or of a subset of animals, names the row. Other candidates of the same kind: H 1.1 f) (PDF 44, printed 42), the VHWP must include an effective procedure for identifying animals that are undergoing or have undergone treatment; H 5.5 (PDF 51, printed 49), any cows with mastitis must be marked and milked last; H 5.3 (PDF 51, printed 49), cows with chronic mastitis must be identified and humanely slaughtered, where identified means found to have the condition. Related and not counted: M 6.1 (PDF 35, printed 33), neckbands, tailbands or legbands must only be used for identification purposes and fitted with care, and M 6.2, marking done with care by trained operators; both govern how marking is done and do not require that animals be identified. The information box after M 6.2 (PDF 35, printed 33) says ear tagging as approved by Defra is a legal requirement and names implanted electronic transponders as acceptable; a box is not a standard (rule 2). The cross reference in M 2.3 e) i. to M 5.2 points to the standard on animal handler training. how_checked is left empty: no RSPCA text says how the method of identification is checked.</t>
+          <t>Candidate: "Managers must: ... e) develop and implement a transport plan to a slaughterhouse which: i. includes a method of identification of animals (see standard M 5.2)" (M 2.3 e) i., PDF 31 (printed 29)). Candidate: M 2.3 e) i. requires every farm's transport plan to a slaughterhouse to include a method of identification of animals. Reading one: animal identification is a management measure, and under rule 7 a requirement that names a management measure names it; the plan applies to every certified farm, so the row is required. Reading two: the requirement names identification only within a transport plan for animals going to slaughter, not identification of every animal on the farm, so it is narrower than the row and under rule 6 is not a direct synonym. Rules 6 and 7 do not settle whether identification for a stated purpose, or of a subset of animals, names the row. Other candidates of the same kind: H 1.1 f) (PDF 44, printed 42), the VHWP must include an effective procedure for identifying animals that are undergoing or have undergone treatment; H 5.5 (PDF 51, printed 49), any cows with mastitis must be marked and milked last; H 5.3 (PDF 51, printed 49), cows with chronic mastitis must be identified and humanely slaughtered, where identified means found to have the condition. Related and not counted: M 6.1 (PDF 35, printed 33), neckbands, tailbands or legbands must only be used for identification purposes and fitted with care, and M 6.2, marking done with care by trained operators; both govern how marking is done and do not require that animals be identified. The information box after M 6.2 (PDF 35, printed 33) says ear tagging as approved by Defra is a legal requirement and names implanted electronic transponders as acceptable; a box is not a standard (rule 2). The cross reference in M 2.3 e) i. to M 5.2 points to the standard on animal handler training. how_checked is left empty: no RSPCA text says how the method of identification is checked.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -22483,7 +22488,7 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Searched for blood, bloody, abnormal milk, clots and forestrip. No standard names blood in milk. Blood appears only as a calf blood sample for testing passive immunity (Chapter 5, PDF 88) and in euthanasia text (Chapter 7, PDF 127). The nearest standards are the milking procedures protocol (Chapter 4, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56); FARM's text does not tie either to blood in milk.</t>
+          <t>Searched for blood, bloody, abnormal milk, clots and forestrip. No standard names blood in milk. Blood appears only as a calf blood sample for testing passive immunity (Chapter 5, PDF 88) in euthanasia text (Chapter 7, PDF 127), and as blood flow in science and guidance text (Chapter 3, PDF 36; Chapter 6, PDF 112). The nearest standards are the milking procedures protocol (Chapter 4, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56); FARM's text does not tie either to blood in milk.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -22494,7 +22499,7 @@
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Searched for blood, bloody, abnormal milk and fore milk. "Blood" appears only in "Bloodless" castration tools (PDF 32, printed 22; PDF 95 and 97). No numbered requirement names blood in milk. Related: 7.D.2, all Steps (PDF 42, printed 32), each cow checked for symptoms of clinical mastitis at each milking with records if found, which names clinical mastitis (row I006), not blood in milk (rule 6); its info note mentions examining "fore milk" (guidance, rule 2).</t>
+          <t>Searched for blood, bloody, abnormal milk and fore milk. "Blood" appears only in "Bloodless" castration tools (PDF 32, printed 22; PDF 95 and 97, printed 85 and 87). No numbered requirement names blood in milk. Related: 7.D.2, all Steps (PDF 42, printed 32), each cow checked for symptoms of clinical mastitis at each milking with records if found, which names clinical mastitis (row I006), not blood in milk (rule 6); its info note mentions examining "fore milk" (guidance, rule 2).</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -22689,7 +22694,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>"The feed itself must be pushed up regularly to ensure additional ease of access to feed." (FW 9 c, PDF 13 (printed 4))</t>
+          <t>"Cattle must have free access to nutritious food each day, except when directed otherwise by an attending veterinarian." (FW 2, PDF 11 (printed 2))</t>
         </is>
       </c>
     </row>
@@ -22716,7 +22721,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "The following health and welfare conditions, where applicable to the unit, must be listed in the VHWP (see standard H 1.4): a) metabolic disorders (hypocalcaemia, hypomagnesaemia, ketosis, displaced abomasum, bloat, acidosis)" (H 1.5 a), PDF 45 (printed 43)). Candidate: H 1.5 a) lists acidosis among the metabolic disorders the VHWP must list, and under H 1.4 (PDF 45, printed 43) the level of each condition is recorded, thresholded and monitored, a record of cases under rule 11. Reading one: acidosis named without its form names the condition row, as ketosis in the same clause names I020 under rule 5, so this row is required. Reading two: this row is defined as rumen acidosis including subacute ruminal acidosis (SARA), the form the sensor products detect, and rule 5 says a condition named without its form never names a subclinical row; rule 5 does not say whether a row that joins the condition with its subacute form counts as the clinical case row. Rule 6 also does not settle whether acidosis, without the word rumen, is a direct synonym of rumen acidosis. So the row is unsure. how_checked is records_review if counted: the condition is listed, recorded and monitored in the VHWP, a farm record, as in the I020 row. Rule 4 check as in I020: where applicable to the unit follows whether the condition occurs on the farm. Searched: acidosis, SARA, rumen, ruminal, subacute. related_resource: FW 1.7, fibre of such quality and length as to help avoid acidosis (PDF 7, printed 5); E 8.2 d), provisions before turnout so the risk of acidosis and bloat is minimised (PDF 24, printed 22). The test rows I025, I026 and I027 are not_required.</t>
+          <t>Candidate: "The following health and welfare conditions, where applicable to the unit, must be listed in the VHWP (see standard H 1.4): a) metabolic disorders (hypocalcaemia, hypomagnesaemia, ketosis, displaced abomasum, bloat, acidosis)" (H 1.5 a), PDF 45 (printed 43)). Candidate: H 1.5 a) lists acidosis among the metabolic disorders the VHWP must list, and under H 1.4 (PDF 45, printed 43) the level of each condition is recorded, thresholded and monitored, a record of cases under rule 11. Reading one: acidosis named without its form names the condition row, as ketosis in the same clause names I020 under rule 5, so this row is required. Reading two: the row's welfare_state is subacute ruminal acidosis (SARA), and one of its products names SARA detection, although its definition is rumen acidosis as a condition; and rule 5 says a condition named without its form never names a subclinical row; rule 5 does not say whether a row that joins the condition with its subacute form counts as the clinical case row. Rule 6 also does not settle whether acidosis, without the word rumen, is a direct synonym of rumen acidosis. So the row is unsure. how_checked is records_review if counted: the condition is listed, recorded and monitored in the VHWP, a farm record, as in the I020 row. Rule 4 check as in I020: where applicable to the unit follows whether the condition occurs on the farm. Searched: acidosis, SARA, rumen, ruminal, subacute. related_resource: FW 1.7, fibre of such quality and length as to help avoid acidosis (PDF 7, printed 5); E 8.2 d), provisions before turnout so the risk of acidosis and bloat is minimised (PDF 24, printed 22). The test rows I025, I026 and I027 are not_required.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -22749,7 +22754,7 @@
       <c r="M81" s="2" t="inlineStr"/>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "The herd must be continually monitored for performance, including production diseases, infectious diseases, and injury as a result of housing/husbandry/handling, such as: 1. Metabolic Disorders (e.g., hypocalcemia, hypomagnesemia, ketosis, displaced abomasum, laminitis, bloat, acidosis, etc.)" (H 1 a 1, PDF 34 (printed 25)). Searched for acidosis, SARA, rumen, ruminal and pH. H 1 a 1 names acidosis, without its form, among the conditions the herd must be continually monitored for. It applies to every farm. Read one way, I081 is the condition row for rumen acidosis, and monitoring cases of a named condition names its case measure (rules 5 and 11), as H 1 a 1 does for ketosis on I020 and hypocalcemia on I028, so the row is required. Read the other way, I081 is defined as subacute ruminal acidosis, a subacute form, and rule 5 says a condition named without its form never names a subclinical row, as on I029, so the row is not_required; acidosis is also not qualified as ruminal. Rule 5 does not say whether a subacute condition row with no test in its definition is a clinical case row or a subclinical row, so the rules do not settle it. how_checked is left empty: no numbered requirement says the monitored cases are recorded or how the inspector checks them, as on the I020 row. Related: FW 7 b forage of the appropriate quality and length to stimulate rumination and prevent acidosis (PDF 12, printed 3), a feed provision that states its intended outcome (rule 10); the I025 and I027 rows already read these passages as naming the condition without the test. The box under H 5 on sub-clinical rumen acidosis (PDF 36, printed 27) does not count (rule 2).</t>
+          <t>Candidate: "The herd must be continually monitored for performance, including production diseases, infectious diseases, and injury as a result of housing/husbandry/handling, such as: 1. Metabolic Disorders (e.g., hypocalcemia, hypomagnesemia, ketosis, displaced abomasum, laminitis, bloat, acidosis, etc.)" (H 1 a 1, PDF 34 (printed 25)). Searched for acidosis, SARA, rumen, ruminal and pH. H 1 a 1 names acidosis, without its form, among the conditions the herd must be continually monitored for. It applies to every farm. Read one way, I081 is the condition row for rumen acidosis, and monitoring cases of a named condition names its case measure (rules 5 and 11), as H 1 a 1 does for ketosis on I020 and hypocalcemia on I028, so the row is required. Read the other way, the row's welfare_state is subacute ruminal acidosis, a subacute form (its definition is rumen acidosis as a condition), and rule 5 says a condition named without its form never names a subclinical row, as on I029, so the row is not_required; acidosis is also not qualified as ruminal. Rule 5 does not say whether a subacute condition row with no test in its definition is a clinical case row or a subclinical row, so the rules do not settle it. how_checked is left empty: no numbered requirement says the monitored cases are recorded or how the inspector checks them, as on the I020 row. Related: FW 7 b forage of the appropriate quality and length to stimulate rumination and prevent acidosis (PDF 12, printed 3), a feed provision that states its intended outcome (rule 10); the I025 and I027 rows already read these passages as naming the condition without the test. The box under H 5 on sub-clinical rumen acidosis (PDF 36, printed 27) does not count (rule 2).</t>
         </is>
       </c>
     </row>
@@ -22766,44 +22771,40 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Candidate: "In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73)). Unsure. The row's animals are unweaned calves, so a calf milk standard is in the row's own animals (rule 6). FW(C) 1.3.1 a) sets the amount of milk or milk replacer each calf must be offered per day, which is the milk given to each calf that the row records, a management measure, and rule 7 counts a requirement that names a management measure. The box below it says there is no requirement for calves to consume the full quantities; it is guidance (rule 2), and it confirms the standard is about the milk given, not the milk drunk. FW(C) 1.3.1 b) adds "across at least two feeds per day for the first 42 days of life". On rule 4: the calf standards are to be used by anyone rearing calves on an assured unit (PDF 74, printed 72), but FW(C) 1.3.1 is limited to calves no longer with their dam after 24 hours, and the standards also provide for calves that stay with the dam (FW(C) 1.3 b) i., PDF 74, printed 72; FW(C) 1.6, all non-suckled calves, PDF 76, printed 74; FW(C) 1.18, artificially reared calves, PDF 77, printed 75). Reading one: it applies to every certified farm that rears calves apart from the dam, and that condition is the practice the row itself measures, so the row is required. Reading two: it is limited to one rearing system, which rule 4 does not count, so not_required. Rule 4 does not say whether a condition that is the row's own practice limits a requirement, so the row is unsure. how_checked is left empty: no RSPCA text says how the milk offered is checked. Related: FW(C) 1.6, all non-suckled calves must receive liquid food daily for at least the first eight weeks and until eating at least 1.5kg dry matter per day of a calf starter ration, and FW(C) 1.6.1, abrupt weaning not permitted (PDF 76, printed 74); FW(C) 1.3 a), at least 3 litres of colostrum within the first 6 hours (PDF 74, printed 72), colostrum rather than milk or milk replacer; FW(C) 1.1 b), a diet fed in sufficient quantity (PDF 74, printed 72), broader wording (rule 6); FW(C) 1.17.1, where calves are fed by an ad-lib automated system the producer must show there is no competition that may limit intake, and FW(C) 1.20, where calves are rationed by transponder the feed station must let all calves drink without hindrance (PDF 77, printed 75), provisions limited to farms with those systems (rules 10 and 4); FW(C) 1.18, milk feeds through teat feeders for artificially reared calves (PDF 77, printed 75), an equipment provision (rule 10).</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>inspector checks farm records</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>"The Herd Health Plan (HHP) has a written protocol for pre-weaned calf care that includes language specific to all pre-weaned calves (heifers, bulls, and steers) receiving a volume and quality of milk or milk replacer to maintain health, growth, and vigor until weaned or marketed." (Chapter 5: Pre-Weaned Calves, Milk Feeding, PDF 94 (printed 94))</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
         <is>
           <t>required, but the scheme does not say how it is checked</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>"In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73))</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>inspector checks farm records</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>"The Herd Health Plan (HHP) has a written protocol for pre-weaned calf care that includes language specific to all pre-weaned calves (heifers, bulls, and steers) receiving a volume and quality of milk or milk replacer to maintain health, growth, and vigor until weaned or marketed." (Chapter 5: Pre-Weaned Calves, Milk Feeding, PDF 94 (printed 94))</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>required, but the scheme does not say how it is checked</t>
-        </is>
-      </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
           <t>"From day 1 until 8 weeks of age, Calves must be offered approximately 20% of their current body weight in milk or milk replacer each day." (6.B.1 (Feeding Requirements, Unweaned Calves), PDF 38 (printed 28))</t>
@@ -22811,17 +22812,13 @@
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="M82" s="2" t="inlineStr">
-        <is>
-          <t>required, but the scheme does not say how it is checked</t>
-        </is>
-      </c>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr"/>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>"All calves must receive milk or milk replacer at least twice daily through the first five weeks of life." (FW 14 a, PDF 14 (printed 5))</t>
+          <t>Candidate: "All calves must receive milk or milk replacer at least twice daily through the first five weeks of life." (FW 14 a, PDF 14 (printed 5)). Unsure. The row's animals are unweaned calves, so the calf standards in Part 2 B, Food, Specific Provisions for Calves, are in the row's own animals (rule 6). FW 14 a requires that every calf receive milk or milk replacer, with a frequency and a period, and it applies to all calves on every farm (rule 4). Reading one: it names the milk given to each calf, a management measure that rule 7 counts, so the row is required. Reading two: it sets only how often milk is fed, with no amount, while the row is the amount each calf is given and the feeder records; as on the I062 rows, a feeding requirement with no amount for each animal does not name the amount, so not_required. Rules 6, 7 and 13 do not settle whether a frequency without an amount names the measure, so the row is unsure. It sets no volume; the only volume, a daily ration of at least 20% of body weight (approximately 8 liters for larger breeds like Holstein calves) for calves aged 3 to 28 days, is in the recommendation below FW 12 (PDF 13 and 14, printed 4 and 5), which does not count (rule 2). FW 13 c (PDF 14, printed 5) also names it: "Twice per day over the subsequent 48 hours, calves must receive additional colostrum or whole milk in an amount that is breed and size appropriate." how_checked is left empty: no numbered requirement says how milk feeding is checked. Related (all PDF 14, printed 5): FW 14 e, milk replacer mixed according to the manufacturer's instructions; FW 14 b, an individual bucket for each calf where calves are bucket fed, limited to bucket feeding (rules 10 and 4); FW 14 f, calves not weaned until eating at least 1.5 lbs. (680 g) per calf per day of calf starter, which is feed, not milk; FW 15 a, weaning by diluting the milk or reducing the milk volume over at least 5 days; FW 13 a and b, colostrum within the first 6 hours and at least 2 quarts in two feedings within 12 h when the calf has not nursed, colostrum rather than milk, and b only when the calf has not nursed (rule 4).</t>
         </is>
       </c>
     </row>
@@ -31403,7 +31400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -32232,7 +32229,7 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019.</t>
+          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019. Used for I082 only for section 2.1's statement that an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan; it gives no amount and no sale status for the feeder.</t>
         </is>
       </c>
     </row>
@@ -33606,7 +33603,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>somatic cell count recorded by AMS</t>
+          <t>somatic cell count recorded by AMS; daily milk yield, AMS against same day official milk recording (OMR)</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -33616,7 +33613,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>correlation AMS vs official milk recording: somatic cell count (r = 0.62); milk yield r = 0.93, fat r = 0.52, protein r = 0.48</t>
+          <t>correlation AMS vs official milk recording: somatic cell count (r = 0.62); milk yield r = 0.93, fat r = 0.52, protein r = 0.48; Table 2: milk yield r = 0.931 (dataset 3, 19,488 observations from 1982 cows)</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
@@ -33636,7 +33633,7 @@
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
-          <t>COI: 'Fernando Masia and Elisa Vrieze are employed by the company Lely International N.V.' Text says AMS 'could also be equipped with sensors performing somatic cell count' and that external calibration data were not entered on these farms. Bausewein 2022 names Lely's SCC system as MQC-C. Licence CC BY. Published online on 19 December 2025 in the 2026 volume; the year of the journal issue is used.</t>
+          <t>COI: 'Fernando Masia and Elisa Vrieze are employed by the company Lely International N.V.' Text says AMS 'could also be equipped with sensors performing somatic cell count' and that external calibration data were not entered on these farms. Bausewein 2022 names Lely's SCC system as MQC-C. Licence CC BY. Published online on 19 December 2025 in the 2026 volume; the year of the journal issue is used. For milk yield (I075) the product is not shown to be on sale by a source since 2021, so the test is recorded but no grade rests on it.</t>
         </is>
       </c>
     </row>
@@ -35028,7 +35025,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>I039;I062;I066;I071;I072;I073</t>
+          <t>I039;I062;I066;I071;I072;I073;I068</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -35114,7 +35111,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>I022;I069;I078</t>
+          <t>I022;I069;I078;I068</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -35716,7 +35713,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>I039;I071;I073</t>
+          <t>I039;I071;I073;I068</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -35888,7 +35885,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>I013</t>
+          <t>I013;I068</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -35974,7 +35971,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>I027;I063;I064;I070;I071;I081</t>
+          <t>I027;I063;I064;I070;I071;I081;I068</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -36558,12 +36555,12 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>research_farm</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>36 (dataset row 36)</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -36571,11 +36568,7 @@
           <t>not_stated</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>funding (Europe PMC grant list names Nedap Livestock Management, as recorded in step 3; the funding wording was not read)</t>
-        </is>
-      </c>
+      <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr">
         <is>
           <t>eating, ruminating and inactive time</t>
@@ -36588,12 +36581,12 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>Lee Table 4: CCC = 0.93 to 0.98, Pearson correlation, Bland-Altman plots; validity Yes. Abstract (as recorded in step 3): CCC at least 0.88, no bias in Bland-Altman plots</t>
+          <t>Lee Table 4: CCC = 0.93 to 0.98, Pearson correlation, Bland-Altman plots; validity Yes</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>dataset row; review table; abstract as recorded in step 3 (scratchpad step3/out_lee_records.csv), not re-read</t>
+          <t>dataset row 36; review table (Lee Table 4)</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -36608,7 +36601,7 @@
       </c>
       <c r="T54" s="2" t="inlineStr">
         <is>
-          <t>Step 3 recorded this study under the same key for I012 and did not use it there. on_sale rests on Lee Table 3 and its discussion naming Nedap Smart Tag among commercial wearables. University of Kentucky research herd per step 3.</t>
+          <t>on_sale rests on Lee Table 3 and its discussion naming Nedap Smart Tag among commercial wearables. Only the dataset row and Lee's tables are on disk; the paper itself was not read.</t>
         </is>
       </c>
     </row>
@@ -36660,12 +36653,12 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>research_farm</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12 (dataset row 37)</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -36673,11 +36666,7 @@
           <t>not_stated</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr">
-        <is>
-          <t>not_stated (abstract silent, full text not on disk)</t>
-        </is>
-      </c>
+      <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr">
         <is>
           <t>rumination, grazing, standing and lying time of grazing cows</t>
@@ -36690,12 +36679,12 @@
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Abstract (as recorded in step 3): Pearson r 0.84 rumination, 0.76 grazing, 0.83 standing, 0.91 lying. Lee Table 4: precision 0.90 to 1.00; validity 'Yes, but grazing and standing only'</t>
+          <t>Lee Table 4: precision 0.90 to 1.00; validity 'Yes, but grazing and standing only'</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>dataset row; review table; abstract as recorded in step 3 (scratchpad step3/out_lee_records.csv), not re-read</t>
+          <t>dataset row 37; review table (Lee Table 4)</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -36710,7 +36699,7 @@
       </c>
       <c r="T55" s="2" t="inlineStr">
         <is>
-          <t>Step 3 used this key for I012 but it was not carried into evidence_since_2021.csv. on_sale rests on Lee, which counts RumiWatch among its commercial wearables (Table 3, discussion); Pichlbauer 2024 calls it a widely used research tool.</t>
+          <t>on_sale rests on Lee, which counts RumiWatch among its commercial wearables (Table 3, discussion). Only the dataset row and Lee's tables are on disk; the paper itself was not read.</t>
         </is>
       </c>
     </row>
@@ -36921,7 +36910,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Pfeiffer2021tail</t>
+          <t>Saar2022intake</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -36931,47 +36920,43 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Pfeiffer J, Spykman O, Gandorfer M. 2021. Sensor and Video: Two Complementary Approaches for Evaluation of Dairy Cow Behavior after Calving Sensor Attachment. Animals 11(7): 1917</t>
+          <t>Saar M, Edan Y, Godo A, Lepar J, Parmet Y, Halachmi I. 2022. A machine vision system to predict individual cow feed intake of different feeds in a cowshed. Animal 16: 100432</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>10.3390/ani11071917</t>
+          <t>10.1016/j.animal.2021.100432</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>I070</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>Moocall (Moocall Ltd.) and CalveSense (Allflex) tail calving sensors; smaXtec rumen bolus</t>
-        </is>
-      </c>
+          <t>I062;I080</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>tail mounted calving sensors; rumen bolus activity; video</t>
+          <t>camera images of feed piles before and after meals, CNN with transfer learning</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>research_farm</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>18 cows (video subgroup of 9)</t>
+          <t>60 (Islam Table 5)</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -36981,49 +36966,49 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>not_stated (not checked)</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>cow activity and behaviour after attaching a calving sensor; not calving detection</t>
+          <t>individual cow feed intake from feed pile images</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>not applicable for calving detection (video was used for behaviour)</t>
+          <t>not stated in the review</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>not used</t>
+          <t>Islam Table 5: MAE = 0.12 to 0.23 kg</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>dataset row; full text (abstract, introduction, methods, institutional review statement)</t>
+          <t>review table; review text</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>lee_2025_dataset.xlsx sheet Sifted articles row 32; full text read from scratchpad step3/primary/pfeiffer_2021_PMC8300263.xml</t>
+          <t>islam_2026_computer_vision.xml Table 5 ref [119]; section 3.5.2</t>
         </is>
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t>lee_2025_dataset.xlsx</t>
+          <t>islam_2026_computer_vision.xml</t>
         </is>
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>Used only for the facts that the tail sensors are sold for early calving detection: the abstract says the sensors are attached to the tail for early detection of calving, and the review statement calls them commercially available technologies also used on commercial dairy farms. The full text is not in 1_sources. Dairy research and demonstration farm in Bavaria, 2018.</t>
+          <t>Abstract and full text not on disk. Dairy cows per the review table.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Saar2022intake</t>
+          <t>Lassen2023camera</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -37033,22 +37018,22 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Saar M, Edan Y, Godo A, Lepar J, Parmet Y, Halachmi I. 2022. A machine vision system to predict individual cow feed intake of different feeds in a cowshed. Animal 16: 100432</t>
+          <t>Lassen J, Thomasen JR, Borchersen S. 2023. Repeatabilities of individual measures of feed intake and body weight on in-house commercial dairy cattle using a 3-dimensional camera system. Journal of Dairy Science 106: 9105 to 9114</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>10.1016/j.animal.2021.100432</t>
+          <t>10.3168/jds.2022-23177</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>I062;I080</t>
+          <t>I062;I079</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
@@ -37059,24 +37044,24 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>camera images of feed piles before and after meals, CNN with transfer learning</t>
+          <t>3D camera system, image processing</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
+          <t>commercial_farm</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>9142 (Islam Table 3)</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
           <t>not_stated</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>60 (Islam Table 5)</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>not_stated</t>
-        </is>
-      </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
           <t>not stated</t>
@@ -37084,7 +37069,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>individual cow feed intake from feed pile images</t>
+          <t>individual feed intake and body weight (Islam Table 3: Body Weight, Feed Intake)</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr">
@@ -37094,7 +37079,7 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Islam Table 5: MAE = 0.12 to 0.23 kg</t>
+          <t>Islam Table 3: Accuracy = 88%</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr">
@@ -37104,7 +37089,7 @@
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>islam_2026_computer_vision.xml Table 5 ref [119]; section 3.5.2</t>
+          <t>islam_2026_computer_vision.xml Table 3 ref [85]; section 3.3.1</t>
         </is>
       </c>
       <c r="S59" s="2" t="inlineStr">
@@ -37114,14 +37099,14 @@
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>Abstract and full text not on disk. Dairy cows per the review table.</t>
+          <t>Setting from the title (in house commercial dairy cattle). The title reports repeatabilities, so the 88% may not be agreement with a scale or a feed weighing reference; the abstract is not on disk. The review does not say whether the camera system is a product on sale.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Lassen2023camera</t>
+          <t>Bi2023bw</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -37131,12 +37116,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Lassen J, Thomasen JR, Borchersen S. 2023. Repeatabilities of individual measures of feed intake and body weight on in-house commercial dairy cattle using a 3-dimensional camera system. Journal of Dairy Science 106: 9105 to 9114</t>
+          <t>Bi Y, Campos LM, Wang J, Yu H, Hanigan MD, Morota G. 2023. Depth video data-enabled predictions of longitudinal dairy cow body weight using thresholding and Mask R-CNN algorithms. Smart Agricultural Technology 6: 100352</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>10.3168/jds.2022-23177</t>
+          <t>10.1016/j.atech.2023.100352</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -37146,7 +37131,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>I062;I079</t>
+          <t>I079</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
@@ -37157,17 +37142,17 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>3D camera system, image processing</t>
+          <t>depth camera video, Mask R-CNN</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>commercial_farm</t>
+          <t>not_stated</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>9142 (Islam Table 3)</t>
+          <t>12 (Islam Table 3)</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -37182,7 +37167,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>individual feed intake and body weight (Islam Table 3: Body Weight, Feed Intake)</t>
+          <t>dairy cow body weight</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr">
@@ -37192,7 +37177,7 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Islam Table 3: Accuracy = 88%</t>
+          <t>Islam Table 3: Accuracy = 98%</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr">
@@ -37202,7 +37187,7 @@
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>islam_2026_computer_vision.xml Table 3 ref [85]; section 3.3.1</t>
+          <t>islam_2026_computer_vision.xml Table 3 ref [86]; section 3.3.1</t>
         </is>
       </c>
       <c r="S60" s="2" t="inlineStr">
@@ -37211,104 +37196,6 @@
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr">
-        <is>
-          <t>Setting from the title (in house commercial dairy cattle). The title reports repeatabilities, so the 88% may not be agreement with a scale or a feed weighing reference; the abstract is not on disk. The review does not say whether the camera system is a product on sale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Bi2023bw</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>study</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>Bi Y, Campos LM, Wang J, Yu H, Hanigan MD, Morota G. 2023. Depth video data-enabled predictions of longitudinal dairy cow body weight using thresholding and Mask R-CNN algorithms. Smart Agricultural Technology 6: 100352</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>10.1016/j.atech.2023.100352</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>I079</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>not_stated</t>
-        </is>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>depth camera video, Mask R-CNN</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>not_stated</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>12 (Islam Table 3)</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>not_stated</t>
-        </is>
-      </c>
-      <c r="M61" s="2" t="inlineStr">
-        <is>
-          <t>not stated</t>
-        </is>
-      </c>
-      <c r="N61" s="2" t="inlineStr">
-        <is>
-          <t>dairy cow body weight</t>
-        </is>
-      </c>
-      <c r="O61" s="2" t="inlineStr">
-        <is>
-          <t>not stated in the review</t>
-        </is>
-      </c>
-      <c r="P61" s="2" t="inlineStr">
-        <is>
-          <t>Islam Table 3: Accuracy = 98%</t>
-        </is>
-      </c>
-      <c r="Q61" s="2" t="inlineStr">
-        <is>
-          <t>review table; review text</t>
-        </is>
-      </c>
-      <c r="R61" s="2" t="inlineStr">
-        <is>
-          <t>islam_2026_computer_vision.xml Table 3 ref [86]; section 3.3.1</t>
-        </is>
-      </c>
-      <c r="S61" s="2" t="inlineStr">
-        <is>
-          <t>islam_2026_computer_vision.xml</t>
-        </is>
-      </c>
-      <c r="T61" s="2" t="inlineStr">
         <is>
           <t>Abstract and full text not on disk.</t>
         </is>

</xml_diff>

<commit_message>
Second round of audit corrections to step 4: I075 unsure since 2021, Certified Humane I080 back to FW 9 c, I082 readings completed, records and wording fixed; rules 0.8.2.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Studies and maker pages since 2021, read in October 2026: 12 tested; 17 claimed; 5 shown in research; 8 proposed only; 28 nothing found; 11 unclear. The stronger of the two grades, used for the score and Kevin's lists: 16 tested; 19 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 7 unclear.</t>
+          <t>Studies and maker pages since 2021, read in October 2026: 12 tested; 16 claimed; 5 shown in research; 8 proposed only; 28 nothing found; 12 unclear. The stronger of the two grades, used for the score and Kevin's lists: 16 tested; 19 claimed; 3 shown in research; 27 proposed only; 9 nothing found; 7 unclear.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>No welfare validation: none of the three sources links it to welfare, but a product's description says it is for health, welfare or a named condition, or it is itself a health or condition status, or a scheme requires it</t>
+          <t>No welfare validation: none of the three sources links it to welfare, but a product's description says it is for health, welfare or a named condition, or it is itself a health, welfare or condition status, or a scheme requires it</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>The sensor evidence is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products and studies are as those papers found them, and so are the links in the column Link (2021); what those links open today is in the Product list sheet; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
+          <t>The 2021 sensor grade is a baseline from two papers, Stygar et al. 2021 and Maroto Molina et al. 2020. Products and studies are as those papers found them, and so are the links in the column Link (2021); what those links open today is in the Product list sheet; 'Nothing found' means nothing in those two papers, not nothing anywhere.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       <c r="A50" s="3" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>A sensor side row is on list 1 when a product measures it and no scheme requires it, whatever its welfare relevance. Read column (1) beside it: a row with no welfare validation is a finding about what the market measures, not a welfare indicator that schemes have missed.</t>
+          <t>A sensor side row is on list 1 when a product is tested for it or claims it and no scheme requires it, whatever its welfare relevance. Read column (1) beside it: a row with no welfare validation is a finding about what the market measures, not a welfare indicator that schemes have missed.</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Link: EFSA 2023, Table 26 (PDF 42), measures used for assessment of mastitis: severe clinical mastitis includes "systemic signs of illness such as apathy, anorexia, dehydration, or fever". No passage questions the link. Linstädt et al. 2024 (PDF 15) discusses nasal surface temperature and emotional state, a different parameter, not counted. Nasal temperature is excluded as a different parameter: Linstädt et al. 2024 (PDF 15) treat the temperature of the nose, a local skin temperature, as a sign of emotional state; the class counts the thermal cameras only for their claim to detect fever, a raised body temperature, not for local skin temperature.</t>
+          <t>Link: EFSA 2023, Table 26 (PDF 42), measures used for assessment of mastitis: severe clinical mastitis includes "systemic signs of illness such as apathy, anorexia, dehydration, or fever". No passage questions the link. Nasal temperature is excluded as a different parameter: Linstädt et al. 2024 (PDF 15) treat the temperature of the nose, a local skin temperature, as a sign of emotional state; the class counts the thermal cameras only for their claim to detect fever, a raised body temperature, not for local skin temperature.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -3593,7 +3593,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, titled an evaluation of the estrus alerts of the SmartBow ear tag in 216 cows, compared with the HeatWatch System, another electronic system; the row codes the behaviours detected as physical activity and rumination time, and no result values are on disk. Rule 4.11 does not say whether another system is a reference method, and Lee (PDF page 2) gives a laboratory assay as the gold standard for oestrus. The maker pages of Herd Navigator, smaXtec, SenseHub, Cowmed and IDS i-QUBE claim heat or oestrus detection. Candidate readings: validated_commercial if the oestrus alerts and the HeatWatch comparison count, or commercial_unvalidated on the maker pages. The 2021 grade, commercial_unvalidated, stands either way.</t>
+          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, titled an evaluation of the estrus alerts of the SmartBow ear tag in 216 cows, compared with the HeatWatch System, another electronic system; the row codes the behaviours detected as physical activity and rumination time, and no result values are on disk. Rule 4.11 does not say whether another system is a reference method, Lee (PDF page 2) says some common comparison standards have poor sensitivity "compared to a gold standard such as a laboratory assay; this is especially true for estrus detection", while it counts "cross-validation against another sensor" (25 of 101 studies) among the comparison methods of the studies it reviews (PDF page 6). The maker pages of Herd Navigator, smaXtec, SenseHub, Cowmed and IDS i-QUBE claim heat or oestrus detection. Candidate readings: validated_commercial if the oestrus alerts and the HeatWatch comparison count, or commercial_unvalidated on the maker pages. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -3708,7 +3708,7 @@
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Claimed: the maker's current page, or a source since 2021, says a product on sale measures it; no test against a reference was found</t>
+          <t>Unclear: the written rules do not settle it (see open questions)</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Bausewein 2022 (ev_bausewein2022ams.xml) says the commercially available sensor systems in automatic milking systems provide milk yield. Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records, with two Lely employees among the authors; but no source since 2021 says the Astronaut A5 is on sale (Lely's page sells the Astronaut A5 Next), so, as for fat and protein on I021 and I025, the test is recorded and the grade is commercial_unvalidated.</t>
+          <t>Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records, with two Lely employees among the authors. No source since 2021 on disk says the Astronaut A5 is on sale. Bausewein 2022 (ev_bausewein2022ams.xml) says only that the commercially available sensor systems in automatic milking systems provide milk yield, naming no product for it. Rule 4.11 gives validated_commercial only to a product a source shows on sale, and commercial_unvalidated only where no test against a reference was found, so neither fits. Candidate readings: validated_commercial, if Bausewein's statement shows the tested robots on sale, or commercial_unvalidated, if a test of a product not shown on sale leaves the claim untested. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Unsure under rule 4.14. Link: Linstädt et al. 2024 (PDF 8): combining automatic indicators "offers the potential for an early warning system in addressing welfare problems". Possible questions: Linstädt et al. 2024 (PDF 16): "Precision Livestock Farming offers real-time welfare assessment, but validation is important."; (PDF 12): PLF technologies "currently have limited potential for assessing appropriate behavior in dairy cows, necessitating further validation studies". These two say that sensor based welfare assessment still needs validation; they do not use rule 4.14's words for a question (indirect, insufficient on its own, weak, inconsistent, unclear or not fully understood), and validation of a technology belongs to column (a), but the parameter is itself a sensor based welfare assessment. Candidate readings: supported (the PDF 8 link, with no question) or indirect_or_contested (the validation passages as questions). See open_questions.md.</t>
+          <t>Unsure under rule 4.14. Link: Linstädt et al. 2024 (PDF 8): combining automatic indicators "offers the potential for an early warning system in addressing welfare problems". Possible questions: Linstädt et al. 2024 (PDF 16): "Precision Livestock Farming offers real-time welfare assessment, but validation is important."; (PDF 12): PLF technologies "currently have limited potential for assessing appropriate behavior in dairy cows, necessitating further validation studies". PDF 16 says PLF welfare assessment needs validation, and PDF 12 says PLF tools for assessing behaviour need further validation studies; they do not use rule 4.14's words for a question (indirect, insufficient on its own, weak, inconsistent, unclear or not fully understood), and validation of a technology belongs to column (a), but the parameter is itself a sensor based welfare assessment. Candidate readings: supported (the PDF 8 link, with no question) or indirect_or_contested (the validation passages as questions). See open_questions.md.</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -22488,7 +22488,7 @@
       <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Searched for blood, bloody, abnormal milk, clots and forestrip. No standard names blood in milk. Blood appears only as a calf blood sample for testing passive immunity (Chapter 5, PDF 88) in euthanasia text (Chapter 7, PDF 127), and as blood flow in science and guidance text (Chapter 3, PDF 36; Chapter 6, PDF 112). The nearest standards are the milking procedures protocol (Chapter 4, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56); FARM's text does not tie either to blood in milk.</t>
+          <t>Searched for blood, bloody, abnormal milk, clots and forestrip. No standard names blood in milk. Blood appears only as a calf blood sample for testing passive immunity (Chapter 5, PDF 88), in euthanasia text (Chapter 7, PDF 127), and as blood flow in science and guidance text (Chapter 3, PDF 36; Chapter 6, PDF 112). The nearest standards are the milking procedures protocol (Chapter 4, PDF 70) and the mastitis treatment protocol (Chapter 4, PDF 56); FARM's text does not tie either to blood in milk.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -22694,7 +22694,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>"Cattle must have free access to nutritious food each day, except when directed otherwise by an attending veterinarian." (FW 2, PDF 11 (printed 2))</t>
+          <t>"The feed itself must be pushed up regularly to ensure additional ease of access to feed." (FW 9 c, PDF 13 (printed 4))</t>
         </is>
       </c>
     </row>
@@ -22777,7 +22777,7 @@
       <c r="D82" s="2" t="inlineStr"/>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73)). Unsure. The row's animals are unweaned calves, so a calf milk standard is in the row's own animals (rule 6). FW(C) 1.3.1 a) sets the amount of milk or milk replacer each calf must be offered per day, which is the milk given to each calf that the row records, a management measure, and rule 7 counts a requirement that names a management measure. The box below it says there is no requirement for calves to consume the full quantities; it is guidance (rule 2), and it confirms the standard is about the milk given, not the milk drunk. FW(C) 1.3.1 b) adds "across at least two feeds per day for the first 42 days of life". On rule 4: the calf standards are to be used by anyone rearing calves on an assured unit (PDF 74, printed 72), but FW(C) 1.3.1 is limited to calves no longer with their dam after 24 hours, and the standards also provide for calves that stay with the dam (FW(C) 1.3 b) i., PDF 74, printed 72; FW(C) 1.6, all non-suckled calves, PDF 76, printed 74; FW(C) 1.18, artificially reared calves, PDF 77, printed 75). Reading one: it applies to every certified farm that rears calves apart from the dam, and that condition is the practice the row itself measures, so the row is required. Reading two: it is limited to one rearing system, which rule 4 does not count, so not_required. Rule 4 does not say whether a condition that is the row's own practice limits a requirement, so the row is unsure. how_checked is left empty: no RSPCA text says how the milk offered is checked. Related: FW(C) 1.6, all non-suckled calves must receive liquid food daily for at least the first eight weeks and until eating at least 1.5kg dry matter per day of a calf starter ration, and FW(C) 1.6.1, abrupt weaning not permitted (PDF 76, printed 74); FW(C) 1.3 a), at least 3 litres of colostrum within the first 6 hours (PDF 74, printed 72), colostrum rather than milk or milk replacer; FW(C) 1.1 b), a diet fed in sufficient quantity (PDF 74, printed 72), broader wording (rule 6); FW(C) 1.17.1, where calves are fed by an ad-lib automated system the producer must show there is no competition that may limit intake, and FW(C) 1.20, where calves are rationed by transponder the feed station must let all calves drink without hindrance (PDF 77, printed 75), provisions limited to farms with those systems (rules 10 and 4); FW(C) 1.18, milk feeds through teat feeders for artificially reared calves (PDF 77, printed 75), an equipment provision (rule 10).</t>
+          <t>Candidate: "In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73)). Unsure. The row's animals are unweaned calves, so a calf milk standard is in the row's own animals (rule 6). FW(C) 1.3.1 a) sets the amount of milk or milk replacer each calf must be offered per day, which is the milk given to each calf that the row records, a management measure, and rule 7 counts a requirement that names a management measure. The box below it says there is no requirement for calves to consume the full quantities; it is guidance (rule 2), and it confirms the standard is about the milk given, not the milk drunk. FW(C) 1.3.1 b) adds "across at least two feeds per day for the first 42 days of life". On rule 4: the calf standards are to be used by anyone rearing calves on an assured unit (PDF 74, printed 72), but FW(C) 1.3.1 is limited to calves no longer with their dam after 24 hours, and the standards also provide for calves that are not artificially reared (FW(C) 1.6, all non-suckled calves, PDF 76, printed 74; FW(C) 1.18, artificially reared calves, PDF 77, printed 75). Reading one: it applies to every certified farm that rears calves apart from the dam, and that condition is the practice the row itself measures, so the row is required. Reading two: it is limited to one rearing system, which rule 4 does not count, so not_required. Rule 4 does not say whether a condition that is the row's own practice limits a requirement, so the row is unsure. The FARM_v5 row of I051 reads such a condition as applying to every farm; it rests on the same question, which rule 4 itself does not settle. how_checked is left empty: no RSPCA text says how the milk offered is checked. Related: FW(C) 1.6, all non-suckled calves must receive liquid food daily for at least the first eight weeks and until eating at least 1.5kg dry matter per day of a calf starter ration, and FW(C) 1.6.1, abrupt weaning not permitted (PDF 76, printed 74); FW(C) 1.3 a), at least 3 litres of colostrum within the first 6 hours (PDF 74, printed 72), colostrum rather than milk or milk replacer; FW(C) 1.1 b), a diet fed in sufficient quantity (PDF 74, printed 72), broader wording (rule 6); FW(C) 1.17.1, where calves are fed by an ad-lib automated system the producer must show there is no competition that may limit intake, and FW(C) 1.20, where calves are rationed by transponder the feed station must let all calves drink without hindrance (PDF 77, printed 75), provisions limited to farms with those systems (rules 10 and 4); FW(C) 1.18, milk feeds through teat feeders for artificially reared calves (PDF 77, printed 75), an equipment provision (rule 10).</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -22818,7 +22818,7 @@
       <c r="M82" s="2" t="inlineStr"/>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "All calves must receive milk or milk replacer at least twice daily through the first five weeks of life." (FW 14 a, PDF 14 (printed 5)). Unsure. The row's animals are unweaned calves, so the calf standards in Part 2 B, Food, Specific Provisions for Calves, are in the row's own animals (rule 6). FW 14 a requires that every calf receive milk or milk replacer, with a frequency and a period, and it applies to all calves on every farm (rule 4). Reading one: it names the milk given to each calf, a management measure that rule 7 counts, so the row is required. Reading two: it sets only how often milk is fed, with no amount, while the row is the amount each calf is given and the feeder records; as on the I062 rows, a feeding requirement with no amount for each animal does not name the amount, so not_required. Rules 6, 7 and 13 do not settle whether a frequency without an amount names the measure, so the row is unsure. It sets no volume; the only volume, a daily ration of at least 20% of body weight (approximately 8 liters for larger breeds like Holstein calves) for calves aged 3 to 28 days, is in the recommendation below FW 12 (PDF 13 and 14, printed 4 and 5), which does not count (rule 2). FW 13 c (PDF 14, printed 5) also names it: "Twice per day over the subsequent 48 hours, calves must receive additional colostrum or whole milk in an amount that is breed and size appropriate." how_checked is left empty: no numbered requirement says how milk feeding is checked. Related (all PDF 14, printed 5): FW 14 e, milk replacer mixed according to the manufacturer's instructions; FW 14 b, an individual bucket for each calf where calves are bucket fed, limited to bucket feeding (rules 10 and 4); FW 14 f, calves not weaned until eating at least 1.5 lbs. (680 g) per calf per day of calf starter, which is feed, not milk; FW 15 a, weaning by diluting the milk or reducing the milk volume over at least 5 days; FW 13 a and b, colostrum within the first 6 hours and at least 2 quarts in two feedings within 12 h when the calf has not nursed, colostrum rather than milk, and b only when the calf has not nursed (rule 4).</t>
+          <t>Candidate: "All calves must receive milk or milk replacer at least twice daily through the first five weeks of life." (FW 14 a, PDF 14 (printed 5)). Unsure. The row's animals are unweaned calves, so the calf standards in Part 2 B, Food, Specific Provisions for Calves, are in the row's own animals (rule 6). FW 14 a requires that every calf receive milk or milk replacer, with a frequency and a period, and it applies to all calves on every farm (rule 4). Reading one: it names the milk given to each calf, a management measure that rule 7 counts, so the row is required. Reading two: it sets only how often milk is fed, with no amount, while the row is the amount each calf is given and the feeder records; as on the I062 rows, a feeding requirement with no amount for each animal does not name the amount, so not_required. Rules 6, 7 and 13 do not settle whether a frequency without an amount names the measure, so the row is unsure. It sets no volume; the only volume, a daily ration of at least 20% of body weight (approximately 8 liters for larger breeds like Holstein calves) for calves aged 3 to 28 days, is in the recommendation below FW 12 (PDF 13 and 14, printed 4 and 5), which does not count (rule 2). FW 13 c (PDF 14, printed 5) is a further candidate under both readings, since it sets an amount, but only as breed and size appropriate and only for colostrum or whole milk in the 48 hours after birth: "Twice per day over the subsequent 48 hours, calves must receive additional colostrum or whole milk in an amount that is breed and size appropriate." how_checked is left empty: no numbered requirement says how milk feeding is checked. Related (all PDF 14, printed 5): FW 14 e, milk replacer mixed according to the manufacturer's instructions; FW 14 b, an individual bucket for each calf where calves are bucket fed, limited to bucket feeding (rules 10 and 4); FW 14 f, calves not weaned until eating at least 1.5 lbs. (680 g) per calf per day of calf starter, which is feed, not milk; FW 15 a, weaning by diluting the milk or reducing the milk volume over at least 5 days; FW 13 a and b, colostrum within the first 6 hours and at least 2 quarts in two feedings within 12 h when the calf has not nursed, colostrum rather than milk, and b only when the calf has not nursed (rule 4).</t>
         </is>
       </c>
     </row>
@@ -32229,7 +32229,7 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019. Used for I082 only for section 2.1's statement that an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan; it gives no amount and no sale status for the feeder.</t>
+          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019. Used for I082 only for section 2.1's statement that an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan; it gives no amount and no sale status for the feeder. For I082 the feeder's sale status is not stated; on_sale no refers to the SparkFun IMU.</t>
         </is>
       </c>
     </row>
@@ -36576,7 +36576,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>video (dataset Comparison); visual observation, 4 h per cow, per the abstract as recorded in step 3</t>
+          <t>video (Lee dataset, column Comparison)</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -36674,7 +36674,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>video (dataset Comparison); visual observation by 3 observers per the abstract as recorded in step 3</t>
+          <t>video (Lee dataset, column Comparison)</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rule 4: a condition that is only the row's own practice does not limit a requirement (Manisha, 17 October 2026); RSPCA I082 required; final audit wording fixes; rules 0.8.3.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_output/welfare_crosswalk_dairy.xlsx
+++ b/4_output/welfare_crosswalk_dairy.xlsx
@@ -1010,7 +1010,7 @@
       <c r="A50" s="3" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>A sensor side row is on list 1 when a product is tested for it or claims it and no scheme requires it, whatever its welfare relevance. Read column (1) beside it: a row with no welfare validation is a finding about what the market measures, not a welfare indicator that schemes have missed.</t>
+          <t>A sensor side row is on list 1 when a product is tested for it or claims it, no scheme requires it and no scheme row is unclear (otherwise it shows Unclear), whatever its welfare relevance. Read column (1) beside it: a row with no welfare validation is a finding about what the market measures, not a welfare indicator that schemes have missed.</t>
         </is>
       </c>
     </row>
@@ -1640,11 +1640,11 @@
         </is>
       </c>
       <c r="W4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>FARM v5 (US industry): inspector checks farm records; Global Animal Partnership (US): required, but the scheme does not say how it is checked; unclear whether RSPCA Assured (UK), Certified Humane (US) requires it</t>
+          <t>RSPCA Assured (UK): required, but the scheme does not say how it is checked; FARM v5 (US industry): inspector checks farm records; Global Animal Partnership (US): required, but the scheme does not say how it is checked; unclear whether Certified Humane (US) requires it</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, titled an evaluation of the estrus alerts of the SmartBow ear tag in 216 cows, compared with the HeatWatch System, another electronic system; the row codes the behaviours detected as physical activity and rumination time, and no result values are on disk. Rule 4.11 does not say whether another system is a reference method, Lee (PDF page 2) says some common comparison standards have poor sensitivity "compared to a gold standard such as a laboratory assay; this is especially true for estrus detection", while it counts "cross-validation against another sensor" (25 of 101 studies) among the comparison methods of the studies it reviews (PDF page 6). The maker pages of Herd Navigator, smaXtec, SenseHub, Cowmed and IDS i-QUBE claim heat or oestrus detection. Candidate readings: validated_commercial if the oestrus alerts and the HeatWatch comparison count, or commercial_unvalidated on the maker pages. The 2021 grade, commercial_unvalidated, stands either way.</t>
+          <t>Lee's dataset row 35 (lee_2025_dataset.xlsx) records Schilkowsky 2021, titled an evaluation of the estrus alerts of the SmartBow ear tag in 216 cows, compared with the HeatWatch System, another electronic system; the row codes the behaviours detected as physical activity and rumination time, and no result values are on disk. Rule 4.11 does not say whether another system is a reference method, Lee (PDF page 2) says that some common comparison standards "(i.e., human observation) have poor sensitivity compared to a gold standard such as a laboratory assay; this is especially true for estrus detection", while under its heading on gold standard comparison it counts "cross-validation against another sensor" in 25 of 101 studies (PDF page 6). The maker pages of Herd Navigator, smaXtec, SenseHub, Cowmed and IDS i-QUBE claim heat or oestrus detection. Candidate readings: validated_commercial if the oestrus alerts and the HeatWatch comparison count, or commercial_unvalidated on the maker pages. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -3713,12 +3713,12 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Ponzo2026AMS;Bausewein2022AMS</t>
+          <t>Ponzo2026AMS;Bausewein2022AMS;Maker:lely_astronaut_a5_next</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records, with two Lely employees among the authors. No source since 2021 on disk says the Astronaut A5 is on sale. Bausewein 2022 (ev_bausewein2022ams.xml) says only that the commercially available sensor systems in automatic milking systems provide milk yield, naming no product for it. Rule 4.11 gives validated_commercial only to a product a source shows on sale, and commercial_unvalidated only where no test against a reference was found, so neither fits. Candidate readings: validated_commercial, if Bausewein's statement shows the tested robots on sale, or commercial_unvalidated, if a test of a product not shown on sale leaves the claim untested. The 2021 grade, commercial_unvalidated, stands either way.</t>
+          <t>Ponzo 2026 (ev_ponzo2026ams.xml, Table 2) compared daily milk yield from Lely Astronaut A5 robots on five commercial farms with same day official milk recording, which it calls the gold standard: r 0.931 on 19,488 records, with two Lely employees among the authors. No source since 2021 on disk says the Astronaut A5 is on sale: Lely's page (maker_lely_astronaut_a5_next.txt, saved 16 October 2026) sells the Astronaut A5 Next, which it says builds on the A5, and claims no milk yield, as on I021 and I025. Bausewein 2022 (ev_bausewein2022ams.xml) says only that the commercially available sensor systems in automatic milking systems provide milk yield, naming no product for it. Rule 4.11 gives validated_commercial only to a product a source shows on sale, and commercial_unvalidated only where no test against a reference was found, so neither fits. Candidate readings: validated_commercial, if Bausewein's statement shows the tested robots on sale, or commercial_unvalidated, if a test of a product not shown on sale leaves the claim untested. The 2021 grade, commercial_unvalidated, stands either way.</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
@@ -22771,13 +22771,17 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr"/>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>required, but the scheme does not say how it is checked</t>
+        </is>
+      </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Candidate: "In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73)). Unsure. The row's animals are unweaned calves, so a calf milk standard is in the row's own animals (rule 6). FW(C) 1.3.1 a) sets the amount of milk or milk replacer each calf must be offered per day, which is the milk given to each calf that the row records, a management measure, and rule 7 counts a requirement that names a management measure. The box below it says there is no requirement for calves to consume the full quantities; it is guidance (rule 2), and it confirms the standard is about the milk given, not the milk drunk. FW(C) 1.3.1 b) adds "across at least two feeds per day for the first 42 days of life". On rule 4: the calf standards are to be used by anyone rearing calves on an assured unit (PDF 74, printed 72), but FW(C) 1.3.1 is limited to calves no longer with their dam after 24 hours, and the standards also provide for calves that are not artificially reared (FW(C) 1.6, all non-suckled calves, PDF 76, printed 74; FW(C) 1.18, artificially reared calves, PDF 77, printed 75). Reading one: it applies to every certified farm that rears calves apart from the dam, and that condition is the practice the row itself measures, so the row is required. Reading two: it is limited to one rearing system, which rule 4 does not count, so not_required. Rule 4 does not say whether a condition that is the row's own practice limits a requirement, so the row is unsure. The FARM_v5 row of I051 reads such a condition as applying to every farm; it rests on the same question, which rule 4 itself does not settle. how_checked is left empty: no RSPCA text says how the milk offered is checked. Related: FW(C) 1.6, all non-suckled calves must receive liquid food daily for at least the first eight weeks and until eating at least 1.5kg dry matter per day of a calf starter ration, and FW(C) 1.6.1, abrupt weaning not permitted (PDF 76, printed 74); FW(C) 1.3 a), at least 3 litres of colostrum within the first 6 hours (PDF 74, printed 72), colostrum rather than milk or milk replacer; FW(C) 1.1 b), a diet fed in sufficient quantity (PDF 74, printed 72), broader wording (rule 6); FW(C) 1.17.1, where calves are fed by an ad-lib automated system the producer must show there is no competition that may limit intake, and FW(C) 1.20, where calves are rationed by transponder the feed station must let all calves drink without hindrance (PDF 77, printed 75), provisions limited to farms with those systems (rules 10 and 4); FW(C) 1.18, milk feeds through teat feeders for artificially reared calves (PDF 77, printed 75), an equipment provision (rule 10).</t>
+          <t>"In relation to standard FW(C) 1.3, after the first 24 hours of being born, calves no longer with their dam must be maintained at a healthy body weight and offered: a) either access to at least eight litres of pasteurised whole milk or transition milk per day (or 15% of their bodyweight, whichever is the most), OR at least 900g of good quality artificial calf milk replacer powder per day, mixed according to manufacturer’s instructions" (FW(C) 1.3.1 a), PDF 75 (printed 73))</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -32229,7 +32233,7 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019. Used for I082 only for section 2.1's statement that an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan; it gives no amount and no sale status for the feeder. For I082 the feeder's sale status is not stated; on_sale no refers to the SparkFun IMU.</t>
+          <t>Lee's dataset names the sensor as 'Forster Technik COMPACT smart', but in the paper that is the calves' automatic milk feeder; the sensor is a SparkFun research IMU, so not a product sold for this measure. Year: Europe PMC gives epub 25 December 2020 and the issue as January 2021 (volume 21, issue 1); Lee cites 2021. Conflicts: none declared; funded by the BBSRC (BB/M008770/1). Centre for Dairy Science Innovation, University of Nottingham, January and February 2019. Used for I082 only for section 2.1's statement that an automatic feeder, the Forster Technik COMPACT smart, fed the calves milk replacer on an individualised feeding plan; it gives no amount and no sale status for the feeder. on_sale no refers to the SparkFun IMU, not the feeder.</t>
         </is>
       </c>
     </row>
@@ -36245,7 +36249,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>I021;I025;I076</t>
+          <t>I021;I025;I076;I075</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">

</xml_diff>